<commit_message>
Add year switcher dropdown to Бюджет
Год was a free-typed number; now it's a dropdown (2023-2032) sourced
from Справочник, matching the Месяц switcher.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6CkgouQ8AhQXxstTSck9L
</commit_message>
<xml_diff>
--- a/Планировщик_Бюджет_Привычки.xlsx
+++ b/Планировщик_Бюджет_Привычки.xlsx
@@ -4619,9 +4619,12 @@
       <formula>D27="Расход"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочник!$L$3:$L$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Справочник!$M$3:$M$12</formula1>
     </dataValidation>
     <dataValidation sqref="C27:C226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочник!$K$3:$K$9</formula1>
@@ -8351,7 +8354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8365,6 +8368,7 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -8427,6 +8431,11 @@
           <t>Месяцы</t>
         </is>
       </c>
+      <c r="M2" s="62" t="inlineStr">
+        <is>
+          <t>Годы</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -8474,6 +8483,9 @@
           <t>Январь</t>
         </is>
       </c>
+      <c r="M3" s="31" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -8521,6 +8533,9 @@
           <t>Февраль</t>
         </is>
       </c>
+      <c r="M4" s="31" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -8568,6 +8583,9 @@
           <t>Март</t>
         </is>
       </c>
+      <c r="M5" s="31" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="16" t="inlineStr">
@@ -8600,6 +8618,9 @@
           <t>Апрель</t>
         </is>
       </c>
+      <c r="M6" s="31" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="16" t="inlineStr">
@@ -8627,6 +8648,9 @@
           <t>Май</t>
         </is>
       </c>
+      <c r="M7" s="31" t="n">
+        <v>2027</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="16" t="inlineStr">
@@ -8654,6 +8678,9 @@
           <t>Июнь</t>
         </is>
       </c>
+      <c r="M8" s="31" t="n">
+        <v>2028</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="16" t="inlineStr">
@@ -8681,6 +8708,9 @@
           <t>Июль</t>
         </is>
       </c>
+      <c r="M9" s="31" t="n">
+        <v>2029</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="16" t="inlineStr">
@@ -8703,6 +8733,9 @@
           <t>Август</t>
         </is>
       </c>
+      <c r="M10" s="31" t="n">
+        <v>2030</v>
+      </c>
     </row>
     <row r="11">
       <c r="J11" s="31" t="inlineStr">
@@ -8719,6 +8752,9 @@
         <is>
           <t>Сентябрь</t>
         </is>
+      </c>
+      <c r="M11" s="31" t="n">
+        <v>2031</v>
       </c>
     </row>
     <row r="12">
@@ -8738,6 +8774,9 @@
         <is>
           <t>Октябрь</t>
         </is>
+      </c>
+      <c r="M12" s="31" t="n">
+        <v>2032</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Rework Трекер привычек: month/year switcher, more rows, restacked tables
- Replace the fixed start-date cell with Месяц/Год dropdowns (same pattern
  as Бюджет) so the whole day grid shifts to the selected month/year.
- Grow the daily habit grid from 15 to 24 rows (8 examples + 16 blank).
- Move "Ежемесячные привычки" from beside "Еженедельные привычки" to
  underneath it, and give both tables 10 rows instead of 5/2.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6CkgouQ8AhQXxstTSck9L
</commit_message>
<xml_diff>
--- a/Планировщик_Бюджет_Привычки.xlsx
+++ b/Планировщик_Бюджет_Привычки.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
-    <numFmt numFmtId="166" formatCode="#,##0&quot; ₽&quot;"/>
-    <numFmt numFmtId="167" formatCode="#,##0&quot; ₽&quot;;[RED]-#,##0&quot; ₽&quot;"/>
+    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="165" formatCode="#,##0&quot; ₽&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; ₽&quot;;[RED]-#,##0&quot; ₽&quot;"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -212,7 +212,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -224,15 +224,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -241,7 +241,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -273,7 +273,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4648,7 +4648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG39"/>
+  <dimension ref="A1:AG65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4659,8 +4659,8 @@
     <col width="3.4" customWidth="1" min="6" max="6"/>
     <col width="3.4" customWidth="1" min="7" max="7"/>
     <col width="3.4" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="3.4" customWidth="1" min="9" max="9"/>
+    <col width="3.4" customWidth="1" min="10" max="10"/>
     <col width="3.4" customWidth="1" min="11" max="11"/>
     <col width="3.4" customWidth="1" min="12" max="12"/>
     <col width="3.4" customWidth="1" min="13" max="13"/>
@@ -4728,16 +4728,26 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Дата начала месяца:</t>
-        </is>
-      </c>
-      <c r="B2" s="26" t="n">
-        <v>46204</v>
+          <t>Месяц:</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Июль</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Год:</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="n">
+        <v>2026</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="27">
-        <f>UPPER(TEXT($B$2,"mmmm"))&amp;CHAR(10)&amp;TEXT($B$2,"d mmmm yyyy")</f>
+        <f>UPPER(TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1),"mmmm"))&amp;CHAR(10)&amp;TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1),"d mmmm yyyy")</f>
         <v/>
       </c>
       <c r="C4" s="13" t="inlineStr">
@@ -4795,253 +4805,253 @@
     <row r="5">
       <c r="B5" s="12" t="n"/>
       <c r="C5" s="15">
-        <f>TEXT($B$2+0,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+0,"ddd")</f>
         <v/>
       </c>
       <c r="D5" s="15">
-        <f>TEXT($B$2+1,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+1,"ddd")</f>
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>TEXT($B$2+2,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+2,"ddd")</f>
         <v/>
       </c>
       <c r="F5" s="15">
-        <f>TEXT($B$2+3,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+3,"ddd")</f>
         <v/>
       </c>
       <c r="G5" s="15">
-        <f>TEXT($B$2+4,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+4,"ddd")</f>
         <v/>
       </c>
       <c r="H5" s="15">
-        <f>TEXT($B$2+5,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+5,"ddd")</f>
         <v/>
       </c>
       <c r="I5" s="15">
-        <f>TEXT($B$2+6,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+6,"ddd")</f>
         <v/>
       </c>
       <c r="J5" s="15">
-        <f>TEXT($B$2+7,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+7,"ddd")</f>
         <v/>
       </c>
       <c r="K5" s="15">
-        <f>TEXT($B$2+8,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+8,"ddd")</f>
         <v/>
       </c>
       <c r="L5" s="15">
-        <f>TEXT($B$2+9,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+9,"ddd")</f>
         <v/>
       </c>
       <c r="M5" s="15">
-        <f>TEXT($B$2+10,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+10,"ddd")</f>
         <v/>
       </c>
       <c r="N5" s="15">
-        <f>TEXT($B$2+11,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+11,"ddd")</f>
         <v/>
       </c>
       <c r="O5" s="15">
-        <f>TEXT($B$2+12,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+12,"ddd")</f>
         <v/>
       </c>
       <c r="P5" s="15">
-        <f>TEXT($B$2+13,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+13,"ddd")</f>
         <v/>
       </c>
       <c r="Q5" s="15">
-        <f>TEXT($B$2+14,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+14,"ddd")</f>
         <v/>
       </c>
       <c r="R5" s="15">
-        <f>TEXT($B$2+15,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+15,"ddd")</f>
         <v/>
       </c>
       <c r="S5" s="15">
-        <f>TEXT($B$2+16,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+16,"ddd")</f>
         <v/>
       </c>
       <c r="T5" s="15">
-        <f>TEXT($B$2+17,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+17,"ddd")</f>
         <v/>
       </c>
       <c r="U5" s="15">
-        <f>TEXT($B$2+18,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+18,"ddd")</f>
         <v/>
       </c>
       <c r="V5" s="15">
-        <f>TEXT($B$2+19,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+19,"ddd")</f>
         <v/>
       </c>
       <c r="W5" s="15">
-        <f>TEXT($B$2+20,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+20,"ddd")</f>
         <v/>
       </c>
       <c r="X5" s="15">
-        <f>TEXT($B$2+21,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+21,"ddd")</f>
         <v/>
       </c>
       <c r="Y5" s="15">
-        <f>TEXT($B$2+22,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+22,"ddd")</f>
         <v/>
       </c>
       <c r="Z5" s="15">
-        <f>TEXT($B$2+23,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+23,"ddd")</f>
         <v/>
       </c>
       <c r="AA5" s="15">
-        <f>TEXT($B$2+24,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+24,"ddd")</f>
         <v/>
       </c>
       <c r="AB5" s="15">
-        <f>TEXT($B$2+25,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+25,"ddd")</f>
         <v/>
       </c>
       <c r="AC5" s="15">
-        <f>TEXT($B$2+26,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+26,"ddd")</f>
         <v/>
       </c>
       <c r="AD5" s="15">
-        <f>TEXT($B$2+27,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+27,"ddd")</f>
         <v/>
       </c>
       <c r="AE5" s="15">
-        <f>TEXT($B$2+28,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+28,"ddd")</f>
         <v/>
       </c>
       <c r="AF5" s="15">
-        <f>TEXT($B$2+29,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+29,"ddd")</f>
         <v/>
       </c>
       <c r="AG5" s="15">
-        <f>TEXT($B$2+30,"ddd")</f>
+        <f>TEXT(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+30,"ddd")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="30">
-        <f>DAY($B$2+0)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+0)</f>
         <v/>
       </c>
       <c r="D6" s="30">
-        <f>DAY($B$2+1)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+1)</f>
         <v/>
       </c>
       <c r="E6" s="30">
-        <f>DAY($B$2+2)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+2)</f>
         <v/>
       </c>
       <c r="F6" s="30">
-        <f>DAY($B$2+3)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+3)</f>
         <v/>
       </c>
       <c r="G6" s="30">
-        <f>DAY($B$2+4)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+4)</f>
         <v/>
       </c>
       <c r="H6" s="30">
-        <f>DAY($B$2+5)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+5)</f>
         <v/>
       </c>
       <c r="I6" s="30">
-        <f>DAY($B$2+6)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+6)</f>
         <v/>
       </c>
       <c r="J6" s="30">
-        <f>DAY($B$2+7)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+7)</f>
         <v/>
       </c>
       <c r="K6" s="30">
-        <f>DAY($B$2+8)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+8)</f>
         <v/>
       </c>
       <c r="L6" s="30">
-        <f>DAY($B$2+9)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+9)</f>
         <v/>
       </c>
       <c r="M6" s="30">
-        <f>DAY($B$2+10)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+10)</f>
         <v/>
       </c>
       <c r="N6" s="30">
-        <f>DAY($B$2+11)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+11)</f>
         <v/>
       </c>
       <c r="O6" s="30">
-        <f>DAY($B$2+12)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+12)</f>
         <v/>
       </c>
       <c r="P6" s="30">
-        <f>DAY($B$2+13)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+13)</f>
         <v/>
       </c>
       <c r="Q6" s="30">
-        <f>DAY($B$2+14)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+14)</f>
         <v/>
       </c>
       <c r="R6" s="30">
-        <f>DAY($B$2+15)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+15)</f>
         <v/>
       </c>
       <c r="S6" s="30">
-        <f>DAY($B$2+16)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+16)</f>
         <v/>
       </c>
       <c r="T6" s="30">
-        <f>DAY($B$2+17)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+17)</f>
         <v/>
       </c>
       <c r="U6" s="30">
-        <f>DAY($B$2+18)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+18)</f>
         <v/>
       </c>
       <c r="V6" s="30">
-        <f>DAY($B$2+19)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+19)</f>
         <v/>
       </c>
       <c r="W6" s="30">
-        <f>DAY($B$2+20)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+20)</f>
         <v/>
       </c>
       <c r="X6" s="30">
-        <f>DAY($B$2+21)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+21)</f>
         <v/>
       </c>
       <c r="Y6" s="30">
-        <f>DAY($B$2+22)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+22)</f>
         <v/>
       </c>
       <c r="Z6" s="30">
-        <f>DAY($B$2+23)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+23)</f>
         <v/>
       </c>
       <c r="AA6" s="30">
-        <f>DAY($B$2+24)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+24)</f>
         <v/>
       </c>
       <c r="AB6" s="30">
-        <f>DAY($B$2+25)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+25)</f>
         <v/>
       </c>
       <c r="AC6" s="30">
-        <f>DAY($B$2+26)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+26)</f>
         <v/>
       </c>
       <c r="AD6" s="30">
-        <f>DAY($B$2+27)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+27)</f>
         <v/>
       </c>
       <c r="AE6" s="30">
-        <f>DAY($B$2+28)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+28)</f>
         <v/>
       </c>
       <c r="AF6" s="30">
-        <f>DAY($B$2+29)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+29)</f>
         <v/>
       </c>
       <c r="AG6" s="30">
-        <f>DAY($B$2+30)</f>
+        <f>DAY(DATE($D$2,MATCH($B$2,Справочник!$L$3:$L$14,0),1)+30)</f>
         <v/>
       </c>
     </row>
@@ -6563,442 +6573,505 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>ВЫПОЛНЕНЫ</t>
-        </is>
-      </c>
-      <c r="C22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",C7:C21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="D22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",D7:D21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="E22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",E7:E21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="F22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",F7:F21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="G22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",G7:G21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="H22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",H7:H21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="I22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",I7:I21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="J22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",J7:J21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="K22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",K7:K21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="L22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",L7:L21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="M22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",M7:M21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="N22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",N7:N21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="O22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",O7:O21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="P22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",P7:P21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",Q7:Q21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="R22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",R7:R21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="S22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",S7:S21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="T22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",T7:T21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="U22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",U7:U21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="V22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",V7:V21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="W22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",W7:W21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="X22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",X7:X21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="Y22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",Y7:Y21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="Z22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",Z7:Z21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AA22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AA7:AA21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AB22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AB7:AB21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AC22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AC7:AC21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AD22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AD7:AD21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AE22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AE7:AE21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AF22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AF7:AF21,TRUE)</f>
-        <v/>
-      </c>
-      <c r="AG22" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AG7:AG21,TRUE)</f>
-        <v/>
+      <c r="A22" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="32" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>НЕВЫПОЛНЕНЫ</t>
-        </is>
-      </c>
-      <c r="C23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",C7:C21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",D7:D21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="E23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",E7:E21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",F7:F21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="G23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",G7:G21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="H23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",H7:H21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="I23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",I7:I21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",J7:J21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",K7:K21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="L23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",L7:L21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="M23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",M7:M21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="N23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",N7:N21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="O23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",O7:O21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="P23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",P7:P21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="Q23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",Q7:Q21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="R23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",R7:R21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="S23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",S7:S21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="T23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",T7:T21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="U23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",U7:U21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="V23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",V7:V21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="W23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",W7:W21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="X23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",X7:X21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="Y23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",Y7:Y21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="Z23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",Z7:Z21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AA23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AA7:AA21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AB23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AB7:AB21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AC23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AC7:AC21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AD23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AD7:AD21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AE23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AE7:AE21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AF23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AF7:AF21,FALSE)</f>
-        <v/>
-      </c>
-      <c r="AG23" s="34">
-        <f>COUNTIFS($B$7:$B$21,"&lt;&gt;",AG7:AG21,FALSE)</f>
-        <v/>
+      <c r="A23" s="31" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="32" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t>ПРОГРЕСС %</t>
-        </is>
-      </c>
-      <c r="C24" s="35">
-        <f>IFERROR(C22/(C22+C23),0)</f>
-        <v/>
-      </c>
-      <c r="D24" s="35">
-        <f>IFERROR(D22/(D22+D23),0)</f>
-        <v/>
-      </c>
-      <c r="E24" s="35">
-        <f>IFERROR(E22/(E22+E23),0)</f>
-        <v/>
-      </c>
-      <c r="F24" s="35">
-        <f>IFERROR(F22/(F22+F23),0)</f>
-        <v/>
-      </c>
-      <c r="G24" s="35">
-        <f>IFERROR(G22/(G22+G23),0)</f>
-        <v/>
-      </c>
-      <c r="H24" s="35">
-        <f>IFERROR(H22/(H22+H23),0)</f>
-        <v/>
-      </c>
-      <c r="I24" s="35">
-        <f>IFERROR(I22/(I22+I23),0)</f>
-        <v/>
-      </c>
-      <c r="J24" s="35">
-        <f>IFERROR(J22/(J22+J23),0)</f>
-        <v/>
-      </c>
-      <c r="K24" s="35">
-        <f>IFERROR(K22/(K22+K23),0)</f>
-        <v/>
-      </c>
-      <c r="L24" s="35">
-        <f>IFERROR(L22/(L22+L23),0)</f>
-        <v/>
-      </c>
-      <c r="M24" s="35">
-        <f>IFERROR(M22/(M22+M23),0)</f>
-        <v/>
-      </c>
-      <c r="N24" s="35">
-        <f>IFERROR(N22/(N22+N23),0)</f>
-        <v/>
-      </c>
-      <c r="O24" s="35">
-        <f>IFERROR(O22/(O22+O23),0)</f>
-        <v/>
-      </c>
-      <c r="P24" s="35">
-        <f>IFERROR(P22/(P22+P23),0)</f>
-        <v/>
-      </c>
-      <c r="Q24" s="35">
-        <f>IFERROR(Q22/(Q22+Q23),0)</f>
-        <v/>
-      </c>
-      <c r="R24" s="35">
-        <f>IFERROR(R22/(R22+R23),0)</f>
-        <v/>
-      </c>
-      <c r="S24" s="35">
-        <f>IFERROR(S22/(S22+S23),0)</f>
-        <v/>
-      </c>
-      <c r="T24" s="35">
-        <f>IFERROR(T22/(T22+T23),0)</f>
-        <v/>
-      </c>
-      <c r="U24" s="35">
-        <f>IFERROR(U22/(U22+U23),0)</f>
-        <v/>
-      </c>
-      <c r="V24" s="35">
-        <f>IFERROR(V22/(V22+V23),0)</f>
-        <v/>
-      </c>
-      <c r="W24" s="35">
-        <f>IFERROR(W22/(W22+W23),0)</f>
-        <v/>
-      </c>
-      <c r="X24" s="35">
-        <f>IFERROR(X22/(X22+X23),0)</f>
-        <v/>
-      </c>
-      <c r="Y24" s="35">
-        <f>IFERROR(Y22/(Y22+Y23),0)</f>
-        <v/>
-      </c>
-      <c r="Z24" s="35">
-        <f>IFERROR(Z22/(Z22+Z23),0)</f>
-        <v/>
-      </c>
-      <c r="AA24" s="35">
-        <f>IFERROR(AA22/(AA22+AA23),0)</f>
-        <v/>
-      </c>
-      <c r="AB24" s="35">
-        <f>IFERROR(AB22/(AB22+AB23),0)</f>
-        <v/>
-      </c>
-      <c r="AC24" s="35">
-        <f>IFERROR(AC22/(AC22+AC23),0)</f>
-        <v/>
-      </c>
-      <c r="AD24" s="35">
-        <f>IFERROR(AD22/(AD22+AD23),0)</f>
-        <v/>
-      </c>
-      <c r="AE24" s="35">
-        <f>IFERROR(AE22/(AE22+AE23),0)</f>
-        <v/>
-      </c>
-      <c r="AF24" s="35">
-        <f>IFERROR(AF22/(AF22+AF23),0)</f>
-        <v/>
-      </c>
-      <c r="AG24" s="35">
-        <f>IFERROR(AG22/(AG22+AG23),0)</f>
-        <v/>
+      <c r="A24" s="31" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF24" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG24" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG25" s="32" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>ЕЖЕНЕДЕЛЬНЫЕ ПРИВЫЧКИ</t>
-        </is>
-      </c>
-      <c r="C26" s="36" t="inlineStr">
-        <is>
-          <t>НЕДЕЛЯ 1</t>
-        </is>
-      </c>
-      <c r="D26" s="36" t="inlineStr">
-        <is>
-          <t>НЕДЕЛЯ 2</t>
-        </is>
-      </c>
-      <c r="E26" s="36" t="inlineStr">
-        <is>
-          <t>НЕДЕЛЯ 3</t>
-        </is>
-      </c>
-      <c r="F26" s="36" t="inlineStr">
-        <is>
-          <t>НЕДЕЛЯ 4</t>
-        </is>
-      </c>
-      <c r="G26" s="36" t="inlineStr">
-        <is>
-          <t>НЕДЕЛЯ 5</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="inlineStr">
-        <is>
-          <t>ЕЖЕМЕСЯЧНЫЕ ПРИВЫЧКИ</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="n"/>
+      <c r="A26" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>🏋 Спортзал 3 раза в неделю</t>
-        </is>
-      </c>
+      <c r="A27" s="31" t="n">
+        <v>21</v>
+      </c>
+      <c r="B27" s="16" t="n"/>
       <c r="C27" s="32" t="b">
         <v>0</v>
       </c>
@@ -7014,21 +7087,90 @@
       <c r="G27" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="I27" s="16" t="inlineStr">
-        <is>
-          <t>📏 Сделать замеры до/после</t>
-        </is>
+      <c r="H27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" s="32" t="b">
+        <v>0</v>
       </c>
       <c r="J27" s="32" t="b">
         <v>0</v>
       </c>
+      <c r="K27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG27" s="32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>💰 Анализ расходов</t>
-        </is>
-      </c>
+      <c r="A28" s="31" t="n">
+        <v>22</v>
+      </c>
+      <c r="B28" s="16" t="n"/>
       <c r="C28" s="32" t="b">
         <v>0</v>
       </c>
@@ -7044,12 +7186,89 @@
       <c r="G28" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="I28" s="16" t="n"/>
+      <c r="H28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" s="32" t="b">
+        <v>0</v>
+      </c>
       <c r="J28" s="32" t="b">
         <v>0</v>
       </c>
+      <c r="K28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG28" s="32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
+      <c r="A29" s="31" t="n">
+        <v>23</v>
+      </c>
       <c r="B29" s="16" t="n"/>
       <c r="C29" s="32" t="b">
         <v>0</v>
@@ -7066,8 +7285,89 @@
       <c r="G29" s="32" t="b">
         <v>0</v>
       </c>
+      <c r="H29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
+      <c r="A30" s="31" t="n">
+        <v>24</v>
+      </c>
       <c r="B30" s="16" t="n"/>
       <c r="C30" s="32" t="b">
         <v>0</v>
@@ -7084,166 +7384,910 @@
       <c r="G30" s="32" t="b">
         <v>0</v>
       </c>
+      <c r="H30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="L30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="V30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="W30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="X30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG30" s="32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
-      <c r="B31" s="16" t="n"/>
-      <c r="C31" s="32" t="b">
-        <v>0</v>
-      </c>
-      <c r="D31" s="32" t="b">
-        <v>0</v>
-      </c>
-      <c r="E31" s="32" t="b">
-        <v>0</v>
-      </c>
-      <c r="F31" s="32" t="b">
-        <v>0</v>
-      </c>
-      <c r="G31" s="32" t="b">
-        <v>0</v>
+      <c r="B31" s="33" t="inlineStr">
+        <is>
+          <t>ВЫПОЛНЕНЫ</t>
+        </is>
+      </c>
+      <c r="C31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",C7:C30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="D31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",D7:D30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="E31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",E7:E30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="F31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",F7:F30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="G31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",G7:G30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="H31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",H7:H30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="I31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",I7:I30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="J31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",J7:J30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="K31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",K7:K30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="L31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",L7:L30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="M31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",M7:M30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="N31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",N7:N30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="O31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",O7:O30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="P31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",P7:P30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="Q31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",Q7:Q30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="R31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",R7:R30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="S31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",S7:S30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="T31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",T7:T30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="U31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",U7:U30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="V31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",V7:V30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="W31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",W7:W30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="X31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",X7:X30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="Y31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",Y7:Y30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="Z31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",Z7:Z30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AA31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AA7:AA30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AB31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AB7:AB30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AC31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AC7:AC30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AD31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AD7:AD30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AE31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AE7:AE30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AF31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AF7:AF30,TRUE)</f>
+        <v/>
+      </c>
+      <c r="AG31" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AG7:AG30,TRUE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="33" t="inlineStr">
+        <is>
+          <t>НЕВЫПОЛНЕНЫ</t>
+        </is>
+      </c>
+      <c r="C32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",C7:C30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",D7:D30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",E7:E30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",F7:F30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",G7:G30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="H32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",H7:H30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",I7:I30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",J7:J30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",K7:K30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="L32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",L7:L30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="M32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",M7:M30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="N32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",N7:N30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="O32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",O7:O30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="P32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",P7:P30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="Q32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",Q7:Q30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="R32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",R7:R30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="S32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",S7:S30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="T32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",T7:T30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="U32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",U7:U30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",V7:V30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="W32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",W7:W30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",X7:X30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="Y32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",Y7:Y30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="Z32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",Z7:Z30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AA32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AA7:AA30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AB32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AB7:AB30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AC32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AC7:AC30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AD32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AD7:AD30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AE32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AE7:AE30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AF32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AF7:AF30,FALSE)</f>
+        <v/>
+      </c>
+      <c r="AG32" s="34">
+        <f>COUNTIFS($B$7:$B$30,"&lt;&gt;",AG7:AG30,FALSE)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="33" t="inlineStr">
+        <is>
+          <t>ПРОГРЕСС %</t>
+        </is>
+      </c>
+      <c r="C33" s="35">
+        <f>IFERROR(C31/(C31+C32),0)</f>
+        <v/>
+      </c>
+      <c r="D33" s="35">
+        <f>IFERROR(D31/(D31+D32),0)</f>
+        <v/>
+      </c>
+      <c r="E33" s="35">
+        <f>IFERROR(E31/(E31+E32),0)</f>
+        <v/>
+      </c>
+      <c r="F33" s="35">
+        <f>IFERROR(F31/(F31+F32),0)</f>
+        <v/>
+      </c>
+      <c r="G33" s="35">
+        <f>IFERROR(G31/(G31+G32),0)</f>
+        <v/>
+      </c>
+      <c r="H33" s="35">
+        <f>IFERROR(H31/(H31+H32),0)</f>
+        <v/>
+      </c>
+      <c r="I33" s="35">
+        <f>IFERROR(I31/(I31+I32),0)</f>
+        <v/>
+      </c>
+      <c r="J33" s="35">
+        <f>IFERROR(J31/(J31+J32),0)</f>
+        <v/>
+      </c>
+      <c r="K33" s="35">
+        <f>IFERROR(K31/(K31+K32),0)</f>
+        <v/>
+      </c>
+      <c r="L33" s="35">
+        <f>IFERROR(L31/(L31+L32),0)</f>
+        <v/>
+      </c>
+      <c r="M33" s="35">
+        <f>IFERROR(M31/(M31+M32),0)</f>
+        <v/>
+      </c>
+      <c r="N33" s="35">
+        <f>IFERROR(N31/(N31+N32),0)</f>
+        <v/>
+      </c>
+      <c r="O33" s="35">
+        <f>IFERROR(O31/(O31+O32),0)</f>
+        <v/>
+      </c>
+      <c r="P33" s="35">
+        <f>IFERROR(P31/(P31+P32),0)</f>
+        <v/>
+      </c>
+      <c r="Q33" s="35">
+        <f>IFERROR(Q31/(Q31+Q32),0)</f>
+        <v/>
+      </c>
+      <c r="R33" s="35">
+        <f>IFERROR(R31/(R31+R32),0)</f>
+        <v/>
+      </c>
+      <c r="S33" s="35">
+        <f>IFERROR(S31/(S31+S32),0)</f>
+        <v/>
+      </c>
+      <c r="T33" s="35">
+        <f>IFERROR(T31/(T31+T32),0)</f>
+        <v/>
+      </c>
+      <c r="U33" s="35">
+        <f>IFERROR(U31/(U31+U32),0)</f>
+        <v/>
+      </c>
+      <c r="V33" s="35">
+        <f>IFERROR(V31/(V31+V32),0)</f>
+        <v/>
+      </c>
+      <c r="W33" s="35">
+        <f>IFERROR(W31/(W31+W32),0)</f>
+        <v/>
+      </c>
+      <c r="X33" s="35">
+        <f>IFERROR(X31/(X31+X32),0)</f>
+        <v/>
+      </c>
+      <c r="Y33" s="35">
+        <f>IFERROR(Y31/(Y31+Y32),0)</f>
+        <v/>
+      </c>
+      <c r="Z33" s="35">
+        <f>IFERROR(Z31/(Z31+Z32),0)</f>
+        <v/>
+      </c>
+      <c r="AA33" s="35">
+        <f>IFERROR(AA31/(AA31+AA32),0)</f>
+        <v/>
+      </c>
+      <c r="AB33" s="35">
+        <f>IFERROR(AB31/(AB31+AB32),0)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="35">
+        <f>IFERROR(AC31/(AC31+AC32),0)</f>
+        <v/>
+      </c>
+      <c r="AD33" s="35">
+        <f>IFERROR(AD31/(AD31+AD32),0)</f>
+        <v/>
+      </c>
+      <c r="AE33" s="35">
+        <f>IFERROR(AE31/(AE31+AE32),0)</f>
+        <v/>
+      </c>
+      <c r="AF33" s="35">
+        <f>IFERROR(AF31/(AF31+AF32),0)</f>
+        <v/>
+      </c>
+      <c r="AG33" s="35">
+        <f>IFERROR(AG31/(AG31+AG32),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>ЕЖЕНЕДЕЛЬНЫЕ ПРИВЫЧКИ</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t>НЕДЕЛЯ 1</t>
+        </is>
+      </c>
+      <c r="D35" s="36" t="inlineStr">
+        <is>
+          <t>НЕДЕЛЯ 2</t>
+        </is>
+      </c>
+      <c r="E35" s="36" t="inlineStr">
+        <is>
+          <t>НЕДЕЛЯ 3</t>
+        </is>
+      </c>
+      <c r="F35" s="36" t="inlineStr">
+        <is>
+          <t>НЕДЕЛЯ 4</t>
+        </is>
+      </c>
+      <c r="G35" s="36" t="inlineStr">
+        <is>
+          <t>НЕДЕЛЯ 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>🏋 Спортзал 3 раза в неделю</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D36" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>💰 Анализ расходов</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D37" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F37" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G37" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="16" t="n"/>
+      <c r="C38" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D38" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F38" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G38" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="16" t="n"/>
+      <c r="C39" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D39" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F39" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G39" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="16" t="n"/>
+      <c r="C40" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D40" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F40" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G40" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="16" t="n"/>
+      <c r="C41" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G41" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="16" t="n"/>
+      <c r="C42" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D42" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F42" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G42" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="16" t="n"/>
+      <c r="C43" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D43" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E43" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G43" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="16" t="n"/>
+      <c r="C44" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D44" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E44" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F44" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G44" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="16" t="n"/>
+      <c r="C45" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D45" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E45" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F45" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G45" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>ЕЖЕМЕСЯЧНЫЕ ПРИВЫЧКИ</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>📏 Сделать замеры до/после</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="16" t="n"/>
+      <c r="C49" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="16" t="n"/>
+      <c r="C50" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="16" t="n"/>
+      <c r="C51" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="16" t="n"/>
+      <c r="C52" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="16" t="n"/>
+      <c r="C53" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="16" t="n"/>
+      <c r="C54" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="16" t="n"/>
+      <c r="C55" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="16" t="n"/>
+      <c r="C56" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="16" t="n"/>
+      <c r="C57" s="32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="13" t="inlineStr">
         <is>
           <t>ЗАМЕТКИ</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="14" t="n"/>
-      <c r="I33" s="14" t="n"/>
-      <c r="J33" s="14" t="n"/>
-      <c r="K33" s="14" t="n"/>
-      <c r="L33" s="14" t="n"/>
-      <c r="M33" s="14" t="n"/>
-      <c r="N33" s="14" t="n"/>
-      <c r="O33" s="14" t="n"/>
-      <c r="P33" s="14" t="n"/>
-    </row>
-    <row r="34">
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="37" t="n"/>
-      <c r="D34" s="37" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="37" t="n"/>
-      <c r="G34" s="37" t="n"/>
-      <c r="H34" s="37" t="n"/>
-      <c r="I34" s="37" t="n"/>
-      <c r="J34" s="37" t="n"/>
-      <c r="K34" s="37" t="n"/>
-      <c r="L34" s="37" t="n"/>
-      <c r="M34" s="37" t="n"/>
-      <c r="N34" s="37" t="n"/>
-      <c r="O34" s="37" t="n"/>
-      <c r="P34" s="37" t="n"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="37" t="n"/>
-      <c r="C35" s="37" t="n"/>
-      <c r="D35" s="37" t="n"/>
-      <c r="E35" s="37" t="n"/>
-      <c r="F35" s="37" t="n"/>
-      <c r="G35" s="37" t="n"/>
-      <c r="H35" s="37" t="n"/>
-      <c r="I35" s="37" t="n"/>
-      <c r="J35" s="37" t="n"/>
-      <c r="K35" s="37" t="n"/>
-      <c r="L35" s="37" t="n"/>
-      <c r="M35" s="37" t="n"/>
-      <c r="N35" s="37" t="n"/>
-      <c r="O35" s="37" t="n"/>
-      <c r="P35" s="37" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="37" t="n"/>
-      <c r="C36" s="37" t="n"/>
-      <c r="D36" s="37" t="n"/>
-      <c r="E36" s="37" t="n"/>
-      <c r="F36" s="37" t="n"/>
-      <c r="G36" s="37" t="n"/>
-      <c r="H36" s="37" t="n"/>
-      <c r="I36" s="37" t="n"/>
-      <c r="J36" s="37" t="n"/>
-      <c r="K36" s="37" t="n"/>
-      <c r="L36" s="37" t="n"/>
-      <c r="M36" s="37" t="n"/>
-      <c r="N36" s="37" t="n"/>
-      <c r="O36" s="37" t="n"/>
-      <c r="P36" s="37" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="D37" s="37" t="n"/>
-      <c r="E37" s="37" t="n"/>
-      <c r="F37" s="37" t="n"/>
-      <c r="G37" s="37" t="n"/>
-      <c r="H37" s="37" t="n"/>
-      <c r="I37" s="37" t="n"/>
-      <c r="J37" s="37" t="n"/>
-      <c r="K37" s="37" t="n"/>
-      <c r="L37" s="37" t="n"/>
-      <c r="M37" s="37" t="n"/>
-      <c r="N37" s="37" t="n"/>
-      <c r="O37" s="37" t="n"/>
-      <c r="P37" s="37" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="37" t="n"/>
-      <c r="D38" s="37" t="n"/>
-      <c r="E38" s="37" t="n"/>
-      <c r="F38" s="37" t="n"/>
-      <c r="G38" s="37" t="n"/>
-      <c r="H38" s="37" t="n"/>
-      <c r="I38" s="37" t="n"/>
-      <c r="J38" s="37" t="n"/>
-      <c r="K38" s="37" t="n"/>
-      <c r="L38" s="37" t="n"/>
-      <c r="M38" s="37" t="n"/>
-      <c r="N38" s="37" t="n"/>
-      <c r="O38" s="37" t="n"/>
-      <c r="P38" s="37" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="37" t="n"/>
-      <c r="C39" s="37" t="n"/>
-      <c r="D39" s="37" t="n"/>
-      <c r="E39" s="37" t="n"/>
-      <c r="F39" s="37" t="n"/>
-      <c r="G39" s="37" t="n"/>
-      <c r="H39" s="37" t="n"/>
-      <c r="I39" s="37" t="n"/>
-      <c r="J39" s="37" t="n"/>
-      <c r="K39" s="37" t="n"/>
-      <c r="L39" s="37" t="n"/>
-      <c r="M39" s="37" t="n"/>
-      <c r="N39" s="37" t="n"/>
-      <c r="O39" s="37" t="n"/>
-      <c r="P39" s="37" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="14" t="n"/>
+      <c r="F59" s="14" t="n"/>
+      <c r="G59" s="14" t="n"/>
+      <c r="H59" s="14" t="n"/>
+      <c r="I59" s="14" t="n"/>
+      <c r="J59" s="14" t="n"/>
+      <c r="K59" s="14" t="n"/>
+      <c r="L59" s="14" t="n"/>
+      <c r="M59" s="14" t="n"/>
+      <c r="N59" s="14" t="n"/>
+      <c r="O59" s="14" t="n"/>
+      <c r="P59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="37" t="n"/>
+      <c r="C60" s="37" t="n"/>
+      <c r="D60" s="37" t="n"/>
+      <c r="E60" s="37" t="n"/>
+      <c r="F60" s="37" t="n"/>
+      <c r="G60" s="37" t="n"/>
+      <c r="H60" s="37" t="n"/>
+      <c r="I60" s="37" t="n"/>
+      <c r="J60" s="37" t="n"/>
+      <c r="K60" s="37" t="n"/>
+      <c r="L60" s="37" t="n"/>
+      <c r="M60" s="37" t="n"/>
+      <c r="N60" s="37" t="n"/>
+      <c r="O60" s="37" t="n"/>
+      <c r="P60" s="37" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="37" t="n"/>
+      <c r="C61" s="37" t="n"/>
+      <c r="D61" s="37" t="n"/>
+      <c r="E61" s="37" t="n"/>
+      <c r="F61" s="37" t="n"/>
+      <c r="G61" s="37" t="n"/>
+      <c r="H61" s="37" t="n"/>
+      <c r="I61" s="37" t="n"/>
+      <c r="J61" s="37" t="n"/>
+      <c r="K61" s="37" t="n"/>
+      <c r="L61" s="37" t="n"/>
+      <c r="M61" s="37" t="n"/>
+      <c r="N61" s="37" t="n"/>
+      <c r="O61" s="37" t="n"/>
+      <c r="P61" s="37" t="n"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="37" t="n"/>
+      <c r="C62" s="37" t="n"/>
+      <c r="D62" s="37" t="n"/>
+      <c r="E62" s="37" t="n"/>
+      <c r="F62" s="37" t="n"/>
+      <c r="G62" s="37" t="n"/>
+      <c r="H62" s="37" t="n"/>
+      <c r="I62" s="37" t="n"/>
+      <c r="J62" s="37" t="n"/>
+      <c r="K62" s="37" t="n"/>
+      <c r="L62" s="37" t="n"/>
+      <c r="M62" s="37" t="n"/>
+      <c r="N62" s="37" t="n"/>
+      <c r="O62" s="37" t="n"/>
+      <c r="P62" s="37" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="37" t="n"/>
+      <c r="C63" s="37" t="n"/>
+      <c r="D63" s="37" t="n"/>
+      <c r="E63" s="37" t="n"/>
+      <c r="F63" s="37" t="n"/>
+      <c r="G63" s="37" t="n"/>
+      <c r="H63" s="37" t="n"/>
+      <c r="I63" s="37" t="n"/>
+      <c r="J63" s="37" t="n"/>
+      <c r="K63" s="37" t="n"/>
+      <c r="L63" s="37" t="n"/>
+      <c r="M63" s="37" t="n"/>
+      <c r="N63" s="37" t="n"/>
+      <c r="O63" s="37" t="n"/>
+      <c r="P63" s="37" t="n"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="37" t="n"/>
+      <c r="C64" s="37" t="n"/>
+      <c r="D64" s="37" t="n"/>
+      <c r="E64" s="37" t="n"/>
+      <c r="F64" s="37" t="n"/>
+      <c r="G64" s="37" t="n"/>
+      <c r="H64" s="37" t="n"/>
+      <c r="I64" s="37" t="n"/>
+      <c r="J64" s="37" t="n"/>
+      <c r="K64" s="37" t="n"/>
+      <c r="L64" s="37" t="n"/>
+      <c r="M64" s="37" t="n"/>
+      <c r="N64" s="37" t="n"/>
+      <c r="O64" s="37" t="n"/>
+      <c r="P64" s="37" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="37" t="n"/>
+      <c r="C65" s="37" t="n"/>
+      <c r="D65" s="37" t="n"/>
+      <c r="E65" s="37" t="n"/>
+      <c r="F65" s="37" t="n"/>
+      <c r="G65" s="37" t="n"/>
+      <c r="H65" s="37" t="n"/>
+      <c r="I65" s="37" t="n"/>
+      <c r="J65" s="37" t="n"/>
+      <c r="K65" s="37" t="n"/>
+      <c r="L65" s="37" t="n"/>
+      <c r="M65" s="37" t="n"/>
+      <c r="N65" s="37" t="n"/>
+      <c r="O65" s="37" t="n"/>
+      <c r="P65" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="15">
     <mergeCell ref="A1:AG1"/>
-    <mergeCell ref="B33:P33"/>
-    <mergeCell ref="B26"/>
+    <mergeCell ref="B35"/>
+    <mergeCell ref="F35"/>
+    <mergeCell ref="C35"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="E26"/>
-    <mergeCell ref="C26"/>
+    <mergeCell ref="D35"/>
+    <mergeCell ref="E35"/>
     <mergeCell ref="X4:AD4"/>
-    <mergeCell ref="D26"/>
-    <mergeCell ref="F26"/>
+    <mergeCell ref="G35"/>
+    <mergeCell ref="B47:C47"/>
     <mergeCell ref="Q4:W4"/>
-    <mergeCell ref="G26"/>
+    <mergeCell ref="B59:P59"/>
     <mergeCell ref="C4:I4"/>
-    <mergeCell ref="A2"/>
     <mergeCell ref="J4:P4"/>
     <mergeCell ref="AE4:AG4"/>
-    <mergeCell ref="I26:J26"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:AG7">
     <cfRule type="expression" priority="1" dxfId="1">
@@ -7320,8 +8364,53 @@
       <formula>C21=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C22:AG22">
+    <cfRule type="expression" priority="16" dxfId="1">
+      <formula>C22=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C23:AG23">
+    <cfRule type="expression" priority="17" dxfId="1">
+      <formula>C23=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C24:AG24">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="expression" priority="18" dxfId="1">
+      <formula>C24=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25:AG25">
+    <cfRule type="expression" priority="19" dxfId="1">
+      <formula>C25=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C26:AG26">
+    <cfRule type="expression" priority="20" dxfId="1">
+      <formula>C26=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C27:AG27">
+    <cfRule type="expression" priority="21" dxfId="1">
+      <formula>C27=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C28:AG28">
+    <cfRule type="expression" priority="22" dxfId="1">
+      <formula>C28=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C29:AG29">
+    <cfRule type="expression" priority="23" dxfId="1">
+      <formula>C29=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C30:AG30">
+    <cfRule type="expression" priority="24" dxfId="1">
+      <formula>C30=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C33:AG33">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -7330,42 +8419,23 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27:G27">
-    <cfRule type="expression" priority="17" dxfId="1">
-      <formula>C27=TRUE</formula>
+  <conditionalFormatting sqref="C36:G45">
+    <cfRule type="expression" priority="26" dxfId="1">
+      <formula>C36=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28:G28">
-    <cfRule type="expression" priority="18" dxfId="1">
-      <formula>C28=TRUE</formula>
+  <conditionalFormatting sqref="C48:C57">
+    <cfRule type="expression" priority="27" dxfId="2">
+      <formula>C48=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29:G29">
-    <cfRule type="expression" priority="19" dxfId="1">
-      <formula>C29=TRUE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C30:G30">
-    <cfRule type="expression" priority="20" dxfId="1">
-      <formula>C30=TRUE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31:G31">
-    <cfRule type="expression" priority="21" dxfId="1">
-      <formula>C31=TRUE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J27">
-    <cfRule type="expression" priority="22" dxfId="2">
-      <formula>J27=TRUE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J28">
-    <cfRule type="expression" priority="23" dxfId="2">
-      <formula>J28=TRUE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="22">
+  <dataValidations count="28">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Справочник!$L$3:$L$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Справочник!$M$3:$M$12</formula1>
+    </dataValidation>
     <dataValidation sqref="C7:AG7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
@@ -7411,25 +8481,37 @@
     <dataValidation sqref="C21:AG21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C27:G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C22:AG22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C28:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C23:AG23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C29:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C24:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C30:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C25:AG25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="C31:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C26:AG26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="J27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C27:AG27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="J28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C28:AG28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C29:AG29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C30:AG30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C36:G45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C48:C57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Бюджет: move category/dynamics tables above the journal
"Доходы/Расходы по категориям" and "Динамика за год" were placed after
the 200-row journal (row ~229), effectively invisible without a lot of
scrolling — that's why the yearly dynamics table looked missing. Moved
that whole block (plus its 3 charts) to right after the accounts
dashboard, before the journal. Journal now starts at row 41 instead of 25.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6CkgouQ8AhQXxstTSck9L
</commit_message>
<xml_diff>
--- a/Планировщик_Бюджет_Привычки.xlsx
+++ b/Планировщик_Бюджет_Привычки.xlsx
@@ -230,13 +230,13 @@
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -516,12 +516,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Бюджет'!$D$231:$D$233</f>
+              <f>'Бюджет'!$D$27:$D$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Бюджет'!$E$231:$E$233</f>
+              <f>'Бюджет'!$E$27:$E$29</f>
             </numRef>
           </val>
         </ser>
@@ -568,12 +568,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Бюджет'!$H$231:$H$238</f>
+              <f>'Бюджет'!$H$27:$H$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Бюджет'!$I$231:$I$238</f>
+              <f>'Бюджет'!$I$27:$I$34</f>
             </numRef>
           </val>
         </ser>
@@ -615,7 +615,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Бюджет'!M230</f>
+              <f>'Бюджет'!M26</f>
             </strRef>
           </tx>
           <spPr>
@@ -633,12 +633,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Бюджет'!$L$231:$L$242</f>
+              <f>'Бюджет'!$L$27:$L$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Бюджет'!$M$231:$M$242</f>
+              <f>'Бюджет'!$M$27:$M$38</f>
             </numRef>
           </val>
         </ser>
@@ -647,7 +647,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Бюджет'!N230</f>
+              <f>'Бюджет'!N26</f>
             </strRef>
           </tx>
           <spPr>
@@ -665,12 +665,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Бюджет'!$L$231:$L$242</f>
+              <f>'Бюджет'!$L$27:$L$38</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Бюджет'!$N$231:$N$242</f>
+              <f>'Бюджет'!$N$27:$N$38</f>
             </numRef>
           </val>
         </ser>
@@ -1326,12 +1326,12 @@
     </row>
     <row r="6">
       <c r="B6" s="11">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
         <v/>
       </c>
       <c r="C6" s="12" t="n"/>
       <c r="D6" s="11">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
         <v/>
       </c>
       <c r="E6" s="12" t="n"/>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>IF(B13="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B13,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B13,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B13="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B13,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B13,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
         <v/>
       </c>
       <c r="C14" s="17">
-        <f>IF(B14="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B14,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B14,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B14="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B14,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B14,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
         <v/>
       </c>
       <c r="C15" s="17">
-        <f>IF(B15="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B15,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B15,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B15="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B15,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B15,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
         <v/>
       </c>
       <c r="C16" s="17">
-        <f>IF(B16="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B16,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B16,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B16="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B16,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B16,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
         <v/>
       </c>
       <c r="C17" s="17">
-        <f>IF(B17="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B17,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B17,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B17="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B17,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B17,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
         <v/>
       </c>
       <c r="C18" s="17">
-        <f>IF(B18="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B18,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B18,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B18="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B18,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B18,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
         <v/>
       </c>
       <c r="C19" s="17">
-        <f>IF(B19="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B19,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B19,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B19="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B19,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B19,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
         <v/>
       </c>
       <c r="C20" s="17">
-        <f>IF(B20="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B20,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B20,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B20="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B20,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B20,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
         <v/>
       </c>
       <c r="C21" s="17">
-        <f>IF(B21="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B21,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B21,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B21="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B21,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B21,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
@@ -1476,733 +1476,922 @@
         <v/>
       </c>
       <c r="C22" s="17">
-        <f>IF(B22="","",SUMIFS($F$27:$F$226,$C$27:$C$226,B22,$D$27:$D$226,"Доход")-SUMIFS($F$27:$F$226,$C$27:$C$226,B22,$D$27:$D$226,"Расход"))</f>
+        <f>IF(B22="","",SUMIFS($F$43:$F$242,$C$43:$C$242,B22,$D$43:$D$242,"Доход")-SUMIFS($F$43:$F$242,$C$43:$C$242,B22,$D$43:$D$242,"Расход"))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>✏️  ЖУРНАЛ ОПЕРАЦИЙ — вносите доходы и расходы сюда</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>ДОХОДЫ ПО КАТЕГОРИЯМ (месяц)</t>
+        </is>
+      </c>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>РАСХОДЫ ПО КАТЕГОРИЯМ (месяц)</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8" t="n"/>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>ДИНАМИКА ЗА ГОД</t>
+        </is>
+      </c>
+      <c r="M25" s="14" t="n"/>
+      <c r="N25" s="14" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Категория</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Сумма</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>Категория</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>Сумма</t>
+        </is>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>Месяц</t>
+        </is>
+      </c>
+      <c r="M26" s="15" t="inlineStr">
+        <is>
+          <t>Доход</t>
+        </is>
+      </c>
+      <c r="N26" s="15" t="inlineStr">
+        <is>
+          <t>Расход</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Зарплата</t>
+        </is>
+      </c>
+      <c r="E27" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*($E$43:$E$242="Зарплата")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="F27" s="20">
+        <f>IFERROR(E27/$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>Аренда</t>
+        </is>
+      </c>
+      <c r="I27" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Аренда")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J27" s="20">
+        <f>IFERROR(I27/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="16">
+        <f>TEXT(DATE($F$3,1,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M27" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=1)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N27" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=1)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Заказы</t>
+        </is>
+      </c>
+      <c r="E28" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*($E$43:$E$242="Заказы")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="F28" s="20">
+        <f>IFERROR(E28/$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Продукты</t>
+        </is>
+      </c>
+      <c r="I28" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Продукты")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J28" s="20">
+        <f>IFERROR(I28/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L28" s="16">
+        <f>TEXT(DATE($F$3,2,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M28" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=2)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N28" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=2)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Подарок</t>
+        </is>
+      </c>
+      <c r="E29" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*($E$43:$E$242="Подарок")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="F29" s="20">
+        <f>IFERROR(E29/$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>Обучение</t>
+        </is>
+      </c>
+      <c r="I29" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Обучение")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J29" s="20">
+        <f>IFERROR(I29/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L29" s="16">
+        <f>TEXT(DATE($F$3,3,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M29" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=3)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N29" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=3)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Кредит</t>
+        </is>
+      </c>
+      <c r="I30" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Кредит")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J30" s="20">
+        <f>IFERROR(I30/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L30" s="16">
+        <f>TEXT(DATE($F$3,4,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M30" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=4)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N30" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=4)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Субподряд</t>
+        </is>
+      </c>
+      <c r="I31" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Субподряд")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J31" s="20">
+        <f>IFERROR(I31/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L31" s="16">
+        <f>TEXT(DATE($F$3,5,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M31" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=5)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N31" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=5)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Ипотека</t>
+        </is>
+      </c>
+      <c r="I32" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Ипотека")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J32" s="20">
+        <f>IFERROR(I32/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L32" s="16">
+        <f>TEXT(DATE($F$3,6,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M32" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=6)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N32" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=6)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Подарок</t>
+        </is>
+      </c>
+      <c r="I33" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Подарок")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J33" s="20">
+        <f>IFERROR(I33/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L33" s="16">
+        <f>TEXT(DATE($F$3,7,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M33" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=7)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N33" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=7)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>Аутсорс</t>
+        </is>
+      </c>
+      <c r="I34" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*($E$43:$E$242="Аутсорс")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="J34" s="20">
+        <f>IFERROR(I34/$D$6,0)</f>
+        <v/>
+      </c>
+      <c r="L34" s="16">
+        <f>TEXT(DATE($F$3,8,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M34" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=8)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N34" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=8)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="L35" s="16">
+        <f>TEXT(DATE($F$3,9,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M35" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=9)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N35" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=9)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="L36" s="16">
+        <f>TEXT(DATE($F$3,10,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M36" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=10)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N36" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=10)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="L37" s="16">
+        <f>TEXT(DATE($F$3,11,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M37" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=11)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N37" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=11)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="L38" s="16">
+        <f>TEXT(DATE($F$3,12,1),"mmm yy")</f>
+        <v/>
+      </c>
+      <c r="M38" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Доход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=12)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+      <c r="N38" s="16">
+        <f>SUMPRODUCT(($D$43:$D$242="Расход")*(YEAR($B$43:$B$242+0)=$F$3)*(MONTH($B$43:$B$242+0)=12)*(COUNTIF(Справочник!$C$3:$C$10,$E$43:$E$242)=0)*$F$43:$F$242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>✏️  ЖУРНАЛ ОПЕРАЦИЙ — вносите доходы и расходы сюда</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="18" t="inlineStr">
         <is>
           <t>Дата</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C42" s="18" t="inlineStr">
         <is>
           <t>Счёт</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D42" s="18" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E42" s="18" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F42" s="18" t="inlineStr">
         <is>
           <t>Сумма</t>
         </is>
       </c>
-      <c r="G26" s="18" t="inlineStr">
+      <c r="G42" s="18" t="inlineStr">
         <is>
           <t>Описание</t>
         </is>
       </c>
-      <c r="H26" s="18" t="inlineStr">
+      <c r="H42" s="18" t="inlineStr">
         <is>
           <t>Остаток</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="19" t="n">
+    <row r="43">
+      <c r="B43" s="21" t="n">
         <v>46027</v>
       </c>
-      <c r="C27" s="16" t="inlineStr">
+      <c r="C43" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E43" s="16" t="inlineStr">
         <is>
           <t>Зарплата</t>
         </is>
       </c>
-      <c r="F27" s="20" t="n">
+      <c r="F43" s="22" t="n">
         <v>75000</v>
       </c>
-      <c r="G27" s="16" t="inlineStr"/>
-      <c r="H27" s="21">
-        <f>IF(C27="","",SUMPRODUCT(($C$27:C27=C27)*(2*($D$27:D27="Доход")-1)*$F$27:F27))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="19" t="n">
+      <c r="G43" s="16" t="inlineStr"/>
+      <c r="H43" s="23">
+        <f>IF(C43="","",SUMPRODUCT(($C$43:C43=C43)*(2*($D$43:D43="Доход")-1)*$F$43:F43))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="21" t="n">
         <v>46028</v>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C44" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E44" s="16" t="inlineStr">
         <is>
           <t>Аренда</t>
         </is>
       </c>
-      <c r="F28" s="20" t="n">
+      <c r="F44" s="22" t="n">
         <v>28000</v>
       </c>
-      <c r="G28" s="16" t="inlineStr"/>
-      <c r="H28" s="21">
-        <f>IF(C28="","",SUMPRODUCT(($C$27:C28=C28)*(2*($D$27:D28="Доход")-1)*$F$27:F28))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="19" t="n">
+      <c r="G44" s="16" t="inlineStr"/>
+      <c r="H44" s="23">
+        <f>IF(C44="","",SUMPRODUCT(($C$43:C44=C44)*(2*($D$43:D44="Доход")-1)*$F$43:F44))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="21" t="n">
         <v>46030</v>
       </c>
-      <c r="C29" s="16" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
         <is>
           <t>Наличные</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E45" s="16" t="inlineStr">
         <is>
           <t>Продукты</t>
         </is>
       </c>
-      <c r="F29" s="20" t="n">
+      <c r="F45" s="22" t="n">
         <v>7500</v>
       </c>
-      <c r="G29" s="16" t="inlineStr"/>
-      <c r="H29" s="21">
-        <f>IF(C29="","",SUMPRODUCT(($C$27:C29=C29)*(2*($D$27:D29="Доход")-1)*$F$27:F29))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="19" t="n">
+      <c r="G45" s="16" t="inlineStr"/>
+      <c r="H45" s="23">
+        <f>IF(C45="","",SUMPRODUCT(($C$43:C45=C45)*(2*($D$43:D45="Доход")-1)*$F$43:F45))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="21" t="n">
         <v>46032</v>
       </c>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C46" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E30" s="16" t="inlineStr">
+      <c r="E46" s="16" t="inlineStr">
         <is>
           <t>Пополнение вклада</t>
         </is>
       </c>
-      <c r="F30" s="20" t="n">
+      <c r="F46" s="22" t="n">
         <v>15000</v>
       </c>
-      <c r="G30" s="16" t="inlineStr">
+      <c r="G46" s="16" t="inlineStr">
         <is>
           <t>перевод на вклад</t>
         </is>
       </c>
-      <c r="H30" s="21">
-        <f>IF(C30="","",SUMPRODUCT(($C$27:C30=C30)*(2*($D$27:D30="Доход")-1)*$F$27:F30))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="19" t="n">
+      <c r="H46" s="23">
+        <f>IF(C46="","",SUMPRODUCT(($C$43:C46=C46)*(2*($D$43:D46="Доход")-1)*$F$43:F46))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="21" t="n">
         <v>46032</v>
       </c>
-      <c r="C31" s="16" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>Вклад</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
+      <c r="E47" s="16" t="inlineStr">
         <is>
           <t>Пополнение вклада</t>
         </is>
       </c>
-      <c r="F31" s="20" t="n">
+      <c r="F47" s="22" t="n">
         <v>15000</v>
       </c>
-      <c r="G31" s="16" t="inlineStr"/>
-      <c r="H31" s="21">
-        <f>IF(C31="","",SUMPRODUCT(($C$27:C31=C31)*(2*($D$27:D31="Доход")-1)*$F$27:F31))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="19" t="n">
+      <c r="G47" s="16" t="inlineStr"/>
+      <c r="H47" s="23">
+        <f>IF(C47="","",SUMPRODUCT(($C$43:C47=C47)*(2*($D$43:D47="Доход")-1)*$F$43:F47))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="21" t="n">
         <v>46037</v>
       </c>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
         <is>
           <t>Карта Тинькофф</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E32" s="16" t="inlineStr">
+      <c r="E48" s="16" t="inlineStr">
         <is>
           <t>Заказы</t>
         </is>
       </c>
-      <c r="F32" s="20" t="n">
+      <c r="F48" s="22" t="n">
         <v>20000</v>
       </c>
-      <c r="G32" s="16" t="inlineStr">
+      <c r="G48" s="16" t="inlineStr">
         <is>
           <t>у друга</t>
         </is>
       </c>
-      <c r="H32" s="21">
-        <f>IF(C32="","",SUMPRODUCT(($C$27:C32=C32)*(2*($D$27:D32="Доход")-1)*$F$27:F32))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="19" t="n">
+      <c r="H48" s="23">
+        <f>IF(C48="","",SUMPRODUCT(($C$43:C48=C48)*(2*($D$43:D48="Доход")-1)*$F$43:F48))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="21" t="n">
         <v>46040</v>
       </c>
-      <c r="C33" s="16" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
+      <c r="E49" s="16" t="inlineStr">
         <is>
           <t>Кредит</t>
         </is>
       </c>
-      <c r="F33" s="20" t="n">
+      <c r="F49" s="22" t="n">
         <v>9000</v>
       </c>
-      <c r="G33" s="16" t="inlineStr"/>
-      <c r="H33" s="21">
-        <f>IF(C33="","",SUMPRODUCT(($C$27:C33=C33)*(2*($D$27:D33="Доход")-1)*$F$27:F33))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="19" t="n">
+      <c r="G49" s="16" t="inlineStr"/>
+      <c r="H49" s="23">
+        <f>IF(C49="","",SUMPRODUCT(($C$43:C49=C49)*(2*($D$43:D49="Доход")-1)*$F$43:F49))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="21" t="n">
         <v>46042</v>
       </c>
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C50" s="16" t="inlineStr">
         <is>
           <t>Наличные</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E34" s="16" t="inlineStr">
+      <c r="E50" s="16" t="inlineStr">
         <is>
           <t>Взял в долг</t>
         </is>
       </c>
-      <c r="F34" s="20" t="n">
+      <c r="F50" s="22" t="n">
         <v>10000</v>
       </c>
-      <c r="G34" s="16" t="inlineStr"/>
-      <c r="H34" s="21">
-        <f>IF(C34="","",SUMPRODUCT(($C$27:C34=C34)*(2*($D$27:D34="Доход")-1)*$F$27:F34))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="19" t="n">
+      <c r="G50" s="16" t="inlineStr"/>
+      <c r="H50" s="23">
+        <f>IF(C50="","",SUMPRODUCT(($C$43:C50=C50)*(2*($D$43:D50="Доход")-1)*$F$43:F50))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="21" t="n">
         <v>46047</v>
       </c>
-      <c r="C35" s="16" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
+      <c r="E51" s="16" t="inlineStr">
         <is>
           <t>Обучение</t>
         </is>
       </c>
-      <c r="F35" s="20" t="n">
+      <c r="F51" s="22" t="n">
         <v>10000</v>
       </c>
-      <c r="G35" s="16" t="inlineStr"/>
-      <c r="H35" s="21">
-        <f>IF(C35="","",SUMPRODUCT(($C$27:C35=C35)*(2*($D$27:D35="Доход")-1)*$F$27:F35))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="19" t="n">
+      <c r="G51" s="16" t="inlineStr"/>
+      <c r="H51" s="23">
+        <f>IF(C51="","",SUMPRODUCT(($C$43:C51=C51)*(2*($D$43:D51="Доход")-1)*$F$43:F51))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="21" t="n">
         <v>46055</v>
       </c>
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C52" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E36" s="16" t="inlineStr">
+      <c r="E52" s="16" t="inlineStr">
         <is>
           <t>Зарплата</t>
         </is>
       </c>
-      <c r="F36" s="20" t="n">
+      <c r="F52" s="22" t="n">
         <v>75000</v>
       </c>
-      <c r="G36" s="16" t="inlineStr"/>
-      <c r="H36" s="21">
-        <f>IF(C36="","",SUMPRODUCT(($C$27:C36=C36)*(2*($D$27:D36="Доход")-1)*$F$27:F36))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="19" t="n">
+      <c r="G52" s="16" t="inlineStr"/>
+      <c r="H52" s="23">
+        <f>IF(C52="","",SUMPRODUCT(($C$43:C52=C52)*(2*($D$43:D52="Доход")-1)*$F$43:F52))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="21" t="n">
         <v>46056</v>
       </c>
-      <c r="C37" s="16" t="inlineStr">
+      <c r="C53" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E37" s="16" t="inlineStr">
+      <c r="E53" s="16" t="inlineStr">
         <is>
           <t>Аренда</t>
         </is>
       </c>
-      <c r="F37" s="20" t="n">
+      <c r="F53" s="22" t="n">
         <v>28000</v>
       </c>
-      <c r="G37" s="16" t="inlineStr"/>
-      <c r="H37" s="21">
-        <f>IF(C37="","",SUMPRODUCT(($C$27:C37=C37)*(2*($D$27:D37="Доход")-1)*$F$27:F37))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="19" t="n">
+      <c r="G53" s="16" t="inlineStr"/>
+      <c r="H53" s="23">
+        <f>IF(C53="","",SUMPRODUCT(($C$43:C53=C53)*(2*($D$43:D53="Доход")-1)*$F$43:F53))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="21" t="n">
         <v>46058</v>
       </c>
-      <c r="C38" s="16" t="inlineStr">
+      <c r="C54" s="16" t="inlineStr">
         <is>
           <t>Наличные</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E38" s="16" t="inlineStr">
+      <c r="E54" s="16" t="inlineStr">
         <is>
           <t>Продукты</t>
         </is>
       </c>
-      <c r="F38" s="20" t="n">
+      <c r="F54" s="22" t="n">
         <v>8000</v>
       </c>
-      <c r="G38" s="16" t="inlineStr"/>
-      <c r="H38" s="21">
-        <f>IF(C38="","",SUMPRODUCT(($C$27:C38=C38)*(2*($D$27:D38="Доход")-1)*$F$27:F38))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="19" t="n">
+      <c r="G54" s="16" t="inlineStr"/>
+      <c r="H54" s="23">
+        <f>IF(C54="","",SUMPRODUCT(($C$43:C54=C54)*(2*($D$43:D54="Доход")-1)*$F$43:F54))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="21" t="n">
         <v>46061</v>
       </c>
-      <c r="C39" s="16" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E39" s="16" t="inlineStr">
+      <c r="E55" s="16" t="inlineStr">
         <is>
           <t>Пополнение вклада</t>
         </is>
       </c>
-      <c r="F39" s="20" t="n">
+      <c r="F55" s="22" t="n">
         <v>20000</v>
       </c>
-      <c r="G39" s="16" t="inlineStr"/>
-      <c r="H39" s="21">
-        <f>IF(C39="","",SUMPRODUCT(($C$27:C39=C39)*(2*($D$27:D39="Доход")-1)*$F$27:F39))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="19" t="n">
+      <c r="G55" s="16" t="inlineStr"/>
+      <c r="H55" s="23">
+        <f>IF(C55="","",SUMPRODUCT(($C$43:C55=C55)*(2*($D$43:D55="Доход")-1)*$F$43:F55))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="21" t="n">
         <v>46061</v>
       </c>
-      <c r="C40" s="16" t="inlineStr">
+      <c r="C56" s="16" t="inlineStr">
         <is>
           <t>Вклад</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E40" s="16" t="inlineStr">
+      <c r="E56" s="16" t="inlineStr">
         <is>
           <t>Пополнение вклада</t>
         </is>
       </c>
-      <c r="F40" s="20" t="n">
+      <c r="F56" s="22" t="n">
         <v>20000</v>
       </c>
-      <c r="G40" s="16" t="inlineStr"/>
-      <c r="H40" s="21">
-        <f>IF(C40="","",SUMPRODUCT(($C$27:C40=C40)*(2*($D$27:D40="Доход")-1)*$F$27:F40))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="19" t="n">
+      <c r="G56" s="16" t="inlineStr"/>
+      <c r="H56" s="23">
+        <f>IF(C56="","",SUMPRODUCT(($C$43:C56=C56)*(2*($D$43:D56="Доход")-1)*$F$43:F56))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="21" t="n">
         <v>46065</v>
       </c>
-      <c r="C41" s="16" t="inlineStr">
+      <c r="C57" s="16" t="inlineStr">
         <is>
           <t>Карта Тинькофф</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>Доход</t>
         </is>
       </c>
-      <c r="E41" s="16" t="inlineStr">
+      <c r="E57" s="16" t="inlineStr">
         <is>
           <t>Заказы</t>
         </is>
       </c>
-      <c r="F41" s="20" t="n">
+      <c r="F57" s="22" t="n">
         <v>30000</v>
       </c>
-      <c r="G41" s="16" t="inlineStr"/>
-      <c r="H41" s="21">
-        <f>IF(C41="","",SUMPRODUCT(($C$27:C41=C41)*(2*($D$27:D41="Доход")-1)*$F$27:F41))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="19" t="n">
+      <c r="G57" s="16" t="inlineStr"/>
+      <c r="H57" s="23">
+        <f>IF(C57="","",SUMPRODUCT(($C$43:C57=C57)*(2*($D$43:D57="Доход")-1)*$F$43:F57))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="21" t="n">
         <v>46068</v>
       </c>
-      <c r="C42" s="16" t="inlineStr">
+      <c r="C58" s="16" t="inlineStr">
         <is>
           <t>Наличные</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E42" s="16" t="inlineStr">
+      <c r="E58" s="16" t="inlineStr">
         <is>
           <t>Вернул долг</t>
         </is>
       </c>
-      <c r="F42" s="20" t="n">
+      <c r="F58" s="22" t="n">
         <v>5000</v>
       </c>
-      <c r="G42" s="16" t="inlineStr"/>
-      <c r="H42" s="21">
-        <f>IF(C42="","",SUMPRODUCT(($C$27:C42=C42)*(2*($D$27:D42="Доход")-1)*$F$27:F42))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="19" t="n">
+      <c r="G58" s="16" t="inlineStr"/>
+      <c r="H58" s="23">
+        <f>IF(C58="","",SUMPRODUCT(($C$43:C58=C58)*(2*($D$43:D58="Доход")-1)*$F$43:F58))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="21" t="n">
         <v>46071</v>
       </c>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="C59" s="16" t="inlineStr">
         <is>
           <t>Карта Сбербанк</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="E43" s="16" t="inlineStr">
+      <c r="E59" s="16" t="inlineStr">
         <is>
           <t>Ипотека</t>
         </is>
       </c>
-      <c r="F43" s="20" t="n">
+      <c r="F59" s="22" t="n">
         <v>18000</v>
       </c>
-      <c r="G43" s="16" t="inlineStr"/>
-      <c r="H43" s="21">
-        <f>IF(C43="","",SUMPRODUCT(($C$27:C43=C43)*(2*($D$27:D43="Доход")-1)*$F$27:F43))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="16" t="n"/>
-      <c r="C44" s="16" t="n"/>
-      <c r="D44" s="16" t="n"/>
-      <c r="E44" s="16" t="n"/>
-      <c r="F44" s="20" t="n"/>
-      <c r="G44" s="16" t="n"/>
-      <c r="H44" s="21">
-        <f>IF(C44="","",SUMPRODUCT(($C$27:C44=C44)*(2*($D$27:D44="Доход")-1)*$F$27:F44))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="16" t="n"/>
-      <c r="C45" s="16" t="n"/>
-      <c r="D45" s="16" t="n"/>
-      <c r="E45" s="16" t="n"/>
-      <c r="F45" s="20" t="n"/>
-      <c r="G45" s="16" t="n"/>
-      <c r="H45" s="21">
-        <f>IF(C45="","",SUMPRODUCT(($C$27:C45=C45)*(2*($D$27:D45="Доход")-1)*$F$27:F45))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="16" t="n"/>
-      <c r="C46" s="16" t="n"/>
-      <c r="D46" s="16" t="n"/>
-      <c r="E46" s="16" t="n"/>
-      <c r="F46" s="20" t="n"/>
-      <c r="G46" s="16" t="n"/>
-      <c r="H46" s="21">
-        <f>IF(C46="","",SUMPRODUCT(($C$27:C46=C46)*(2*($D$27:D46="Доход")-1)*$F$27:F46))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="16" t="n"/>
-      <c r="C47" s="16" t="n"/>
-      <c r="D47" s="16" t="n"/>
-      <c r="E47" s="16" t="n"/>
-      <c r="F47" s="20" t="n"/>
-      <c r="G47" s="16" t="n"/>
-      <c r="H47" s="21">
-        <f>IF(C47="","",SUMPRODUCT(($C$27:C47=C47)*(2*($D$27:D47="Доход")-1)*$F$27:F47))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="16" t="n"/>
-      <c r="C48" s="16" t="n"/>
-      <c r="D48" s="16" t="n"/>
-      <c r="E48" s="16" t="n"/>
-      <c r="F48" s="20" t="n"/>
-      <c r="G48" s="16" t="n"/>
-      <c r="H48" s="21">
-        <f>IF(C48="","",SUMPRODUCT(($C$27:C48=C48)*(2*($D$27:D48="Доход")-1)*$F$27:F48))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="16" t="n"/>
-      <c r="C49" s="16" t="n"/>
-      <c r="D49" s="16" t="n"/>
-      <c r="E49" s="16" t="n"/>
-      <c r="F49" s="20" t="n"/>
-      <c r="G49" s="16" t="n"/>
-      <c r="H49" s="21">
-        <f>IF(C49="","",SUMPRODUCT(($C$27:C49=C49)*(2*($D$27:D49="Доход")-1)*$F$27:F49))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="16" t="n"/>
-      <c r="C50" s="16" t="n"/>
-      <c r="D50" s="16" t="n"/>
-      <c r="E50" s="16" t="n"/>
-      <c r="F50" s="20" t="n"/>
-      <c r="G50" s="16" t="n"/>
-      <c r="H50" s="21">
-        <f>IF(C50="","",SUMPRODUCT(($C$27:C50=C50)*(2*($D$27:D50="Доход")-1)*$F$27:F50))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="16" t="n"/>
-      <c r="C51" s="16" t="n"/>
-      <c r="D51" s="16" t="n"/>
-      <c r="E51" s="16" t="n"/>
-      <c r="F51" s="20" t="n"/>
-      <c r="G51" s="16" t="n"/>
-      <c r="H51" s="21">
-        <f>IF(C51="","",SUMPRODUCT(($C$27:C51=C51)*(2*($D$27:D51="Доход")-1)*$F$27:F51))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="16" t="n"/>
-      <c r="C52" s="16" t="n"/>
-      <c r="D52" s="16" t="n"/>
-      <c r="E52" s="16" t="n"/>
-      <c r="F52" s="20" t="n"/>
-      <c r="G52" s="16" t="n"/>
-      <c r="H52" s="21">
-        <f>IF(C52="","",SUMPRODUCT(($C$27:C52=C52)*(2*($D$27:D52="Доход")-1)*$F$27:F52))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="16" t="n"/>
-      <c r="C53" s="16" t="n"/>
-      <c r="D53" s="16" t="n"/>
-      <c r="E53" s="16" t="n"/>
-      <c r="F53" s="20" t="n"/>
-      <c r="G53" s="16" t="n"/>
-      <c r="H53" s="21">
-        <f>IF(C53="","",SUMPRODUCT(($C$27:C53=C53)*(2*($D$27:D53="Доход")-1)*$F$27:F53))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="16" t="n"/>
-      <c r="C54" s="16" t="n"/>
-      <c r="D54" s="16" t="n"/>
-      <c r="E54" s="16" t="n"/>
-      <c r="F54" s="20" t="n"/>
-      <c r="G54" s="16" t="n"/>
-      <c r="H54" s="21">
-        <f>IF(C54="","",SUMPRODUCT(($C$27:C54=C54)*(2*($D$27:D54="Доход")-1)*$F$27:F54))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="16" t="n"/>
-      <c r="C55" s="16" t="n"/>
-      <c r="D55" s="16" t="n"/>
-      <c r="E55" s="16" t="n"/>
-      <c r="F55" s="20" t="n"/>
-      <c r="G55" s="16" t="n"/>
-      <c r="H55" s="21">
-        <f>IF(C55="","",SUMPRODUCT(($C$27:C55=C55)*(2*($D$27:D55="Доход")-1)*$F$27:F55))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="16" t="n"/>
-      <c r="C56" s="16" t="n"/>
-      <c r="D56" s="16" t="n"/>
-      <c r="E56" s="16" t="n"/>
-      <c r="F56" s="20" t="n"/>
-      <c r="G56" s="16" t="n"/>
-      <c r="H56" s="21">
-        <f>IF(C56="","",SUMPRODUCT(($C$27:C56=C56)*(2*($D$27:D56="Доход")-1)*$F$27:F56))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="16" t="n"/>
-      <c r="C57" s="16" t="n"/>
-      <c r="D57" s="16" t="n"/>
-      <c r="E57" s="16" t="n"/>
-      <c r="F57" s="20" t="n"/>
-      <c r="G57" s="16" t="n"/>
-      <c r="H57" s="21">
-        <f>IF(C57="","",SUMPRODUCT(($C$27:C57=C57)*(2*($D$27:D57="Доход")-1)*$F$27:F57))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="16" t="n"/>
-      <c r="C58" s="16" t="n"/>
-      <c r="D58" s="16" t="n"/>
-      <c r="E58" s="16" t="n"/>
-      <c r="F58" s="20" t="n"/>
-      <c r="G58" s="16" t="n"/>
-      <c r="H58" s="21">
-        <f>IF(C58="","",SUMPRODUCT(($C$27:C58=C58)*(2*($D$27:D58="Доход")-1)*$F$27:F58))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="16" t="n"/>
-      <c r="C59" s="16" t="n"/>
-      <c r="D59" s="16" t="n"/>
-      <c r="E59" s="16" t="n"/>
-      <c r="F59" s="20" t="n"/>
-      <c r="G59" s="16" t="n"/>
-      <c r="H59" s="21">
-        <f>IF(C59="","",SUMPRODUCT(($C$27:C59=C59)*(2*($D$27:D59="Доход")-1)*$F$27:F59))</f>
+      <c r="G59" s="16" t="inlineStr"/>
+      <c r="H59" s="23">
+        <f>IF(C59="","",SUMPRODUCT(($C$43:C59=C59)*(2*($D$43:D59="Доход")-1)*$F$43:F59))</f>
         <v/>
       </c>
     </row>
@@ -2211,10 +2400,10 @@
       <c r="C60" s="16" t="n"/>
       <c r="D60" s="16" t="n"/>
       <c r="E60" s="16" t="n"/>
-      <c r="F60" s="20" t="n"/>
+      <c r="F60" s="22" t="n"/>
       <c r="G60" s="16" t="n"/>
-      <c r="H60" s="21">
-        <f>IF(C60="","",SUMPRODUCT(($C$27:C60=C60)*(2*($D$27:D60="Доход")-1)*$F$27:F60))</f>
+      <c r="H60" s="23">
+        <f>IF(C60="","",SUMPRODUCT(($C$43:C60=C60)*(2*($D$43:D60="Доход")-1)*$F$43:F60))</f>
         <v/>
       </c>
     </row>
@@ -2223,10 +2412,10 @@
       <c r="C61" s="16" t="n"/>
       <c r="D61" s="16" t="n"/>
       <c r="E61" s="16" t="n"/>
-      <c r="F61" s="20" t="n"/>
+      <c r="F61" s="22" t="n"/>
       <c r="G61" s="16" t="n"/>
-      <c r="H61" s="21">
-        <f>IF(C61="","",SUMPRODUCT(($C$27:C61=C61)*(2*($D$27:D61="Доход")-1)*$F$27:F61))</f>
+      <c r="H61" s="23">
+        <f>IF(C61="","",SUMPRODUCT(($C$43:C61=C61)*(2*($D$43:D61="Доход")-1)*$F$43:F61))</f>
         <v/>
       </c>
     </row>
@@ -2235,10 +2424,10 @@
       <c r="C62" s="16" t="n"/>
       <c r="D62" s="16" t="n"/>
       <c r="E62" s="16" t="n"/>
-      <c r="F62" s="20" t="n"/>
+      <c r="F62" s="22" t="n"/>
       <c r="G62" s="16" t="n"/>
-      <c r="H62" s="21">
-        <f>IF(C62="","",SUMPRODUCT(($C$27:C62=C62)*(2*($D$27:D62="Доход")-1)*$F$27:F62))</f>
+      <c r="H62" s="23">
+        <f>IF(C62="","",SUMPRODUCT(($C$43:C62=C62)*(2*($D$43:D62="Доход")-1)*$F$43:F62))</f>
         <v/>
       </c>
     </row>
@@ -2247,10 +2436,10 @@
       <c r="C63" s="16" t="n"/>
       <c r="D63" s="16" t="n"/>
       <c r="E63" s="16" t="n"/>
-      <c r="F63" s="20" t="n"/>
+      <c r="F63" s="22" t="n"/>
       <c r="G63" s="16" t="n"/>
-      <c r="H63" s="21">
-        <f>IF(C63="","",SUMPRODUCT(($C$27:C63=C63)*(2*($D$27:D63="Доход")-1)*$F$27:F63))</f>
+      <c r="H63" s="23">
+        <f>IF(C63="","",SUMPRODUCT(($C$43:C63=C63)*(2*($D$43:D63="Доход")-1)*$F$43:F63))</f>
         <v/>
       </c>
     </row>
@@ -2259,10 +2448,10 @@
       <c r="C64" s="16" t="n"/>
       <c r="D64" s="16" t="n"/>
       <c r="E64" s="16" t="n"/>
-      <c r="F64" s="20" t="n"/>
+      <c r="F64" s="22" t="n"/>
       <c r="G64" s="16" t="n"/>
-      <c r="H64" s="21">
-        <f>IF(C64="","",SUMPRODUCT(($C$27:C64=C64)*(2*($D$27:D64="Доход")-1)*$F$27:F64))</f>
+      <c r="H64" s="23">
+        <f>IF(C64="","",SUMPRODUCT(($C$43:C64=C64)*(2*($D$43:D64="Доход")-1)*$F$43:F64))</f>
         <v/>
       </c>
     </row>
@@ -2271,10 +2460,10 @@
       <c r="C65" s="16" t="n"/>
       <c r="D65" s="16" t="n"/>
       <c r="E65" s="16" t="n"/>
-      <c r="F65" s="20" t="n"/>
+      <c r="F65" s="22" t="n"/>
       <c r="G65" s="16" t="n"/>
-      <c r="H65" s="21">
-        <f>IF(C65="","",SUMPRODUCT(($C$27:C65=C65)*(2*($D$27:D65="Доход")-1)*$F$27:F65))</f>
+      <c r="H65" s="23">
+        <f>IF(C65="","",SUMPRODUCT(($C$43:C65=C65)*(2*($D$43:D65="Доход")-1)*$F$43:F65))</f>
         <v/>
       </c>
     </row>
@@ -2283,10 +2472,10 @@
       <c r="C66" s="16" t="n"/>
       <c r="D66" s="16" t="n"/>
       <c r="E66" s="16" t="n"/>
-      <c r="F66" s="20" t="n"/>
+      <c r="F66" s="22" t="n"/>
       <c r="G66" s="16" t="n"/>
-      <c r="H66" s="21">
-        <f>IF(C66="","",SUMPRODUCT(($C$27:C66=C66)*(2*($D$27:D66="Доход")-1)*$F$27:F66))</f>
+      <c r="H66" s="23">
+        <f>IF(C66="","",SUMPRODUCT(($C$43:C66=C66)*(2*($D$43:D66="Доход")-1)*$F$43:F66))</f>
         <v/>
       </c>
     </row>
@@ -2295,10 +2484,10 @@
       <c r="C67" s="16" t="n"/>
       <c r="D67" s="16" t="n"/>
       <c r="E67" s="16" t="n"/>
-      <c r="F67" s="20" t="n"/>
+      <c r="F67" s="22" t="n"/>
       <c r="G67" s="16" t="n"/>
-      <c r="H67" s="21">
-        <f>IF(C67="","",SUMPRODUCT(($C$27:C67=C67)*(2*($D$27:D67="Доход")-1)*$F$27:F67))</f>
+      <c r="H67" s="23">
+        <f>IF(C67="","",SUMPRODUCT(($C$43:C67=C67)*(2*($D$43:D67="Доход")-1)*$F$43:F67))</f>
         <v/>
       </c>
     </row>
@@ -2307,10 +2496,10 @@
       <c r="C68" s="16" t="n"/>
       <c r="D68" s="16" t="n"/>
       <c r="E68" s="16" t="n"/>
-      <c r="F68" s="20" t="n"/>
+      <c r="F68" s="22" t="n"/>
       <c r="G68" s="16" t="n"/>
-      <c r="H68" s="21">
-        <f>IF(C68="","",SUMPRODUCT(($C$27:C68=C68)*(2*($D$27:D68="Доход")-1)*$F$27:F68))</f>
+      <c r="H68" s="23">
+        <f>IF(C68="","",SUMPRODUCT(($C$43:C68=C68)*(2*($D$43:D68="Доход")-1)*$F$43:F68))</f>
         <v/>
       </c>
     </row>
@@ -2319,10 +2508,10 @@
       <c r="C69" s="16" t="n"/>
       <c r="D69" s="16" t="n"/>
       <c r="E69" s="16" t="n"/>
-      <c r="F69" s="20" t="n"/>
+      <c r="F69" s="22" t="n"/>
       <c r="G69" s="16" t="n"/>
-      <c r="H69" s="21">
-        <f>IF(C69="","",SUMPRODUCT(($C$27:C69=C69)*(2*($D$27:D69="Доход")-1)*$F$27:F69))</f>
+      <c r="H69" s="23">
+        <f>IF(C69="","",SUMPRODUCT(($C$43:C69=C69)*(2*($D$43:D69="Доход")-1)*$F$43:F69))</f>
         <v/>
       </c>
     </row>
@@ -2331,10 +2520,10 @@
       <c r="C70" s="16" t="n"/>
       <c r="D70" s="16" t="n"/>
       <c r="E70" s="16" t="n"/>
-      <c r="F70" s="20" t="n"/>
+      <c r="F70" s="22" t="n"/>
       <c r="G70" s="16" t="n"/>
-      <c r="H70" s="21">
-        <f>IF(C70="","",SUMPRODUCT(($C$27:C70=C70)*(2*($D$27:D70="Доход")-1)*$F$27:F70))</f>
+      <c r="H70" s="23">
+        <f>IF(C70="","",SUMPRODUCT(($C$43:C70=C70)*(2*($D$43:D70="Доход")-1)*$F$43:F70))</f>
         <v/>
       </c>
     </row>
@@ -2343,10 +2532,10 @@
       <c r="C71" s="16" t="n"/>
       <c r="D71" s="16" t="n"/>
       <c r="E71" s="16" t="n"/>
-      <c r="F71" s="20" t="n"/>
+      <c r="F71" s="22" t="n"/>
       <c r="G71" s="16" t="n"/>
-      <c r="H71" s="21">
-        <f>IF(C71="","",SUMPRODUCT(($C$27:C71=C71)*(2*($D$27:D71="Доход")-1)*$F$27:F71))</f>
+      <c r="H71" s="23">
+        <f>IF(C71="","",SUMPRODUCT(($C$43:C71=C71)*(2*($D$43:D71="Доход")-1)*$F$43:F71))</f>
         <v/>
       </c>
     </row>
@@ -2355,10 +2544,10 @@
       <c r="C72" s="16" t="n"/>
       <c r="D72" s="16" t="n"/>
       <c r="E72" s="16" t="n"/>
-      <c r="F72" s="20" t="n"/>
+      <c r="F72" s="22" t="n"/>
       <c r="G72" s="16" t="n"/>
-      <c r="H72" s="21">
-        <f>IF(C72="","",SUMPRODUCT(($C$27:C72=C72)*(2*($D$27:D72="Доход")-1)*$F$27:F72))</f>
+      <c r="H72" s="23">
+        <f>IF(C72="","",SUMPRODUCT(($C$43:C72=C72)*(2*($D$43:D72="Доход")-1)*$F$43:F72))</f>
         <v/>
       </c>
     </row>
@@ -2367,10 +2556,10 @@
       <c r="C73" s="16" t="n"/>
       <c r="D73" s="16" t="n"/>
       <c r="E73" s="16" t="n"/>
-      <c r="F73" s="20" t="n"/>
+      <c r="F73" s="22" t="n"/>
       <c r="G73" s="16" t="n"/>
-      <c r="H73" s="21">
-        <f>IF(C73="","",SUMPRODUCT(($C$27:C73=C73)*(2*($D$27:D73="Доход")-1)*$F$27:F73))</f>
+      <c r="H73" s="23">
+        <f>IF(C73="","",SUMPRODUCT(($C$43:C73=C73)*(2*($D$43:D73="Доход")-1)*$F$43:F73))</f>
         <v/>
       </c>
     </row>
@@ -2379,10 +2568,10 @@
       <c r="C74" s="16" t="n"/>
       <c r="D74" s="16" t="n"/>
       <c r="E74" s="16" t="n"/>
-      <c r="F74" s="20" t="n"/>
+      <c r="F74" s="22" t="n"/>
       <c r="G74" s="16" t="n"/>
-      <c r="H74" s="21">
-        <f>IF(C74="","",SUMPRODUCT(($C$27:C74=C74)*(2*($D$27:D74="Доход")-1)*$F$27:F74))</f>
+      <c r="H74" s="23">
+        <f>IF(C74="","",SUMPRODUCT(($C$43:C74=C74)*(2*($D$43:D74="Доход")-1)*$F$43:F74))</f>
         <v/>
       </c>
     </row>
@@ -2391,10 +2580,10 @@
       <c r="C75" s="16" t="n"/>
       <c r="D75" s="16" t="n"/>
       <c r="E75" s="16" t="n"/>
-      <c r="F75" s="20" t="n"/>
+      <c r="F75" s="22" t="n"/>
       <c r="G75" s="16" t="n"/>
-      <c r="H75" s="21">
-        <f>IF(C75="","",SUMPRODUCT(($C$27:C75=C75)*(2*($D$27:D75="Доход")-1)*$F$27:F75))</f>
+      <c r="H75" s="23">
+        <f>IF(C75="","",SUMPRODUCT(($C$43:C75=C75)*(2*($D$43:D75="Доход")-1)*$F$43:F75))</f>
         <v/>
       </c>
     </row>
@@ -2403,10 +2592,10 @@
       <c r="C76" s="16" t="n"/>
       <c r="D76" s="16" t="n"/>
       <c r="E76" s="16" t="n"/>
-      <c r="F76" s="20" t="n"/>
+      <c r="F76" s="22" t="n"/>
       <c r="G76" s="16" t="n"/>
-      <c r="H76" s="21">
-        <f>IF(C76="","",SUMPRODUCT(($C$27:C76=C76)*(2*($D$27:D76="Доход")-1)*$F$27:F76))</f>
+      <c r="H76" s="23">
+        <f>IF(C76="","",SUMPRODUCT(($C$43:C76=C76)*(2*($D$43:D76="Доход")-1)*$F$43:F76))</f>
         <v/>
       </c>
     </row>
@@ -2415,10 +2604,10 @@
       <c r="C77" s="16" t="n"/>
       <c r="D77" s="16" t="n"/>
       <c r="E77" s="16" t="n"/>
-      <c r="F77" s="20" t="n"/>
+      <c r="F77" s="22" t="n"/>
       <c r="G77" s="16" t="n"/>
-      <c r="H77" s="21">
-        <f>IF(C77="","",SUMPRODUCT(($C$27:C77=C77)*(2*($D$27:D77="Доход")-1)*$F$27:F77))</f>
+      <c r="H77" s="23">
+        <f>IF(C77="","",SUMPRODUCT(($C$43:C77=C77)*(2*($D$43:D77="Доход")-1)*$F$43:F77))</f>
         <v/>
       </c>
     </row>
@@ -2427,10 +2616,10 @@
       <c r="C78" s="16" t="n"/>
       <c r="D78" s="16" t="n"/>
       <c r="E78" s="16" t="n"/>
-      <c r="F78" s="20" t="n"/>
+      <c r="F78" s="22" t="n"/>
       <c r="G78" s="16" t="n"/>
-      <c r="H78" s="21">
-        <f>IF(C78="","",SUMPRODUCT(($C$27:C78=C78)*(2*($D$27:D78="Доход")-1)*$F$27:F78))</f>
+      <c r="H78" s="23">
+        <f>IF(C78="","",SUMPRODUCT(($C$43:C78=C78)*(2*($D$43:D78="Доход")-1)*$F$43:F78))</f>
         <v/>
       </c>
     </row>
@@ -2439,10 +2628,10 @@
       <c r="C79" s="16" t="n"/>
       <c r="D79" s="16" t="n"/>
       <c r="E79" s="16" t="n"/>
-      <c r="F79" s="20" t="n"/>
+      <c r="F79" s="22" t="n"/>
       <c r="G79" s="16" t="n"/>
-      <c r="H79" s="21">
-        <f>IF(C79="","",SUMPRODUCT(($C$27:C79=C79)*(2*($D$27:D79="Доход")-1)*$F$27:F79))</f>
+      <c r="H79" s="23">
+        <f>IF(C79="","",SUMPRODUCT(($C$43:C79=C79)*(2*($D$43:D79="Доход")-1)*$F$43:F79))</f>
         <v/>
       </c>
     </row>
@@ -2451,10 +2640,10 @@
       <c r="C80" s="16" t="n"/>
       <c r="D80" s="16" t="n"/>
       <c r="E80" s="16" t="n"/>
-      <c r="F80" s="20" t="n"/>
+      <c r="F80" s="22" t="n"/>
       <c r="G80" s="16" t="n"/>
-      <c r="H80" s="21">
-        <f>IF(C80="","",SUMPRODUCT(($C$27:C80=C80)*(2*($D$27:D80="Доход")-1)*$F$27:F80))</f>
+      <c r="H80" s="23">
+        <f>IF(C80="","",SUMPRODUCT(($C$43:C80=C80)*(2*($D$43:D80="Доход")-1)*$F$43:F80))</f>
         <v/>
       </c>
     </row>
@@ -2463,10 +2652,10 @@
       <c r="C81" s="16" t="n"/>
       <c r="D81" s="16" t="n"/>
       <c r="E81" s="16" t="n"/>
-      <c r="F81" s="20" t="n"/>
+      <c r="F81" s="22" t="n"/>
       <c r="G81" s="16" t="n"/>
-      <c r="H81" s="21">
-        <f>IF(C81="","",SUMPRODUCT(($C$27:C81=C81)*(2*($D$27:D81="Доход")-1)*$F$27:F81))</f>
+      <c r="H81" s="23">
+        <f>IF(C81="","",SUMPRODUCT(($C$43:C81=C81)*(2*($D$43:D81="Доход")-1)*$F$43:F81))</f>
         <v/>
       </c>
     </row>
@@ -2475,10 +2664,10 @@
       <c r="C82" s="16" t="n"/>
       <c r="D82" s="16" t="n"/>
       <c r="E82" s="16" t="n"/>
-      <c r="F82" s="20" t="n"/>
+      <c r="F82" s="22" t="n"/>
       <c r="G82" s="16" t="n"/>
-      <c r="H82" s="21">
-        <f>IF(C82="","",SUMPRODUCT(($C$27:C82=C82)*(2*($D$27:D82="Доход")-1)*$F$27:F82))</f>
+      <c r="H82" s="23">
+        <f>IF(C82="","",SUMPRODUCT(($C$43:C82=C82)*(2*($D$43:D82="Доход")-1)*$F$43:F82))</f>
         <v/>
       </c>
     </row>
@@ -2487,10 +2676,10 @@
       <c r="C83" s="16" t="n"/>
       <c r="D83" s="16" t="n"/>
       <c r="E83" s="16" t="n"/>
-      <c r="F83" s="20" t="n"/>
+      <c r="F83" s="22" t="n"/>
       <c r="G83" s="16" t="n"/>
-      <c r="H83" s="21">
-        <f>IF(C83="","",SUMPRODUCT(($C$27:C83=C83)*(2*($D$27:D83="Доход")-1)*$F$27:F83))</f>
+      <c r="H83" s="23">
+        <f>IF(C83="","",SUMPRODUCT(($C$43:C83=C83)*(2*($D$43:D83="Доход")-1)*$F$43:F83))</f>
         <v/>
       </c>
     </row>
@@ -2499,10 +2688,10 @@
       <c r="C84" s="16" t="n"/>
       <c r="D84" s="16" t="n"/>
       <c r="E84" s="16" t="n"/>
-      <c r="F84" s="20" t="n"/>
+      <c r="F84" s="22" t="n"/>
       <c r="G84" s="16" t="n"/>
-      <c r="H84" s="21">
-        <f>IF(C84="","",SUMPRODUCT(($C$27:C84=C84)*(2*($D$27:D84="Доход")-1)*$F$27:F84))</f>
+      <c r="H84" s="23">
+        <f>IF(C84="","",SUMPRODUCT(($C$43:C84=C84)*(2*($D$43:D84="Доход")-1)*$F$43:F84))</f>
         <v/>
       </c>
     </row>
@@ -2511,10 +2700,10 @@
       <c r="C85" s="16" t="n"/>
       <c r="D85" s="16" t="n"/>
       <c r="E85" s="16" t="n"/>
-      <c r="F85" s="20" t="n"/>
+      <c r="F85" s="22" t="n"/>
       <c r="G85" s="16" t="n"/>
-      <c r="H85" s="21">
-        <f>IF(C85="","",SUMPRODUCT(($C$27:C85=C85)*(2*($D$27:D85="Доход")-1)*$F$27:F85))</f>
+      <c r="H85" s="23">
+        <f>IF(C85="","",SUMPRODUCT(($C$43:C85=C85)*(2*($D$43:D85="Доход")-1)*$F$43:F85))</f>
         <v/>
       </c>
     </row>
@@ -2523,10 +2712,10 @@
       <c r="C86" s="16" t="n"/>
       <c r="D86" s="16" t="n"/>
       <c r="E86" s="16" t="n"/>
-      <c r="F86" s="20" t="n"/>
+      <c r="F86" s="22" t="n"/>
       <c r="G86" s="16" t="n"/>
-      <c r="H86" s="21">
-        <f>IF(C86="","",SUMPRODUCT(($C$27:C86=C86)*(2*($D$27:D86="Доход")-1)*$F$27:F86))</f>
+      <c r="H86" s="23">
+        <f>IF(C86="","",SUMPRODUCT(($C$43:C86=C86)*(2*($D$43:D86="Доход")-1)*$F$43:F86))</f>
         <v/>
       </c>
     </row>
@@ -2535,10 +2724,10 @@
       <c r="C87" s="16" t="n"/>
       <c r="D87" s="16" t="n"/>
       <c r="E87" s="16" t="n"/>
-      <c r="F87" s="20" t="n"/>
+      <c r="F87" s="22" t="n"/>
       <c r="G87" s="16" t="n"/>
-      <c r="H87" s="21">
-        <f>IF(C87="","",SUMPRODUCT(($C$27:C87=C87)*(2*($D$27:D87="Доход")-1)*$F$27:F87))</f>
+      <c r="H87" s="23">
+        <f>IF(C87="","",SUMPRODUCT(($C$43:C87=C87)*(2*($D$43:D87="Доход")-1)*$F$43:F87))</f>
         <v/>
       </c>
     </row>
@@ -2547,10 +2736,10 @@
       <c r="C88" s="16" t="n"/>
       <c r="D88" s="16" t="n"/>
       <c r="E88" s="16" t="n"/>
-      <c r="F88" s="20" t="n"/>
+      <c r="F88" s="22" t="n"/>
       <c r="G88" s="16" t="n"/>
-      <c r="H88" s="21">
-        <f>IF(C88="","",SUMPRODUCT(($C$27:C88=C88)*(2*($D$27:D88="Доход")-1)*$F$27:F88))</f>
+      <c r="H88" s="23">
+        <f>IF(C88="","",SUMPRODUCT(($C$43:C88=C88)*(2*($D$43:D88="Доход")-1)*$F$43:F88))</f>
         <v/>
       </c>
     </row>
@@ -2559,10 +2748,10 @@
       <c r="C89" s="16" t="n"/>
       <c r="D89" s="16" t="n"/>
       <c r="E89" s="16" t="n"/>
-      <c r="F89" s="20" t="n"/>
+      <c r="F89" s="22" t="n"/>
       <c r="G89" s="16" t="n"/>
-      <c r="H89" s="21">
-        <f>IF(C89="","",SUMPRODUCT(($C$27:C89=C89)*(2*($D$27:D89="Доход")-1)*$F$27:F89))</f>
+      <c r="H89" s="23">
+        <f>IF(C89="","",SUMPRODUCT(($C$43:C89=C89)*(2*($D$43:D89="Доход")-1)*$F$43:F89))</f>
         <v/>
       </c>
     </row>
@@ -2571,10 +2760,10 @@
       <c r="C90" s="16" t="n"/>
       <c r="D90" s="16" t="n"/>
       <c r="E90" s="16" t="n"/>
-      <c r="F90" s="20" t="n"/>
+      <c r="F90" s="22" t="n"/>
       <c r="G90" s="16" t="n"/>
-      <c r="H90" s="21">
-        <f>IF(C90="","",SUMPRODUCT(($C$27:C90=C90)*(2*($D$27:D90="Доход")-1)*$F$27:F90))</f>
+      <c r="H90" s="23">
+        <f>IF(C90="","",SUMPRODUCT(($C$43:C90=C90)*(2*($D$43:D90="Доход")-1)*$F$43:F90))</f>
         <v/>
       </c>
     </row>
@@ -2583,10 +2772,10 @@
       <c r="C91" s="16" t="n"/>
       <c r="D91" s="16" t="n"/>
       <c r="E91" s="16" t="n"/>
-      <c r="F91" s="20" t="n"/>
+      <c r="F91" s="22" t="n"/>
       <c r="G91" s="16" t="n"/>
-      <c r="H91" s="21">
-        <f>IF(C91="","",SUMPRODUCT(($C$27:C91=C91)*(2*($D$27:D91="Доход")-1)*$F$27:F91))</f>
+      <c r="H91" s="23">
+        <f>IF(C91="","",SUMPRODUCT(($C$43:C91=C91)*(2*($D$43:D91="Доход")-1)*$F$43:F91))</f>
         <v/>
       </c>
     </row>
@@ -2595,10 +2784,10 @@
       <c r="C92" s="16" t="n"/>
       <c r="D92" s="16" t="n"/>
       <c r="E92" s="16" t="n"/>
-      <c r="F92" s="20" t="n"/>
+      <c r="F92" s="22" t="n"/>
       <c r="G92" s="16" t="n"/>
-      <c r="H92" s="21">
-        <f>IF(C92="","",SUMPRODUCT(($C$27:C92=C92)*(2*($D$27:D92="Доход")-1)*$F$27:F92))</f>
+      <c r="H92" s="23">
+        <f>IF(C92="","",SUMPRODUCT(($C$43:C92=C92)*(2*($D$43:D92="Доход")-1)*$F$43:F92))</f>
         <v/>
       </c>
     </row>
@@ -2607,10 +2796,10 @@
       <c r="C93" s="16" t="n"/>
       <c r="D93" s="16" t="n"/>
       <c r="E93" s="16" t="n"/>
-      <c r="F93" s="20" t="n"/>
+      <c r="F93" s="22" t="n"/>
       <c r="G93" s="16" t="n"/>
-      <c r="H93" s="21">
-        <f>IF(C93="","",SUMPRODUCT(($C$27:C93=C93)*(2*($D$27:D93="Доход")-1)*$F$27:F93))</f>
+      <c r="H93" s="23">
+        <f>IF(C93="","",SUMPRODUCT(($C$43:C93=C93)*(2*($D$43:D93="Доход")-1)*$F$43:F93))</f>
         <v/>
       </c>
     </row>
@@ -2619,10 +2808,10 @@
       <c r="C94" s="16" t="n"/>
       <c r="D94" s="16" t="n"/>
       <c r="E94" s="16" t="n"/>
-      <c r="F94" s="20" t="n"/>
+      <c r="F94" s="22" t="n"/>
       <c r="G94" s="16" t="n"/>
-      <c r="H94" s="21">
-        <f>IF(C94="","",SUMPRODUCT(($C$27:C94=C94)*(2*($D$27:D94="Доход")-1)*$F$27:F94))</f>
+      <c r="H94" s="23">
+        <f>IF(C94="","",SUMPRODUCT(($C$43:C94=C94)*(2*($D$43:D94="Доход")-1)*$F$43:F94))</f>
         <v/>
       </c>
     </row>
@@ -2631,10 +2820,10 @@
       <c r="C95" s="16" t="n"/>
       <c r="D95" s="16" t="n"/>
       <c r="E95" s="16" t="n"/>
-      <c r="F95" s="20" t="n"/>
+      <c r="F95" s="22" t="n"/>
       <c r="G95" s="16" t="n"/>
-      <c r="H95" s="21">
-        <f>IF(C95="","",SUMPRODUCT(($C$27:C95=C95)*(2*($D$27:D95="Доход")-1)*$F$27:F95))</f>
+      <c r="H95" s="23">
+        <f>IF(C95="","",SUMPRODUCT(($C$43:C95=C95)*(2*($D$43:D95="Доход")-1)*$F$43:F95))</f>
         <v/>
       </c>
     </row>
@@ -2643,10 +2832,10 @@
       <c r="C96" s="16" t="n"/>
       <c r="D96" s="16" t="n"/>
       <c r="E96" s="16" t="n"/>
-      <c r="F96" s="20" t="n"/>
+      <c r="F96" s="22" t="n"/>
       <c r="G96" s="16" t="n"/>
-      <c r="H96" s="21">
-        <f>IF(C96="","",SUMPRODUCT(($C$27:C96=C96)*(2*($D$27:D96="Доход")-1)*$F$27:F96))</f>
+      <c r="H96" s="23">
+        <f>IF(C96="","",SUMPRODUCT(($C$43:C96=C96)*(2*($D$43:D96="Доход")-1)*$F$43:F96))</f>
         <v/>
       </c>
     </row>
@@ -2655,10 +2844,10 @@
       <c r="C97" s="16" t="n"/>
       <c r="D97" s="16" t="n"/>
       <c r="E97" s="16" t="n"/>
-      <c r="F97" s="20" t="n"/>
+      <c r="F97" s="22" t="n"/>
       <c r="G97" s="16" t="n"/>
-      <c r="H97" s="21">
-        <f>IF(C97="","",SUMPRODUCT(($C$27:C97=C97)*(2*($D$27:D97="Доход")-1)*$F$27:F97))</f>
+      <c r="H97" s="23">
+        <f>IF(C97="","",SUMPRODUCT(($C$43:C97=C97)*(2*($D$43:D97="Доход")-1)*$F$43:F97))</f>
         <v/>
       </c>
     </row>
@@ -2667,10 +2856,10 @@
       <c r="C98" s="16" t="n"/>
       <c r="D98" s="16" t="n"/>
       <c r="E98" s="16" t="n"/>
-      <c r="F98" s="20" t="n"/>
+      <c r="F98" s="22" t="n"/>
       <c r="G98" s="16" t="n"/>
-      <c r="H98" s="21">
-        <f>IF(C98="","",SUMPRODUCT(($C$27:C98=C98)*(2*($D$27:D98="Доход")-1)*$F$27:F98))</f>
+      <c r="H98" s="23">
+        <f>IF(C98="","",SUMPRODUCT(($C$43:C98=C98)*(2*($D$43:D98="Доход")-1)*$F$43:F98))</f>
         <v/>
       </c>
     </row>
@@ -2679,10 +2868,10 @@
       <c r="C99" s="16" t="n"/>
       <c r="D99" s="16" t="n"/>
       <c r="E99" s="16" t="n"/>
-      <c r="F99" s="20" t="n"/>
+      <c r="F99" s="22" t="n"/>
       <c r="G99" s="16" t="n"/>
-      <c r="H99" s="21">
-        <f>IF(C99="","",SUMPRODUCT(($C$27:C99=C99)*(2*($D$27:D99="Доход")-1)*$F$27:F99))</f>
+      <c r="H99" s="23">
+        <f>IF(C99="","",SUMPRODUCT(($C$43:C99=C99)*(2*($D$43:D99="Доход")-1)*$F$43:F99))</f>
         <v/>
       </c>
     </row>
@@ -2691,10 +2880,10 @@
       <c r="C100" s="16" t="n"/>
       <c r="D100" s="16" t="n"/>
       <c r="E100" s="16" t="n"/>
-      <c r="F100" s="20" t="n"/>
+      <c r="F100" s="22" t="n"/>
       <c r="G100" s="16" t="n"/>
-      <c r="H100" s="21">
-        <f>IF(C100="","",SUMPRODUCT(($C$27:C100=C100)*(2*($D$27:D100="Доход")-1)*$F$27:F100))</f>
+      <c r="H100" s="23">
+        <f>IF(C100="","",SUMPRODUCT(($C$43:C100=C100)*(2*($D$43:D100="Доход")-1)*$F$43:F100))</f>
         <v/>
       </c>
     </row>
@@ -2703,10 +2892,10 @@
       <c r="C101" s="16" t="n"/>
       <c r="D101" s="16" t="n"/>
       <c r="E101" s="16" t="n"/>
-      <c r="F101" s="20" t="n"/>
+      <c r="F101" s="22" t="n"/>
       <c r="G101" s="16" t="n"/>
-      <c r="H101" s="21">
-        <f>IF(C101="","",SUMPRODUCT(($C$27:C101=C101)*(2*($D$27:D101="Доход")-1)*$F$27:F101))</f>
+      <c r="H101" s="23">
+        <f>IF(C101="","",SUMPRODUCT(($C$43:C101=C101)*(2*($D$43:D101="Доход")-1)*$F$43:F101))</f>
         <v/>
       </c>
     </row>
@@ -2715,10 +2904,10 @@
       <c r="C102" s="16" t="n"/>
       <c r="D102" s="16" t="n"/>
       <c r="E102" s="16" t="n"/>
-      <c r="F102" s="20" t="n"/>
+      <c r="F102" s="22" t="n"/>
       <c r="G102" s="16" t="n"/>
-      <c r="H102" s="21">
-        <f>IF(C102="","",SUMPRODUCT(($C$27:C102=C102)*(2*($D$27:D102="Доход")-1)*$F$27:F102))</f>
+      <c r="H102" s="23">
+        <f>IF(C102="","",SUMPRODUCT(($C$43:C102=C102)*(2*($D$43:D102="Доход")-1)*$F$43:F102))</f>
         <v/>
       </c>
     </row>
@@ -2727,10 +2916,10 @@
       <c r="C103" s="16" t="n"/>
       <c r="D103" s="16" t="n"/>
       <c r="E103" s="16" t="n"/>
-      <c r="F103" s="20" t="n"/>
+      <c r="F103" s="22" t="n"/>
       <c r="G103" s="16" t="n"/>
-      <c r="H103" s="21">
-        <f>IF(C103="","",SUMPRODUCT(($C$27:C103=C103)*(2*($D$27:D103="Доход")-1)*$F$27:F103))</f>
+      <c r="H103" s="23">
+        <f>IF(C103="","",SUMPRODUCT(($C$43:C103=C103)*(2*($D$43:D103="Доход")-1)*$F$43:F103))</f>
         <v/>
       </c>
     </row>
@@ -2739,10 +2928,10 @@
       <c r="C104" s="16" t="n"/>
       <c r="D104" s="16" t="n"/>
       <c r="E104" s="16" t="n"/>
-      <c r="F104" s="20" t="n"/>
+      <c r="F104" s="22" t="n"/>
       <c r="G104" s="16" t="n"/>
-      <c r="H104" s="21">
-        <f>IF(C104="","",SUMPRODUCT(($C$27:C104=C104)*(2*($D$27:D104="Доход")-1)*$F$27:F104))</f>
+      <c r="H104" s="23">
+        <f>IF(C104="","",SUMPRODUCT(($C$43:C104=C104)*(2*($D$43:D104="Доход")-1)*$F$43:F104))</f>
         <v/>
       </c>
     </row>
@@ -2751,10 +2940,10 @@
       <c r="C105" s="16" t="n"/>
       <c r="D105" s="16" t="n"/>
       <c r="E105" s="16" t="n"/>
-      <c r="F105" s="20" t="n"/>
+      <c r="F105" s="22" t="n"/>
       <c r="G105" s="16" t="n"/>
-      <c r="H105" s="21">
-        <f>IF(C105="","",SUMPRODUCT(($C$27:C105=C105)*(2*($D$27:D105="Доход")-1)*$F$27:F105))</f>
+      <c r="H105" s="23">
+        <f>IF(C105="","",SUMPRODUCT(($C$43:C105=C105)*(2*($D$43:D105="Доход")-1)*$F$43:F105))</f>
         <v/>
       </c>
     </row>
@@ -2763,10 +2952,10 @@
       <c r="C106" s="16" t="n"/>
       <c r="D106" s="16" t="n"/>
       <c r="E106" s="16" t="n"/>
-      <c r="F106" s="20" t="n"/>
+      <c r="F106" s="22" t="n"/>
       <c r="G106" s="16" t="n"/>
-      <c r="H106" s="21">
-        <f>IF(C106="","",SUMPRODUCT(($C$27:C106=C106)*(2*($D$27:D106="Доход")-1)*$F$27:F106))</f>
+      <c r="H106" s="23">
+        <f>IF(C106="","",SUMPRODUCT(($C$43:C106=C106)*(2*($D$43:D106="Доход")-1)*$F$43:F106))</f>
         <v/>
       </c>
     </row>
@@ -2775,10 +2964,10 @@
       <c r="C107" s="16" t="n"/>
       <c r="D107" s="16" t="n"/>
       <c r="E107" s="16" t="n"/>
-      <c r="F107" s="20" t="n"/>
+      <c r="F107" s="22" t="n"/>
       <c r="G107" s="16" t="n"/>
-      <c r="H107" s="21">
-        <f>IF(C107="","",SUMPRODUCT(($C$27:C107=C107)*(2*($D$27:D107="Доход")-1)*$F$27:F107))</f>
+      <c r="H107" s="23">
+        <f>IF(C107="","",SUMPRODUCT(($C$43:C107=C107)*(2*($D$43:D107="Доход")-1)*$F$43:F107))</f>
         <v/>
       </c>
     </row>
@@ -2787,10 +2976,10 @@
       <c r="C108" s="16" t="n"/>
       <c r="D108" s="16" t="n"/>
       <c r="E108" s="16" t="n"/>
-      <c r="F108" s="20" t="n"/>
+      <c r="F108" s="22" t="n"/>
       <c r="G108" s="16" t="n"/>
-      <c r="H108" s="21">
-        <f>IF(C108="","",SUMPRODUCT(($C$27:C108=C108)*(2*($D$27:D108="Доход")-1)*$F$27:F108))</f>
+      <c r="H108" s="23">
+        <f>IF(C108="","",SUMPRODUCT(($C$43:C108=C108)*(2*($D$43:D108="Доход")-1)*$F$43:F108))</f>
         <v/>
       </c>
     </row>
@@ -2799,10 +2988,10 @@
       <c r="C109" s="16" t="n"/>
       <c r="D109" s="16" t="n"/>
       <c r="E109" s="16" t="n"/>
-      <c r="F109" s="20" t="n"/>
+      <c r="F109" s="22" t="n"/>
       <c r="G109" s="16" t="n"/>
-      <c r="H109" s="21">
-        <f>IF(C109="","",SUMPRODUCT(($C$27:C109=C109)*(2*($D$27:D109="Доход")-1)*$F$27:F109))</f>
+      <c r="H109" s="23">
+        <f>IF(C109="","",SUMPRODUCT(($C$43:C109=C109)*(2*($D$43:D109="Доход")-1)*$F$43:F109))</f>
         <v/>
       </c>
     </row>
@@ -2811,10 +3000,10 @@
       <c r="C110" s="16" t="n"/>
       <c r="D110" s="16" t="n"/>
       <c r="E110" s="16" t="n"/>
-      <c r="F110" s="20" t="n"/>
+      <c r="F110" s="22" t="n"/>
       <c r="G110" s="16" t="n"/>
-      <c r="H110" s="21">
-        <f>IF(C110="","",SUMPRODUCT(($C$27:C110=C110)*(2*($D$27:D110="Доход")-1)*$F$27:F110))</f>
+      <c r="H110" s="23">
+        <f>IF(C110="","",SUMPRODUCT(($C$43:C110=C110)*(2*($D$43:D110="Доход")-1)*$F$43:F110))</f>
         <v/>
       </c>
     </row>
@@ -2823,10 +3012,10 @@
       <c r="C111" s="16" t="n"/>
       <c r="D111" s="16" t="n"/>
       <c r="E111" s="16" t="n"/>
-      <c r="F111" s="20" t="n"/>
+      <c r="F111" s="22" t="n"/>
       <c r="G111" s="16" t="n"/>
-      <c r="H111" s="21">
-        <f>IF(C111="","",SUMPRODUCT(($C$27:C111=C111)*(2*($D$27:D111="Доход")-1)*$F$27:F111))</f>
+      <c r="H111" s="23">
+        <f>IF(C111="","",SUMPRODUCT(($C$43:C111=C111)*(2*($D$43:D111="Доход")-1)*$F$43:F111))</f>
         <v/>
       </c>
     </row>
@@ -2835,10 +3024,10 @@
       <c r="C112" s="16" t="n"/>
       <c r="D112" s="16" t="n"/>
       <c r="E112" s="16" t="n"/>
-      <c r="F112" s="20" t="n"/>
+      <c r="F112" s="22" t="n"/>
       <c r="G112" s="16" t="n"/>
-      <c r="H112" s="21">
-        <f>IF(C112="","",SUMPRODUCT(($C$27:C112=C112)*(2*($D$27:D112="Доход")-1)*$F$27:F112))</f>
+      <c r="H112" s="23">
+        <f>IF(C112="","",SUMPRODUCT(($C$43:C112=C112)*(2*($D$43:D112="Доход")-1)*$F$43:F112))</f>
         <v/>
       </c>
     </row>
@@ -2847,10 +3036,10 @@
       <c r="C113" s="16" t="n"/>
       <c r="D113" s="16" t="n"/>
       <c r="E113" s="16" t="n"/>
-      <c r="F113" s="20" t="n"/>
+      <c r="F113" s="22" t="n"/>
       <c r="G113" s="16" t="n"/>
-      <c r="H113" s="21">
-        <f>IF(C113="","",SUMPRODUCT(($C$27:C113=C113)*(2*($D$27:D113="Доход")-1)*$F$27:F113))</f>
+      <c r="H113" s="23">
+        <f>IF(C113="","",SUMPRODUCT(($C$43:C113=C113)*(2*($D$43:D113="Доход")-1)*$F$43:F113))</f>
         <v/>
       </c>
     </row>
@@ -2859,10 +3048,10 @@
       <c r="C114" s="16" t="n"/>
       <c r="D114" s="16" t="n"/>
       <c r="E114" s="16" t="n"/>
-      <c r="F114" s="20" t="n"/>
+      <c r="F114" s="22" t="n"/>
       <c r="G114" s="16" t="n"/>
-      <c r="H114" s="21">
-        <f>IF(C114="","",SUMPRODUCT(($C$27:C114=C114)*(2*($D$27:D114="Доход")-1)*$F$27:F114))</f>
+      <c r="H114" s="23">
+        <f>IF(C114="","",SUMPRODUCT(($C$43:C114=C114)*(2*($D$43:D114="Доход")-1)*$F$43:F114))</f>
         <v/>
       </c>
     </row>
@@ -2871,10 +3060,10 @@
       <c r="C115" s="16" t="n"/>
       <c r="D115" s="16" t="n"/>
       <c r="E115" s="16" t="n"/>
-      <c r="F115" s="20" t="n"/>
+      <c r="F115" s="22" t="n"/>
       <c r="G115" s="16" t="n"/>
-      <c r="H115" s="21">
-        <f>IF(C115="","",SUMPRODUCT(($C$27:C115=C115)*(2*($D$27:D115="Доход")-1)*$F$27:F115))</f>
+      <c r="H115" s="23">
+        <f>IF(C115="","",SUMPRODUCT(($C$43:C115=C115)*(2*($D$43:D115="Доход")-1)*$F$43:F115))</f>
         <v/>
       </c>
     </row>
@@ -2883,10 +3072,10 @@
       <c r="C116" s="16" t="n"/>
       <c r="D116" s="16" t="n"/>
       <c r="E116" s="16" t="n"/>
-      <c r="F116" s="20" t="n"/>
+      <c r="F116" s="22" t="n"/>
       <c r="G116" s="16" t="n"/>
-      <c r="H116" s="21">
-        <f>IF(C116="","",SUMPRODUCT(($C$27:C116=C116)*(2*($D$27:D116="Доход")-1)*$F$27:F116))</f>
+      <c r="H116" s="23">
+        <f>IF(C116="","",SUMPRODUCT(($C$43:C116=C116)*(2*($D$43:D116="Доход")-1)*$F$43:F116))</f>
         <v/>
       </c>
     </row>
@@ -2895,10 +3084,10 @@
       <c r="C117" s="16" t="n"/>
       <c r="D117" s="16" t="n"/>
       <c r="E117" s="16" t="n"/>
-      <c r="F117" s="20" t="n"/>
+      <c r="F117" s="22" t="n"/>
       <c r="G117" s="16" t="n"/>
-      <c r="H117" s="21">
-        <f>IF(C117="","",SUMPRODUCT(($C$27:C117=C117)*(2*($D$27:D117="Доход")-1)*$F$27:F117))</f>
+      <c r="H117" s="23">
+        <f>IF(C117="","",SUMPRODUCT(($C$43:C117=C117)*(2*($D$43:D117="Доход")-1)*$F$43:F117))</f>
         <v/>
       </c>
     </row>
@@ -2907,10 +3096,10 @@
       <c r="C118" s="16" t="n"/>
       <c r="D118" s="16" t="n"/>
       <c r="E118" s="16" t="n"/>
-      <c r="F118" s="20" t="n"/>
+      <c r="F118" s="22" t="n"/>
       <c r="G118" s="16" t="n"/>
-      <c r="H118" s="21">
-        <f>IF(C118="","",SUMPRODUCT(($C$27:C118=C118)*(2*($D$27:D118="Доход")-1)*$F$27:F118))</f>
+      <c r="H118" s="23">
+        <f>IF(C118="","",SUMPRODUCT(($C$43:C118=C118)*(2*($D$43:D118="Доход")-1)*$F$43:F118))</f>
         <v/>
       </c>
     </row>
@@ -2919,10 +3108,10 @@
       <c r="C119" s="16" t="n"/>
       <c r="D119" s="16" t="n"/>
       <c r="E119" s="16" t="n"/>
-      <c r="F119" s="20" t="n"/>
+      <c r="F119" s="22" t="n"/>
       <c r="G119" s="16" t="n"/>
-      <c r="H119" s="21">
-        <f>IF(C119="","",SUMPRODUCT(($C$27:C119=C119)*(2*($D$27:D119="Доход")-1)*$F$27:F119))</f>
+      <c r="H119" s="23">
+        <f>IF(C119="","",SUMPRODUCT(($C$43:C119=C119)*(2*($D$43:D119="Доход")-1)*$F$43:F119))</f>
         <v/>
       </c>
     </row>
@@ -2931,10 +3120,10 @@
       <c r="C120" s="16" t="n"/>
       <c r="D120" s="16" t="n"/>
       <c r="E120" s="16" t="n"/>
-      <c r="F120" s="20" t="n"/>
+      <c r="F120" s="22" t="n"/>
       <c r="G120" s="16" t="n"/>
-      <c r="H120" s="21">
-        <f>IF(C120="","",SUMPRODUCT(($C$27:C120=C120)*(2*($D$27:D120="Доход")-1)*$F$27:F120))</f>
+      <c r="H120" s="23">
+        <f>IF(C120="","",SUMPRODUCT(($C$43:C120=C120)*(2*($D$43:D120="Доход")-1)*$F$43:F120))</f>
         <v/>
       </c>
     </row>
@@ -2943,10 +3132,10 @@
       <c r="C121" s="16" t="n"/>
       <c r="D121" s="16" t="n"/>
       <c r="E121" s="16" t="n"/>
-      <c r="F121" s="20" t="n"/>
+      <c r="F121" s="22" t="n"/>
       <c r="G121" s="16" t="n"/>
-      <c r="H121" s="21">
-        <f>IF(C121="","",SUMPRODUCT(($C$27:C121=C121)*(2*($D$27:D121="Доход")-1)*$F$27:F121))</f>
+      <c r="H121" s="23">
+        <f>IF(C121="","",SUMPRODUCT(($C$43:C121=C121)*(2*($D$43:D121="Доход")-1)*$F$43:F121))</f>
         <v/>
       </c>
     </row>
@@ -2955,10 +3144,10 @@
       <c r="C122" s="16" t="n"/>
       <c r="D122" s="16" t="n"/>
       <c r="E122" s="16" t="n"/>
-      <c r="F122" s="20" t="n"/>
+      <c r="F122" s="22" t="n"/>
       <c r="G122" s="16" t="n"/>
-      <c r="H122" s="21">
-        <f>IF(C122="","",SUMPRODUCT(($C$27:C122=C122)*(2*($D$27:D122="Доход")-1)*$F$27:F122))</f>
+      <c r="H122" s="23">
+        <f>IF(C122="","",SUMPRODUCT(($C$43:C122=C122)*(2*($D$43:D122="Доход")-1)*$F$43:F122))</f>
         <v/>
       </c>
     </row>
@@ -2967,10 +3156,10 @@
       <c r="C123" s="16" t="n"/>
       <c r="D123" s="16" t="n"/>
       <c r="E123" s="16" t="n"/>
-      <c r="F123" s="20" t="n"/>
+      <c r="F123" s="22" t="n"/>
       <c r="G123" s="16" t="n"/>
-      <c r="H123" s="21">
-        <f>IF(C123="","",SUMPRODUCT(($C$27:C123=C123)*(2*($D$27:D123="Доход")-1)*$F$27:F123))</f>
+      <c r="H123" s="23">
+        <f>IF(C123="","",SUMPRODUCT(($C$43:C123=C123)*(2*($D$43:D123="Доход")-1)*$F$43:F123))</f>
         <v/>
       </c>
     </row>
@@ -2979,10 +3168,10 @@
       <c r="C124" s="16" t="n"/>
       <c r="D124" s="16" t="n"/>
       <c r="E124" s="16" t="n"/>
-      <c r="F124" s="20" t="n"/>
+      <c r="F124" s="22" t="n"/>
       <c r="G124" s="16" t="n"/>
-      <c r="H124" s="21">
-        <f>IF(C124="","",SUMPRODUCT(($C$27:C124=C124)*(2*($D$27:D124="Доход")-1)*$F$27:F124))</f>
+      <c r="H124" s="23">
+        <f>IF(C124="","",SUMPRODUCT(($C$43:C124=C124)*(2*($D$43:D124="Доход")-1)*$F$43:F124))</f>
         <v/>
       </c>
     </row>
@@ -2991,10 +3180,10 @@
       <c r="C125" s="16" t="n"/>
       <c r="D125" s="16" t="n"/>
       <c r="E125" s="16" t="n"/>
-      <c r="F125" s="20" t="n"/>
+      <c r="F125" s="22" t="n"/>
       <c r="G125" s="16" t="n"/>
-      <c r="H125" s="21">
-        <f>IF(C125="","",SUMPRODUCT(($C$27:C125=C125)*(2*($D$27:D125="Доход")-1)*$F$27:F125))</f>
+      <c r="H125" s="23">
+        <f>IF(C125="","",SUMPRODUCT(($C$43:C125=C125)*(2*($D$43:D125="Доход")-1)*$F$43:F125))</f>
         <v/>
       </c>
     </row>
@@ -3003,10 +3192,10 @@
       <c r="C126" s="16" t="n"/>
       <c r="D126" s="16" t="n"/>
       <c r="E126" s="16" t="n"/>
-      <c r="F126" s="20" t="n"/>
+      <c r="F126" s="22" t="n"/>
       <c r="G126" s="16" t="n"/>
-      <c r="H126" s="21">
-        <f>IF(C126="","",SUMPRODUCT(($C$27:C126=C126)*(2*($D$27:D126="Доход")-1)*$F$27:F126))</f>
+      <c r="H126" s="23">
+        <f>IF(C126="","",SUMPRODUCT(($C$43:C126=C126)*(2*($D$43:D126="Доход")-1)*$F$43:F126))</f>
         <v/>
       </c>
     </row>
@@ -3015,10 +3204,10 @@
       <c r="C127" s="16" t="n"/>
       <c r="D127" s="16" t="n"/>
       <c r="E127" s="16" t="n"/>
-      <c r="F127" s="20" t="n"/>
+      <c r="F127" s="22" t="n"/>
       <c r="G127" s="16" t="n"/>
-      <c r="H127" s="21">
-        <f>IF(C127="","",SUMPRODUCT(($C$27:C127=C127)*(2*($D$27:D127="Доход")-1)*$F$27:F127))</f>
+      <c r="H127" s="23">
+        <f>IF(C127="","",SUMPRODUCT(($C$43:C127=C127)*(2*($D$43:D127="Доход")-1)*$F$43:F127))</f>
         <v/>
       </c>
     </row>
@@ -3027,10 +3216,10 @@
       <c r="C128" s="16" t="n"/>
       <c r="D128" s="16" t="n"/>
       <c r="E128" s="16" t="n"/>
-      <c r="F128" s="20" t="n"/>
+      <c r="F128" s="22" t="n"/>
       <c r="G128" s="16" t="n"/>
-      <c r="H128" s="21">
-        <f>IF(C128="","",SUMPRODUCT(($C$27:C128=C128)*(2*($D$27:D128="Доход")-1)*$F$27:F128))</f>
+      <c r="H128" s="23">
+        <f>IF(C128="","",SUMPRODUCT(($C$43:C128=C128)*(2*($D$43:D128="Доход")-1)*$F$43:F128))</f>
         <v/>
       </c>
     </row>
@@ -3039,10 +3228,10 @@
       <c r="C129" s="16" t="n"/>
       <c r="D129" s="16" t="n"/>
       <c r="E129" s="16" t="n"/>
-      <c r="F129" s="20" t="n"/>
+      <c r="F129" s="22" t="n"/>
       <c r="G129" s="16" t="n"/>
-      <c r="H129" s="21">
-        <f>IF(C129="","",SUMPRODUCT(($C$27:C129=C129)*(2*($D$27:D129="Доход")-1)*$F$27:F129))</f>
+      <c r="H129" s="23">
+        <f>IF(C129="","",SUMPRODUCT(($C$43:C129=C129)*(2*($D$43:D129="Доход")-1)*$F$43:F129))</f>
         <v/>
       </c>
     </row>
@@ -3051,10 +3240,10 @@
       <c r="C130" s="16" t="n"/>
       <c r="D130" s="16" t="n"/>
       <c r="E130" s="16" t="n"/>
-      <c r="F130" s="20" t="n"/>
+      <c r="F130" s="22" t="n"/>
       <c r="G130" s="16" t="n"/>
-      <c r="H130" s="21">
-        <f>IF(C130="","",SUMPRODUCT(($C$27:C130=C130)*(2*($D$27:D130="Доход")-1)*$F$27:F130))</f>
+      <c r="H130" s="23">
+        <f>IF(C130="","",SUMPRODUCT(($C$43:C130=C130)*(2*($D$43:D130="Доход")-1)*$F$43:F130))</f>
         <v/>
       </c>
     </row>
@@ -3063,10 +3252,10 @@
       <c r="C131" s="16" t="n"/>
       <c r="D131" s="16" t="n"/>
       <c r="E131" s="16" t="n"/>
-      <c r="F131" s="20" t="n"/>
+      <c r="F131" s="22" t="n"/>
       <c r="G131" s="16" t="n"/>
-      <c r="H131" s="21">
-        <f>IF(C131="","",SUMPRODUCT(($C$27:C131=C131)*(2*($D$27:D131="Доход")-1)*$F$27:F131))</f>
+      <c r="H131" s="23">
+        <f>IF(C131="","",SUMPRODUCT(($C$43:C131=C131)*(2*($D$43:D131="Доход")-1)*$F$43:F131))</f>
         <v/>
       </c>
     </row>
@@ -3075,10 +3264,10 @@
       <c r="C132" s="16" t="n"/>
       <c r="D132" s="16" t="n"/>
       <c r="E132" s="16" t="n"/>
-      <c r="F132" s="20" t="n"/>
+      <c r="F132" s="22" t="n"/>
       <c r="G132" s="16" t="n"/>
-      <c r="H132" s="21">
-        <f>IF(C132="","",SUMPRODUCT(($C$27:C132=C132)*(2*($D$27:D132="Доход")-1)*$F$27:F132))</f>
+      <c r="H132" s="23">
+        <f>IF(C132="","",SUMPRODUCT(($C$43:C132=C132)*(2*($D$43:D132="Доход")-1)*$F$43:F132))</f>
         <v/>
       </c>
     </row>
@@ -3087,10 +3276,10 @@
       <c r="C133" s="16" t="n"/>
       <c r="D133" s="16" t="n"/>
       <c r="E133" s="16" t="n"/>
-      <c r="F133" s="20" t="n"/>
+      <c r="F133" s="22" t="n"/>
       <c r="G133" s="16" t="n"/>
-      <c r="H133" s="21">
-        <f>IF(C133="","",SUMPRODUCT(($C$27:C133=C133)*(2*($D$27:D133="Доход")-1)*$F$27:F133))</f>
+      <c r="H133" s="23">
+        <f>IF(C133="","",SUMPRODUCT(($C$43:C133=C133)*(2*($D$43:D133="Доход")-1)*$F$43:F133))</f>
         <v/>
       </c>
     </row>
@@ -3099,10 +3288,10 @@
       <c r="C134" s="16" t="n"/>
       <c r="D134" s="16" t="n"/>
       <c r="E134" s="16" t="n"/>
-      <c r="F134" s="20" t="n"/>
+      <c r="F134" s="22" t="n"/>
       <c r="G134" s="16" t="n"/>
-      <c r="H134" s="21">
-        <f>IF(C134="","",SUMPRODUCT(($C$27:C134=C134)*(2*($D$27:D134="Доход")-1)*$F$27:F134))</f>
+      <c r="H134" s="23">
+        <f>IF(C134="","",SUMPRODUCT(($C$43:C134=C134)*(2*($D$43:D134="Доход")-1)*$F$43:F134))</f>
         <v/>
       </c>
     </row>
@@ -3111,10 +3300,10 @@
       <c r="C135" s="16" t="n"/>
       <c r="D135" s="16" t="n"/>
       <c r="E135" s="16" t="n"/>
-      <c r="F135" s="20" t="n"/>
+      <c r="F135" s="22" t="n"/>
       <c r="G135" s="16" t="n"/>
-      <c r="H135" s="21">
-        <f>IF(C135="","",SUMPRODUCT(($C$27:C135=C135)*(2*($D$27:D135="Доход")-1)*$F$27:F135))</f>
+      <c r="H135" s="23">
+        <f>IF(C135="","",SUMPRODUCT(($C$43:C135=C135)*(2*($D$43:D135="Доход")-1)*$F$43:F135))</f>
         <v/>
       </c>
     </row>
@@ -3123,10 +3312,10 @@
       <c r="C136" s="16" t="n"/>
       <c r="D136" s="16" t="n"/>
       <c r="E136" s="16" t="n"/>
-      <c r="F136" s="20" t="n"/>
+      <c r="F136" s="22" t="n"/>
       <c r="G136" s="16" t="n"/>
-      <c r="H136" s="21">
-        <f>IF(C136="","",SUMPRODUCT(($C$27:C136=C136)*(2*($D$27:D136="Доход")-1)*$F$27:F136))</f>
+      <c r="H136" s="23">
+        <f>IF(C136="","",SUMPRODUCT(($C$43:C136=C136)*(2*($D$43:D136="Доход")-1)*$F$43:F136))</f>
         <v/>
       </c>
     </row>
@@ -3135,10 +3324,10 @@
       <c r="C137" s="16" t="n"/>
       <c r="D137" s="16" t="n"/>
       <c r="E137" s="16" t="n"/>
-      <c r="F137" s="20" t="n"/>
+      <c r="F137" s="22" t="n"/>
       <c r="G137" s="16" t="n"/>
-      <c r="H137" s="21">
-        <f>IF(C137="","",SUMPRODUCT(($C$27:C137=C137)*(2*($D$27:D137="Доход")-1)*$F$27:F137))</f>
+      <c r="H137" s="23">
+        <f>IF(C137="","",SUMPRODUCT(($C$43:C137=C137)*(2*($D$43:D137="Доход")-1)*$F$43:F137))</f>
         <v/>
       </c>
     </row>
@@ -3147,10 +3336,10 @@
       <c r="C138" s="16" t="n"/>
       <c r="D138" s="16" t="n"/>
       <c r="E138" s="16" t="n"/>
-      <c r="F138" s="20" t="n"/>
+      <c r="F138" s="22" t="n"/>
       <c r="G138" s="16" t="n"/>
-      <c r="H138" s="21">
-        <f>IF(C138="","",SUMPRODUCT(($C$27:C138=C138)*(2*($D$27:D138="Доход")-1)*$F$27:F138))</f>
+      <c r="H138" s="23">
+        <f>IF(C138="","",SUMPRODUCT(($C$43:C138=C138)*(2*($D$43:D138="Доход")-1)*$F$43:F138))</f>
         <v/>
       </c>
     </row>
@@ -3159,10 +3348,10 @@
       <c r="C139" s="16" t="n"/>
       <c r="D139" s="16" t="n"/>
       <c r="E139" s="16" t="n"/>
-      <c r="F139" s="20" t="n"/>
+      <c r="F139" s="22" t="n"/>
       <c r="G139" s="16" t="n"/>
-      <c r="H139" s="21">
-        <f>IF(C139="","",SUMPRODUCT(($C$27:C139=C139)*(2*($D$27:D139="Доход")-1)*$F$27:F139))</f>
+      <c r="H139" s="23">
+        <f>IF(C139="","",SUMPRODUCT(($C$43:C139=C139)*(2*($D$43:D139="Доход")-1)*$F$43:F139))</f>
         <v/>
       </c>
     </row>
@@ -3171,10 +3360,10 @@
       <c r="C140" s="16" t="n"/>
       <c r="D140" s="16" t="n"/>
       <c r="E140" s="16" t="n"/>
-      <c r="F140" s="20" t="n"/>
+      <c r="F140" s="22" t="n"/>
       <c r="G140" s="16" t="n"/>
-      <c r="H140" s="21">
-        <f>IF(C140="","",SUMPRODUCT(($C$27:C140=C140)*(2*($D$27:D140="Доход")-1)*$F$27:F140))</f>
+      <c r="H140" s="23">
+        <f>IF(C140="","",SUMPRODUCT(($C$43:C140=C140)*(2*($D$43:D140="Доход")-1)*$F$43:F140))</f>
         <v/>
       </c>
     </row>
@@ -3183,10 +3372,10 @@
       <c r="C141" s="16" t="n"/>
       <c r="D141" s="16" t="n"/>
       <c r="E141" s="16" t="n"/>
-      <c r="F141" s="20" t="n"/>
+      <c r="F141" s="22" t="n"/>
       <c r="G141" s="16" t="n"/>
-      <c r="H141" s="21">
-        <f>IF(C141="","",SUMPRODUCT(($C$27:C141=C141)*(2*($D$27:D141="Доход")-1)*$F$27:F141))</f>
+      <c r="H141" s="23">
+        <f>IF(C141="","",SUMPRODUCT(($C$43:C141=C141)*(2*($D$43:D141="Доход")-1)*$F$43:F141))</f>
         <v/>
       </c>
     </row>
@@ -3195,10 +3384,10 @@
       <c r="C142" s="16" t="n"/>
       <c r="D142" s="16" t="n"/>
       <c r="E142" s="16" t="n"/>
-      <c r="F142" s="20" t="n"/>
+      <c r="F142" s="22" t="n"/>
       <c r="G142" s="16" t="n"/>
-      <c r="H142" s="21">
-        <f>IF(C142="","",SUMPRODUCT(($C$27:C142=C142)*(2*($D$27:D142="Доход")-1)*$F$27:F142))</f>
+      <c r="H142" s="23">
+        <f>IF(C142="","",SUMPRODUCT(($C$43:C142=C142)*(2*($D$43:D142="Доход")-1)*$F$43:F142))</f>
         <v/>
       </c>
     </row>
@@ -3207,10 +3396,10 @@
       <c r="C143" s="16" t="n"/>
       <c r="D143" s="16" t="n"/>
       <c r="E143" s="16" t="n"/>
-      <c r="F143" s="20" t="n"/>
+      <c r="F143" s="22" t="n"/>
       <c r="G143" s="16" t="n"/>
-      <c r="H143" s="21">
-        <f>IF(C143="","",SUMPRODUCT(($C$27:C143=C143)*(2*($D$27:D143="Доход")-1)*$F$27:F143))</f>
+      <c r="H143" s="23">
+        <f>IF(C143="","",SUMPRODUCT(($C$43:C143=C143)*(2*($D$43:D143="Доход")-1)*$F$43:F143))</f>
         <v/>
       </c>
     </row>
@@ -3219,10 +3408,10 @@
       <c r="C144" s="16" t="n"/>
       <c r="D144" s="16" t="n"/>
       <c r="E144" s="16" t="n"/>
-      <c r="F144" s="20" t="n"/>
+      <c r="F144" s="22" t="n"/>
       <c r="G144" s="16" t="n"/>
-      <c r="H144" s="21">
-        <f>IF(C144="","",SUMPRODUCT(($C$27:C144=C144)*(2*($D$27:D144="Доход")-1)*$F$27:F144))</f>
+      <c r="H144" s="23">
+        <f>IF(C144="","",SUMPRODUCT(($C$43:C144=C144)*(2*($D$43:D144="Доход")-1)*$F$43:F144))</f>
         <v/>
       </c>
     </row>
@@ -3231,10 +3420,10 @@
       <c r="C145" s="16" t="n"/>
       <c r="D145" s="16" t="n"/>
       <c r="E145" s="16" t="n"/>
-      <c r="F145" s="20" t="n"/>
+      <c r="F145" s="22" t="n"/>
       <c r="G145" s="16" t="n"/>
-      <c r="H145" s="21">
-        <f>IF(C145="","",SUMPRODUCT(($C$27:C145=C145)*(2*($D$27:D145="Доход")-1)*$F$27:F145))</f>
+      <c r="H145" s="23">
+        <f>IF(C145="","",SUMPRODUCT(($C$43:C145=C145)*(2*($D$43:D145="Доход")-1)*$F$43:F145))</f>
         <v/>
       </c>
     </row>
@@ -3243,10 +3432,10 @@
       <c r="C146" s="16" t="n"/>
       <c r="D146" s="16" t="n"/>
       <c r="E146" s="16" t="n"/>
-      <c r="F146" s="20" t="n"/>
+      <c r="F146" s="22" t="n"/>
       <c r="G146" s="16" t="n"/>
-      <c r="H146" s="21">
-        <f>IF(C146="","",SUMPRODUCT(($C$27:C146=C146)*(2*($D$27:D146="Доход")-1)*$F$27:F146))</f>
+      <c r="H146" s="23">
+        <f>IF(C146="","",SUMPRODUCT(($C$43:C146=C146)*(2*($D$43:D146="Доход")-1)*$F$43:F146))</f>
         <v/>
       </c>
     </row>
@@ -3255,10 +3444,10 @@
       <c r="C147" s="16" t="n"/>
       <c r="D147" s="16" t="n"/>
       <c r="E147" s="16" t="n"/>
-      <c r="F147" s="20" t="n"/>
+      <c r="F147" s="22" t="n"/>
       <c r="G147" s="16" t="n"/>
-      <c r="H147" s="21">
-        <f>IF(C147="","",SUMPRODUCT(($C$27:C147=C147)*(2*($D$27:D147="Доход")-1)*$F$27:F147))</f>
+      <c r="H147" s="23">
+        <f>IF(C147="","",SUMPRODUCT(($C$43:C147=C147)*(2*($D$43:D147="Доход")-1)*$F$43:F147))</f>
         <v/>
       </c>
     </row>
@@ -3267,10 +3456,10 @@
       <c r="C148" s="16" t="n"/>
       <c r="D148" s="16" t="n"/>
       <c r="E148" s="16" t="n"/>
-      <c r="F148" s="20" t="n"/>
+      <c r="F148" s="22" t="n"/>
       <c r="G148" s="16" t="n"/>
-      <c r="H148" s="21">
-        <f>IF(C148="","",SUMPRODUCT(($C$27:C148=C148)*(2*($D$27:D148="Доход")-1)*$F$27:F148))</f>
+      <c r="H148" s="23">
+        <f>IF(C148="","",SUMPRODUCT(($C$43:C148=C148)*(2*($D$43:D148="Доход")-1)*$F$43:F148))</f>
         <v/>
       </c>
     </row>
@@ -3279,10 +3468,10 @@
       <c r="C149" s="16" t="n"/>
       <c r="D149" s="16" t="n"/>
       <c r="E149" s="16" t="n"/>
-      <c r="F149" s="20" t="n"/>
+      <c r="F149" s="22" t="n"/>
       <c r="G149" s="16" t="n"/>
-      <c r="H149" s="21">
-        <f>IF(C149="","",SUMPRODUCT(($C$27:C149=C149)*(2*($D$27:D149="Доход")-1)*$F$27:F149))</f>
+      <c r="H149" s="23">
+        <f>IF(C149="","",SUMPRODUCT(($C$43:C149=C149)*(2*($D$43:D149="Доход")-1)*$F$43:F149))</f>
         <v/>
       </c>
     </row>
@@ -3291,10 +3480,10 @@
       <c r="C150" s="16" t="n"/>
       <c r="D150" s="16" t="n"/>
       <c r="E150" s="16" t="n"/>
-      <c r="F150" s="20" t="n"/>
+      <c r="F150" s="22" t="n"/>
       <c r="G150" s="16" t="n"/>
-      <c r="H150" s="21">
-        <f>IF(C150="","",SUMPRODUCT(($C$27:C150=C150)*(2*($D$27:D150="Доход")-1)*$F$27:F150))</f>
+      <c r="H150" s="23">
+        <f>IF(C150="","",SUMPRODUCT(($C$43:C150=C150)*(2*($D$43:D150="Доход")-1)*$F$43:F150))</f>
         <v/>
       </c>
     </row>
@@ -3303,10 +3492,10 @@
       <c r="C151" s="16" t="n"/>
       <c r="D151" s="16" t="n"/>
       <c r="E151" s="16" t="n"/>
-      <c r="F151" s="20" t="n"/>
+      <c r="F151" s="22" t="n"/>
       <c r="G151" s="16" t="n"/>
-      <c r="H151" s="21">
-        <f>IF(C151="","",SUMPRODUCT(($C$27:C151=C151)*(2*($D$27:D151="Доход")-1)*$F$27:F151))</f>
+      <c r="H151" s="23">
+        <f>IF(C151="","",SUMPRODUCT(($C$43:C151=C151)*(2*($D$43:D151="Доход")-1)*$F$43:F151))</f>
         <v/>
       </c>
     </row>
@@ -3315,10 +3504,10 @@
       <c r="C152" s="16" t="n"/>
       <c r="D152" s="16" t="n"/>
       <c r="E152" s="16" t="n"/>
-      <c r="F152" s="20" t="n"/>
+      <c r="F152" s="22" t="n"/>
       <c r="G152" s="16" t="n"/>
-      <c r="H152" s="21">
-        <f>IF(C152="","",SUMPRODUCT(($C$27:C152=C152)*(2*($D$27:D152="Доход")-1)*$F$27:F152))</f>
+      <c r="H152" s="23">
+        <f>IF(C152="","",SUMPRODUCT(($C$43:C152=C152)*(2*($D$43:D152="Доход")-1)*$F$43:F152))</f>
         <v/>
       </c>
     </row>
@@ -3327,10 +3516,10 @@
       <c r="C153" s="16" t="n"/>
       <c r="D153" s="16" t="n"/>
       <c r="E153" s="16" t="n"/>
-      <c r="F153" s="20" t="n"/>
+      <c r="F153" s="22" t="n"/>
       <c r="G153" s="16" t="n"/>
-      <c r="H153" s="21">
-        <f>IF(C153="","",SUMPRODUCT(($C$27:C153=C153)*(2*($D$27:D153="Доход")-1)*$F$27:F153))</f>
+      <c r="H153" s="23">
+        <f>IF(C153="","",SUMPRODUCT(($C$43:C153=C153)*(2*($D$43:D153="Доход")-1)*$F$43:F153))</f>
         <v/>
       </c>
     </row>
@@ -3339,10 +3528,10 @@
       <c r="C154" s="16" t="n"/>
       <c r="D154" s="16" t="n"/>
       <c r="E154" s="16" t="n"/>
-      <c r="F154" s="20" t="n"/>
+      <c r="F154" s="22" t="n"/>
       <c r="G154" s="16" t="n"/>
-      <c r="H154" s="21">
-        <f>IF(C154="","",SUMPRODUCT(($C$27:C154=C154)*(2*($D$27:D154="Доход")-1)*$F$27:F154))</f>
+      <c r="H154" s="23">
+        <f>IF(C154="","",SUMPRODUCT(($C$43:C154=C154)*(2*($D$43:D154="Доход")-1)*$F$43:F154))</f>
         <v/>
       </c>
     </row>
@@ -3351,10 +3540,10 @@
       <c r="C155" s="16" t="n"/>
       <c r="D155" s="16" t="n"/>
       <c r="E155" s="16" t="n"/>
-      <c r="F155" s="20" t="n"/>
+      <c r="F155" s="22" t="n"/>
       <c r="G155" s="16" t="n"/>
-      <c r="H155" s="21">
-        <f>IF(C155="","",SUMPRODUCT(($C$27:C155=C155)*(2*($D$27:D155="Доход")-1)*$F$27:F155))</f>
+      <c r="H155" s="23">
+        <f>IF(C155="","",SUMPRODUCT(($C$43:C155=C155)*(2*($D$43:D155="Доход")-1)*$F$43:F155))</f>
         <v/>
       </c>
     </row>
@@ -3363,10 +3552,10 @@
       <c r="C156" s="16" t="n"/>
       <c r="D156" s="16" t="n"/>
       <c r="E156" s="16" t="n"/>
-      <c r="F156" s="20" t="n"/>
+      <c r="F156" s="22" t="n"/>
       <c r="G156" s="16" t="n"/>
-      <c r="H156" s="21">
-        <f>IF(C156="","",SUMPRODUCT(($C$27:C156=C156)*(2*($D$27:D156="Доход")-1)*$F$27:F156))</f>
+      <c r="H156" s="23">
+        <f>IF(C156="","",SUMPRODUCT(($C$43:C156=C156)*(2*($D$43:D156="Доход")-1)*$F$43:F156))</f>
         <v/>
       </c>
     </row>
@@ -3375,10 +3564,10 @@
       <c r="C157" s="16" t="n"/>
       <c r="D157" s="16" t="n"/>
       <c r="E157" s="16" t="n"/>
-      <c r="F157" s="20" t="n"/>
+      <c r="F157" s="22" t="n"/>
       <c r="G157" s="16" t="n"/>
-      <c r="H157" s="21">
-        <f>IF(C157="","",SUMPRODUCT(($C$27:C157=C157)*(2*($D$27:D157="Доход")-1)*$F$27:F157))</f>
+      <c r="H157" s="23">
+        <f>IF(C157="","",SUMPRODUCT(($C$43:C157=C157)*(2*($D$43:D157="Доход")-1)*$F$43:F157))</f>
         <v/>
       </c>
     </row>
@@ -3387,10 +3576,10 @@
       <c r="C158" s="16" t="n"/>
       <c r="D158" s="16" t="n"/>
       <c r="E158" s="16" t="n"/>
-      <c r="F158" s="20" t="n"/>
+      <c r="F158" s="22" t="n"/>
       <c r="G158" s="16" t="n"/>
-      <c r="H158" s="21">
-        <f>IF(C158="","",SUMPRODUCT(($C$27:C158=C158)*(2*($D$27:D158="Доход")-1)*$F$27:F158))</f>
+      <c r="H158" s="23">
+        <f>IF(C158="","",SUMPRODUCT(($C$43:C158=C158)*(2*($D$43:D158="Доход")-1)*$F$43:F158))</f>
         <v/>
       </c>
     </row>
@@ -3399,10 +3588,10 @@
       <c r="C159" s="16" t="n"/>
       <c r="D159" s="16" t="n"/>
       <c r="E159" s="16" t="n"/>
-      <c r="F159" s="20" t="n"/>
+      <c r="F159" s="22" t="n"/>
       <c r="G159" s="16" t="n"/>
-      <c r="H159" s="21">
-        <f>IF(C159="","",SUMPRODUCT(($C$27:C159=C159)*(2*($D$27:D159="Доход")-1)*$F$27:F159))</f>
+      <c r="H159" s="23">
+        <f>IF(C159="","",SUMPRODUCT(($C$43:C159=C159)*(2*($D$43:D159="Доход")-1)*$F$43:F159))</f>
         <v/>
       </c>
     </row>
@@ -3411,10 +3600,10 @@
       <c r="C160" s="16" t="n"/>
       <c r="D160" s="16" t="n"/>
       <c r="E160" s="16" t="n"/>
-      <c r="F160" s="20" t="n"/>
+      <c r="F160" s="22" t="n"/>
       <c r="G160" s="16" t="n"/>
-      <c r="H160" s="21">
-        <f>IF(C160="","",SUMPRODUCT(($C$27:C160=C160)*(2*($D$27:D160="Доход")-1)*$F$27:F160))</f>
+      <c r="H160" s="23">
+        <f>IF(C160="","",SUMPRODUCT(($C$43:C160=C160)*(2*($D$43:D160="Доход")-1)*$F$43:F160))</f>
         <v/>
       </c>
     </row>
@@ -3423,10 +3612,10 @@
       <c r="C161" s="16" t="n"/>
       <c r="D161" s="16" t="n"/>
       <c r="E161" s="16" t="n"/>
-      <c r="F161" s="20" t="n"/>
+      <c r="F161" s="22" t="n"/>
       <c r="G161" s="16" t="n"/>
-      <c r="H161" s="21">
-        <f>IF(C161="","",SUMPRODUCT(($C$27:C161=C161)*(2*($D$27:D161="Доход")-1)*$F$27:F161))</f>
+      <c r="H161" s="23">
+        <f>IF(C161="","",SUMPRODUCT(($C$43:C161=C161)*(2*($D$43:D161="Доход")-1)*$F$43:F161))</f>
         <v/>
       </c>
     </row>
@@ -3435,10 +3624,10 @@
       <c r="C162" s="16" t="n"/>
       <c r="D162" s="16" t="n"/>
       <c r="E162" s="16" t="n"/>
-      <c r="F162" s="20" t="n"/>
+      <c r="F162" s="22" t="n"/>
       <c r="G162" s="16" t="n"/>
-      <c r="H162" s="21">
-        <f>IF(C162="","",SUMPRODUCT(($C$27:C162=C162)*(2*($D$27:D162="Доход")-1)*$F$27:F162))</f>
+      <c r="H162" s="23">
+        <f>IF(C162="","",SUMPRODUCT(($C$43:C162=C162)*(2*($D$43:D162="Доход")-1)*$F$43:F162))</f>
         <v/>
       </c>
     </row>
@@ -3447,10 +3636,10 @@
       <c r="C163" s="16" t="n"/>
       <c r="D163" s="16" t="n"/>
       <c r="E163" s="16" t="n"/>
-      <c r="F163" s="20" t="n"/>
+      <c r="F163" s="22" t="n"/>
       <c r="G163" s="16" t="n"/>
-      <c r="H163" s="21">
-        <f>IF(C163="","",SUMPRODUCT(($C$27:C163=C163)*(2*($D$27:D163="Доход")-1)*$F$27:F163))</f>
+      <c r="H163" s="23">
+        <f>IF(C163="","",SUMPRODUCT(($C$43:C163=C163)*(2*($D$43:D163="Доход")-1)*$F$43:F163))</f>
         <v/>
       </c>
     </row>
@@ -3459,10 +3648,10 @@
       <c r="C164" s="16" t="n"/>
       <c r="D164" s="16" t="n"/>
       <c r="E164" s="16" t="n"/>
-      <c r="F164" s="20" t="n"/>
+      <c r="F164" s="22" t="n"/>
       <c r="G164" s="16" t="n"/>
-      <c r="H164" s="21">
-        <f>IF(C164="","",SUMPRODUCT(($C$27:C164=C164)*(2*($D$27:D164="Доход")-1)*$F$27:F164))</f>
+      <c r="H164" s="23">
+        <f>IF(C164="","",SUMPRODUCT(($C$43:C164=C164)*(2*($D$43:D164="Доход")-1)*$F$43:F164))</f>
         <v/>
       </c>
     </row>
@@ -3471,10 +3660,10 @@
       <c r="C165" s="16" t="n"/>
       <c r="D165" s="16" t="n"/>
       <c r="E165" s="16" t="n"/>
-      <c r="F165" s="20" t="n"/>
+      <c r="F165" s="22" t="n"/>
       <c r="G165" s="16" t="n"/>
-      <c r="H165" s="21">
-        <f>IF(C165="","",SUMPRODUCT(($C$27:C165=C165)*(2*($D$27:D165="Доход")-1)*$F$27:F165))</f>
+      <c r="H165" s="23">
+        <f>IF(C165="","",SUMPRODUCT(($C$43:C165=C165)*(2*($D$43:D165="Доход")-1)*$F$43:F165))</f>
         <v/>
       </c>
     </row>
@@ -3483,10 +3672,10 @@
       <c r="C166" s="16" t="n"/>
       <c r="D166" s="16" t="n"/>
       <c r="E166" s="16" t="n"/>
-      <c r="F166" s="20" t="n"/>
+      <c r="F166" s="22" t="n"/>
       <c r="G166" s="16" t="n"/>
-      <c r="H166" s="21">
-        <f>IF(C166="","",SUMPRODUCT(($C$27:C166=C166)*(2*($D$27:D166="Доход")-1)*$F$27:F166))</f>
+      <c r="H166" s="23">
+        <f>IF(C166="","",SUMPRODUCT(($C$43:C166=C166)*(2*($D$43:D166="Доход")-1)*$F$43:F166))</f>
         <v/>
       </c>
     </row>
@@ -3495,10 +3684,10 @@
       <c r="C167" s="16" t="n"/>
       <c r="D167" s="16" t="n"/>
       <c r="E167" s="16" t="n"/>
-      <c r="F167" s="20" t="n"/>
+      <c r="F167" s="22" t="n"/>
       <c r="G167" s="16" t="n"/>
-      <c r="H167" s="21">
-        <f>IF(C167="","",SUMPRODUCT(($C$27:C167=C167)*(2*($D$27:D167="Доход")-1)*$F$27:F167))</f>
+      <c r="H167" s="23">
+        <f>IF(C167="","",SUMPRODUCT(($C$43:C167=C167)*(2*($D$43:D167="Доход")-1)*$F$43:F167))</f>
         <v/>
       </c>
     </row>
@@ -3507,10 +3696,10 @@
       <c r="C168" s="16" t="n"/>
       <c r="D168" s="16" t="n"/>
       <c r="E168" s="16" t="n"/>
-      <c r="F168" s="20" t="n"/>
+      <c r="F168" s="22" t="n"/>
       <c r="G168" s="16" t="n"/>
-      <c r="H168" s="21">
-        <f>IF(C168="","",SUMPRODUCT(($C$27:C168=C168)*(2*($D$27:D168="Доход")-1)*$F$27:F168))</f>
+      <c r="H168" s="23">
+        <f>IF(C168="","",SUMPRODUCT(($C$43:C168=C168)*(2*($D$43:D168="Доход")-1)*$F$43:F168))</f>
         <v/>
       </c>
     </row>
@@ -3519,10 +3708,10 @@
       <c r="C169" s="16" t="n"/>
       <c r="D169" s="16" t="n"/>
       <c r="E169" s="16" t="n"/>
-      <c r="F169" s="20" t="n"/>
+      <c r="F169" s="22" t="n"/>
       <c r="G169" s="16" t="n"/>
-      <c r="H169" s="21">
-        <f>IF(C169="","",SUMPRODUCT(($C$27:C169=C169)*(2*($D$27:D169="Доход")-1)*$F$27:F169))</f>
+      <c r="H169" s="23">
+        <f>IF(C169="","",SUMPRODUCT(($C$43:C169=C169)*(2*($D$43:D169="Доход")-1)*$F$43:F169))</f>
         <v/>
       </c>
     </row>
@@ -3531,10 +3720,10 @@
       <c r="C170" s="16" t="n"/>
       <c r="D170" s="16" t="n"/>
       <c r="E170" s="16" t="n"/>
-      <c r="F170" s="20" t="n"/>
+      <c r="F170" s="22" t="n"/>
       <c r="G170" s="16" t="n"/>
-      <c r="H170" s="21">
-        <f>IF(C170="","",SUMPRODUCT(($C$27:C170=C170)*(2*($D$27:D170="Доход")-1)*$F$27:F170))</f>
+      <c r="H170" s="23">
+        <f>IF(C170="","",SUMPRODUCT(($C$43:C170=C170)*(2*($D$43:D170="Доход")-1)*$F$43:F170))</f>
         <v/>
       </c>
     </row>
@@ -3543,10 +3732,10 @@
       <c r="C171" s="16" t="n"/>
       <c r="D171" s="16" t="n"/>
       <c r="E171" s="16" t="n"/>
-      <c r="F171" s="20" t="n"/>
+      <c r="F171" s="22" t="n"/>
       <c r="G171" s="16" t="n"/>
-      <c r="H171" s="21">
-        <f>IF(C171="","",SUMPRODUCT(($C$27:C171=C171)*(2*($D$27:D171="Доход")-1)*$F$27:F171))</f>
+      <c r="H171" s="23">
+        <f>IF(C171="","",SUMPRODUCT(($C$43:C171=C171)*(2*($D$43:D171="Доход")-1)*$F$43:F171))</f>
         <v/>
       </c>
     </row>
@@ -3555,10 +3744,10 @@
       <c r="C172" s="16" t="n"/>
       <c r="D172" s="16" t="n"/>
       <c r="E172" s="16" t="n"/>
-      <c r="F172" s="20" t="n"/>
+      <c r="F172" s="22" t="n"/>
       <c r="G172" s="16" t="n"/>
-      <c r="H172" s="21">
-        <f>IF(C172="","",SUMPRODUCT(($C$27:C172=C172)*(2*($D$27:D172="Доход")-1)*$F$27:F172))</f>
+      <c r="H172" s="23">
+        <f>IF(C172="","",SUMPRODUCT(($C$43:C172=C172)*(2*($D$43:D172="Доход")-1)*$F$43:F172))</f>
         <v/>
       </c>
     </row>
@@ -3567,10 +3756,10 @@
       <c r="C173" s="16" t="n"/>
       <c r="D173" s="16" t="n"/>
       <c r="E173" s="16" t="n"/>
-      <c r="F173" s="20" t="n"/>
+      <c r="F173" s="22" t="n"/>
       <c r="G173" s="16" t="n"/>
-      <c r="H173" s="21">
-        <f>IF(C173="","",SUMPRODUCT(($C$27:C173=C173)*(2*($D$27:D173="Доход")-1)*$F$27:F173))</f>
+      <c r="H173" s="23">
+        <f>IF(C173="","",SUMPRODUCT(($C$43:C173=C173)*(2*($D$43:D173="Доход")-1)*$F$43:F173))</f>
         <v/>
       </c>
     </row>
@@ -3579,10 +3768,10 @@
       <c r="C174" s="16" t="n"/>
       <c r="D174" s="16" t="n"/>
       <c r="E174" s="16" t="n"/>
-      <c r="F174" s="20" t="n"/>
+      <c r="F174" s="22" t="n"/>
       <c r="G174" s="16" t="n"/>
-      <c r="H174" s="21">
-        <f>IF(C174="","",SUMPRODUCT(($C$27:C174=C174)*(2*($D$27:D174="Доход")-1)*$F$27:F174))</f>
+      <c r="H174" s="23">
+        <f>IF(C174="","",SUMPRODUCT(($C$43:C174=C174)*(2*($D$43:D174="Доход")-1)*$F$43:F174))</f>
         <v/>
       </c>
     </row>
@@ -3591,10 +3780,10 @@
       <c r="C175" s="16" t="n"/>
       <c r="D175" s="16" t="n"/>
       <c r="E175" s="16" t="n"/>
-      <c r="F175" s="20" t="n"/>
+      <c r="F175" s="22" t="n"/>
       <c r="G175" s="16" t="n"/>
-      <c r="H175" s="21">
-        <f>IF(C175="","",SUMPRODUCT(($C$27:C175=C175)*(2*($D$27:D175="Доход")-1)*$F$27:F175))</f>
+      <c r="H175" s="23">
+        <f>IF(C175="","",SUMPRODUCT(($C$43:C175=C175)*(2*($D$43:D175="Доход")-1)*$F$43:F175))</f>
         <v/>
       </c>
     </row>
@@ -3603,10 +3792,10 @@
       <c r="C176" s="16" t="n"/>
       <c r="D176" s="16" t="n"/>
       <c r="E176" s="16" t="n"/>
-      <c r="F176" s="20" t="n"/>
+      <c r="F176" s="22" t="n"/>
       <c r="G176" s="16" t="n"/>
-      <c r="H176" s="21">
-        <f>IF(C176="","",SUMPRODUCT(($C$27:C176=C176)*(2*($D$27:D176="Доход")-1)*$F$27:F176))</f>
+      <c r="H176" s="23">
+        <f>IF(C176="","",SUMPRODUCT(($C$43:C176=C176)*(2*($D$43:D176="Доход")-1)*$F$43:F176))</f>
         <v/>
       </c>
     </row>
@@ -3615,10 +3804,10 @@
       <c r="C177" s="16" t="n"/>
       <c r="D177" s="16" t="n"/>
       <c r="E177" s="16" t="n"/>
-      <c r="F177" s="20" t="n"/>
+      <c r="F177" s="22" t="n"/>
       <c r="G177" s="16" t="n"/>
-      <c r="H177" s="21">
-        <f>IF(C177="","",SUMPRODUCT(($C$27:C177=C177)*(2*($D$27:D177="Доход")-1)*$F$27:F177))</f>
+      <c r="H177" s="23">
+        <f>IF(C177="","",SUMPRODUCT(($C$43:C177=C177)*(2*($D$43:D177="Доход")-1)*$F$43:F177))</f>
         <v/>
       </c>
     </row>
@@ -3627,10 +3816,10 @@
       <c r="C178" s="16" t="n"/>
       <c r="D178" s="16" t="n"/>
       <c r="E178" s="16" t="n"/>
-      <c r="F178" s="20" t="n"/>
+      <c r="F178" s="22" t="n"/>
       <c r="G178" s="16" t="n"/>
-      <c r="H178" s="21">
-        <f>IF(C178="","",SUMPRODUCT(($C$27:C178=C178)*(2*($D$27:D178="Доход")-1)*$F$27:F178))</f>
+      <c r="H178" s="23">
+        <f>IF(C178="","",SUMPRODUCT(($C$43:C178=C178)*(2*($D$43:D178="Доход")-1)*$F$43:F178))</f>
         <v/>
       </c>
     </row>
@@ -3639,10 +3828,10 @@
       <c r="C179" s="16" t="n"/>
       <c r="D179" s="16" t="n"/>
       <c r="E179" s="16" t="n"/>
-      <c r="F179" s="20" t="n"/>
+      <c r="F179" s="22" t="n"/>
       <c r="G179" s="16" t="n"/>
-      <c r="H179" s="21">
-        <f>IF(C179="","",SUMPRODUCT(($C$27:C179=C179)*(2*($D$27:D179="Доход")-1)*$F$27:F179))</f>
+      <c r="H179" s="23">
+        <f>IF(C179="","",SUMPRODUCT(($C$43:C179=C179)*(2*($D$43:D179="Доход")-1)*$F$43:F179))</f>
         <v/>
       </c>
     </row>
@@ -3651,10 +3840,10 @@
       <c r="C180" s="16" t="n"/>
       <c r="D180" s="16" t="n"/>
       <c r="E180" s="16" t="n"/>
-      <c r="F180" s="20" t="n"/>
+      <c r="F180" s="22" t="n"/>
       <c r="G180" s="16" t="n"/>
-      <c r="H180" s="21">
-        <f>IF(C180="","",SUMPRODUCT(($C$27:C180=C180)*(2*($D$27:D180="Доход")-1)*$F$27:F180))</f>
+      <c r="H180" s="23">
+        <f>IF(C180="","",SUMPRODUCT(($C$43:C180=C180)*(2*($D$43:D180="Доход")-1)*$F$43:F180))</f>
         <v/>
       </c>
     </row>
@@ -3663,10 +3852,10 @@
       <c r="C181" s="16" t="n"/>
       <c r="D181" s="16" t="n"/>
       <c r="E181" s="16" t="n"/>
-      <c r="F181" s="20" t="n"/>
+      <c r="F181" s="22" t="n"/>
       <c r="G181" s="16" t="n"/>
-      <c r="H181" s="21">
-        <f>IF(C181="","",SUMPRODUCT(($C$27:C181=C181)*(2*($D$27:D181="Доход")-1)*$F$27:F181))</f>
+      <c r="H181" s="23">
+        <f>IF(C181="","",SUMPRODUCT(($C$43:C181=C181)*(2*($D$43:D181="Доход")-1)*$F$43:F181))</f>
         <v/>
       </c>
     </row>
@@ -3675,10 +3864,10 @@
       <c r="C182" s="16" t="n"/>
       <c r="D182" s="16" t="n"/>
       <c r="E182" s="16" t="n"/>
-      <c r="F182" s="20" t="n"/>
+      <c r="F182" s="22" t="n"/>
       <c r="G182" s="16" t="n"/>
-      <c r="H182" s="21">
-        <f>IF(C182="","",SUMPRODUCT(($C$27:C182=C182)*(2*($D$27:D182="Доход")-1)*$F$27:F182))</f>
+      <c r="H182" s="23">
+        <f>IF(C182="","",SUMPRODUCT(($C$43:C182=C182)*(2*($D$43:D182="Доход")-1)*$F$43:F182))</f>
         <v/>
       </c>
     </row>
@@ -3687,10 +3876,10 @@
       <c r="C183" s="16" t="n"/>
       <c r="D183" s="16" t="n"/>
       <c r="E183" s="16" t="n"/>
-      <c r="F183" s="20" t="n"/>
+      <c r="F183" s="22" t="n"/>
       <c r="G183" s="16" t="n"/>
-      <c r="H183" s="21">
-        <f>IF(C183="","",SUMPRODUCT(($C$27:C183=C183)*(2*($D$27:D183="Доход")-1)*$F$27:F183))</f>
+      <c r="H183" s="23">
+        <f>IF(C183="","",SUMPRODUCT(($C$43:C183=C183)*(2*($D$43:D183="Доход")-1)*$F$43:F183))</f>
         <v/>
       </c>
     </row>
@@ -3699,10 +3888,10 @@
       <c r="C184" s="16" t="n"/>
       <c r="D184" s="16" t="n"/>
       <c r="E184" s="16" t="n"/>
-      <c r="F184" s="20" t="n"/>
+      <c r="F184" s="22" t="n"/>
       <c r="G184" s="16" t="n"/>
-      <c r="H184" s="21">
-        <f>IF(C184="","",SUMPRODUCT(($C$27:C184=C184)*(2*($D$27:D184="Доход")-1)*$F$27:F184))</f>
+      <c r="H184" s="23">
+        <f>IF(C184="","",SUMPRODUCT(($C$43:C184=C184)*(2*($D$43:D184="Доход")-1)*$F$43:F184))</f>
         <v/>
       </c>
     </row>
@@ -3711,10 +3900,10 @@
       <c r="C185" s="16" t="n"/>
       <c r="D185" s="16" t="n"/>
       <c r="E185" s="16" t="n"/>
-      <c r="F185" s="20" t="n"/>
+      <c r="F185" s="22" t="n"/>
       <c r="G185" s="16" t="n"/>
-      <c r="H185" s="21">
-        <f>IF(C185="","",SUMPRODUCT(($C$27:C185=C185)*(2*($D$27:D185="Доход")-1)*$F$27:F185))</f>
+      <c r="H185" s="23">
+        <f>IF(C185="","",SUMPRODUCT(($C$43:C185=C185)*(2*($D$43:D185="Доход")-1)*$F$43:F185))</f>
         <v/>
       </c>
     </row>
@@ -3723,10 +3912,10 @@
       <c r="C186" s="16" t="n"/>
       <c r="D186" s="16" t="n"/>
       <c r="E186" s="16" t="n"/>
-      <c r="F186" s="20" t="n"/>
+      <c r="F186" s="22" t="n"/>
       <c r="G186" s="16" t="n"/>
-      <c r="H186" s="21">
-        <f>IF(C186="","",SUMPRODUCT(($C$27:C186=C186)*(2*($D$27:D186="Доход")-1)*$F$27:F186))</f>
+      <c r="H186" s="23">
+        <f>IF(C186="","",SUMPRODUCT(($C$43:C186=C186)*(2*($D$43:D186="Доход")-1)*$F$43:F186))</f>
         <v/>
       </c>
     </row>
@@ -3735,10 +3924,10 @@
       <c r="C187" s="16" t="n"/>
       <c r="D187" s="16" t="n"/>
       <c r="E187" s="16" t="n"/>
-      <c r="F187" s="20" t="n"/>
+      <c r="F187" s="22" t="n"/>
       <c r="G187" s="16" t="n"/>
-      <c r="H187" s="21">
-        <f>IF(C187="","",SUMPRODUCT(($C$27:C187=C187)*(2*($D$27:D187="Доход")-1)*$F$27:F187))</f>
+      <c r="H187" s="23">
+        <f>IF(C187="","",SUMPRODUCT(($C$43:C187=C187)*(2*($D$43:D187="Доход")-1)*$F$43:F187))</f>
         <v/>
       </c>
     </row>
@@ -3747,10 +3936,10 @@
       <c r="C188" s="16" t="n"/>
       <c r="D188" s="16" t="n"/>
       <c r="E188" s="16" t="n"/>
-      <c r="F188" s="20" t="n"/>
+      <c r="F188" s="22" t="n"/>
       <c r="G188" s="16" t="n"/>
-      <c r="H188" s="21">
-        <f>IF(C188="","",SUMPRODUCT(($C$27:C188=C188)*(2*($D$27:D188="Доход")-1)*$F$27:F188))</f>
+      <c r="H188" s="23">
+        <f>IF(C188="","",SUMPRODUCT(($C$43:C188=C188)*(2*($D$43:D188="Доход")-1)*$F$43:F188))</f>
         <v/>
       </c>
     </row>
@@ -3759,10 +3948,10 @@
       <c r="C189" s="16" t="n"/>
       <c r="D189" s="16" t="n"/>
       <c r="E189" s="16" t="n"/>
-      <c r="F189" s="20" t="n"/>
+      <c r="F189" s="22" t="n"/>
       <c r="G189" s="16" t="n"/>
-      <c r="H189" s="21">
-        <f>IF(C189="","",SUMPRODUCT(($C$27:C189=C189)*(2*($D$27:D189="Доход")-1)*$F$27:F189))</f>
+      <c r="H189" s="23">
+        <f>IF(C189="","",SUMPRODUCT(($C$43:C189=C189)*(2*($D$43:D189="Доход")-1)*$F$43:F189))</f>
         <v/>
       </c>
     </row>
@@ -3771,10 +3960,10 @@
       <c r="C190" s="16" t="n"/>
       <c r="D190" s="16" t="n"/>
       <c r="E190" s="16" t="n"/>
-      <c r="F190" s="20" t="n"/>
+      <c r="F190" s="22" t="n"/>
       <c r="G190" s="16" t="n"/>
-      <c r="H190" s="21">
-        <f>IF(C190="","",SUMPRODUCT(($C$27:C190=C190)*(2*($D$27:D190="Доход")-1)*$F$27:F190))</f>
+      <c r="H190" s="23">
+        <f>IF(C190="","",SUMPRODUCT(($C$43:C190=C190)*(2*($D$43:D190="Доход")-1)*$F$43:F190))</f>
         <v/>
       </c>
     </row>
@@ -3783,10 +3972,10 @@
       <c r="C191" s="16" t="n"/>
       <c r="D191" s="16" t="n"/>
       <c r="E191" s="16" t="n"/>
-      <c r="F191" s="20" t="n"/>
+      <c r="F191" s="22" t="n"/>
       <c r="G191" s="16" t="n"/>
-      <c r="H191" s="21">
-        <f>IF(C191="","",SUMPRODUCT(($C$27:C191=C191)*(2*($D$27:D191="Доход")-1)*$F$27:F191))</f>
+      <c r="H191" s="23">
+        <f>IF(C191="","",SUMPRODUCT(($C$43:C191=C191)*(2*($D$43:D191="Доход")-1)*$F$43:F191))</f>
         <v/>
       </c>
     </row>
@@ -3795,10 +3984,10 @@
       <c r="C192" s="16" t="n"/>
       <c r="D192" s="16" t="n"/>
       <c r="E192" s="16" t="n"/>
-      <c r="F192" s="20" t="n"/>
+      <c r="F192" s="22" t="n"/>
       <c r="G192" s="16" t="n"/>
-      <c r="H192" s="21">
-        <f>IF(C192="","",SUMPRODUCT(($C$27:C192=C192)*(2*($D$27:D192="Доход")-1)*$F$27:F192))</f>
+      <c r="H192" s="23">
+        <f>IF(C192="","",SUMPRODUCT(($C$43:C192=C192)*(2*($D$43:D192="Доход")-1)*$F$43:F192))</f>
         <v/>
       </c>
     </row>
@@ -3807,10 +3996,10 @@
       <c r="C193" s="16" t="n"/>
       <c r="D193" s="16" t="n"/>
       <c r="E193" s="16" t="n"/>
-      <c r="F193" s="20" t="n"/>
+      <c r="F193" s="22" t="n"/>
       <c r="G193" s="16" t="n"/>
-      <c r="H193" s="21">
-        <f>IF(C193="","",SUMPRODUCT(($C$27:C193=C193)*(2*($D$27:D193="Доход")-1)*$F$27:F193))</f>
+      <c r="H193" s="23">
+        <f>IF(C193="","",SUMPRODUCT(($C$43:C193=C193)*(2*($D$43:D193="Доход")-1)*$F$43:F193))</f>
         <v/>
       </c>
     </row>
@@ -3819,10 +4008,10 @@
       <c r="C194" s="16" t="n"/>
       <c r="D194" s="16" t="n"/>
       <c r="E194" s="16" t="n"/>
-      <c r="F194" s="20" t="n"/>
+      <c r="F194" s="22" t="n"/>
       <c r="G194" s="16" t="n"/>
-      <c r="H194" s="21">
-        <f>IF(C194="","",SUMPRODUCT(($C$27:C194=C194)*(2*($D$27:D194="Доход")-1)*$F$27:F194))</f>
+      <c r="H194" s="23">
+        <f>IF(C194="","",SUMPRODUCT(($C$43:C194=C194)*(2*($D$43:D194="Доход")-1)*$F$43:F194))</f>
         <v/>
       </c>
     </row>
@@ -3831,10 +4020,10 @@
       <c r="C195" s="16" t="n"/>
       <c r="D195" s="16" t="n"/>
       <c r="E195" s="16" t="n"/>
-      <c r="F195" s="20" t="n"/>
+      <c r="F195" s="22" t="n"/>
       <c r="G195" s="16" t="n"/>
-      <c r="H195" s="21">
-        <f>IF(C195="","",SUMPRODUCT(($C$27:C195=C195)*(2*($D$27:D195="Доход")-1)*$F$27:F195))</f>
+      <c r="H195" s="23">
+        <f>IF(C195="","",SUMPRODUCT(($C$43:C195=C195)*(2*($D$43:D195="Доход")-1)*$F$43:F195))</f>
         <v/>
       </c>
     </row>
@@ -3843,10 +4032,10 @@
       <c r="C196" s="16" t="n"/>
       <c r="D196" s="16" t="n"/>
       <c r="E196" s="16" t="n"/>
-      <c r="F196" s="20" t="n"/>
+      <c r="F196" s="22" t="n"/>
       <c r="G196" s="16" t="n"/>
-      <c r="H196" s="21">
-        <f>IF(C196="","",SUMPRODUCT(($C$27:C196=C196)*(2*($D$27:D196="Доход")-1)*$F$27:F196))</f>
+      <c r="H196" s="23">
+        <f>IF(C196="","",SUMPRODUCT(($C$43:C196=C196)*(2*($D$43:D196="Доход")-1)*$F$43:F196))</f>
         <v/>
       </c>
     </row>
@@ -3855,10 +4044,10 @@
       <c r="C197" s="16" t="n"/>
       <c r="D197" s="16" t="n"/>
       <c r="E197" s="16" t="n"/>
-      <c r="F197" s="20" t="n"/>
+      <c r="F197" s="22" t="n"/>
       <c r="G197" s="16" t="n"/>
-      <c r="H197" s="21">
-        <f>IF(C197="","",SUMPRODUCT(($C$27:C197=C197)*(2*($D$27:D197="Доход")-1)*$F$27:F197))</f>
+      <c r="H197" s="23">
+        <f>IF(C197="","",SUMPRODUCT(($C$43:C197=C197)*(2*($D$43:D197="Доход")-1)*$F$43:F197))</f>
         <v/>
       </c>
     </row>
@@ -3867,10 +4056,10 @@
       <c r="C198" s="16" t="n"/>
       <c r="D198" s="16" t="n"/>
       <c r="E198" s="16" t="n"/>
-      <c r="F198" s="20" t="n"/>
+      <c r="F198" s="22" t="n"/>
       <c r="G198" s="16" t="n"/>
-      <c r="H198" s="21">
-        <f>IF(C198="","",SUMPRODUCT(($C$27:C198=C198)*(2*($D$27:D198="Доход")-1)*$F$27:F198))</f>
+      <c r="H198" s="23">
+        <f>IF(C198="","",SUMPRODUCT(($C$43:C198=C198)*(2*($D$43:D198="Доход")-1)*$F$43:F198))</f>
         <v/>
       </c>
     </row>
@@ -3879,10 +4068,10 @@
       <c r="C199" s="16" t="n"/>
       <c r="D199" s="16" t="n"/>
       <c r="E199" s="16" t="n"/>
-      <c r="F199" s="20" t="n"/>
+      <c r="F199" s="22" t="n"/>
       <c r="G199" s="16" t="n"/>
-      <c r="H199" s="21">
-        <f>IF(C199="","",SUMPRODUCT(($C$27:C199=C199)*(2*($D$27:D199="Доход")-1)*$F$27:F199))</f>
+      <c r="H199" s="23">
+        <f>IF(C199="","",SUMPRODUCT(($C$43:C199=C199)*(2*($D$43:D199="Доход")-1)*$F$43:F199))</f>
         <v/>
       </c>
     </row>
@@ -3891,10 +4080,10 @@
       <c r="C200" s="16" t="n"/>
       <c r="D200" s="16" t="n"/>
       <c r="E200" s="16" t="n"/>
-      <c r="F200" s="20" t="n"/>
+      <c r="F200" s="22" t="n"/>
       <c r="G200" s="16" t="n"/>
-      <c r="H200" s="21">
-        <f>IF(C200="","",SUMPRODUCT(($C$27:C200=C200)*(2*($D$27:D200="Доход")-1)*$F$27:F200))</f>
+      <c r="H200" s="23">
+        <f>IF(C200="","",SUMPRODUCT(($C$43:C200=C200)*(2*($D$43:D200="Доход")-1)*$F$43:F200))</f>
         <v/>
       </c>
     </row>
@@ -3903,10 +4092,10 @@
       <c r="C201" s="16" t="n"/>
       <c r="D201" s="16" t="n"/>
       <c r="E201" s="16" t="n"/>
-      <c r="F201" s="20" t="n"/>
+      <c r="F201" s="22" t="n"/>
       <c r="G201" s="16" t="n"/>
-      <c r="H201" s="21">
-        <f>IF(C201="","",SUMPRODUCT(($C$27:C201=C201)*(2*($D$27:D201="Доход")-1)*$F$27:F201))</f>
+      <c r="H201" s="23">
+        <f>IF(C201="","",SUMPRODUCT(($C$43:C201=C201)*(2*($D$43:D201="Доход")-1)*$F$43:F201))</f>
         <v/>
       </c>
     </row>
@@ -3915,10 +4104,10 @@
       <c r="C202" s="16" t="n"/>
       <c r="D202" s="16" t="n"/>
       <c r="E202" s="16" t="n"/>
-      <c r="F202" s="20" t="n"/>
+      <c r="F202" s="22" t="n"/>
       <c r="G202" s="16" t="n"/>
-      <c r="H202" s="21">
-        <f>IF(C202="","",SUMPRODUCT(($C$27:C202=C202)*(2*($D$27:D202="Доход")-1)*$F$27:F202))</f>
+      <c r="H202" s="23">
+        <f>IF(C202="","",SUMPRODUCT(($C$43:C202=C202)*(2*($D$43:D202="Доход")-1)*$F$43:F202))</f>
         <v/>
       </c>
     </row>
@@ -3927,10 +4116,10 @@
       <c r="C203" s="16" t="n"/>
       <c r="D203" s="16" t="n"/>
       <c r="E203" s="16" t="n"/>
-      <c r="F203" s="20" t="n"/>
+      <c r="F203" s="22" t="n"/>
       <c r="G203" s="16" t="n"/>
-      <c r="H203" s="21">
-        <f>IF(C203="","",SUMPRODUCT(($C$27:C203=C203)*(2*($D$27:D203="Доход")-1)*$F$27:F203))</f>
+      <c r="H203" s="23">
+        <f>IF(C203="","",SUMPRODUCT(($C$43:C203=C203)*(2*($D$43:D203="Доход")-1)*$F$43:F203))</f>
         <v/>
       </c>
     </row>
@@ -3939,10 +4128,10 @@
       <c r="C204" s="16" t="n"/>
       <c r="D204" s="16" t="n"/>
       <c r="E204" s="16" t="n"/>
-      <c r="F204" s="20" t="n"/>
+      <c r="F204" s="22" t="n"/>
       <c r="G204" s="16" t="n"/>
-      <c r="H204" s="21">
-        <f>IF(C204="","",SUMPRODUCT(($C$27:C204=C204)*(2*($D$27:D204="Доход")-1)*$F$27:F204))</f>
+      <c r="H204" s="23">
+        <f>IF(C204="","",SUMPRODUCT(($C$43:C204=C204)*(2*($D$43:D204="Доход")-1)*$F$43:F204))</f>
         <v/>
       </c>
     </row>
@@ -3951,10 +4140,10 @@
       <c r="C205" s="16" t="n"/>
       <c r="D205" s="16" t="n"/>
       <c r="E205" s="16" t="n"/>
-      <c r="F205" s="20" t="n"/>
+      <c r="F205" s="22" t="n"/>
       <c r="G205" s="16" t="n"/>
-      <c r="H205" s="21">
-        <f>IF(C205="","",SUMPRODUCT(($C$27:C205=C205)*(2*($D$27:D205="Доход")-1)*$F$27:F205))</f>
+      <c r="H205" s="23">
+        <f>IF(C205="","",SUMPRODUCT(($C$43:C205=C205)*(2*($D$43:D205="Доход")-1)*$F$43:F205))</f>
         <v/>
       </c>
     </row>
@@ -3963,10 +4152,10 @@
       <c r="C206" s="16" t="n"/>
       <c r="D206" s="16" t="n"/>
       <c r="E206" s="16" t="n"/>
-      <c r="F206" s="20" t="n"/>
+      <c r="F206" s="22" t="n"/>
       <c r="G206" s="16" t="n"/>
-      <c r="H206" s="21">
-        <f>IF(C206="","",SUMPRODUCT(($C$27:C206=C206)*(2*($D$27:D206="Доход")-1)*$F$27:F206))</f>
+      <c r="H206" s="23">
+        <f>IF(C206="","",SUMPRODUCT(($C$43:C206=C206)*(2*($D$43:D206="Доход")-1)*$F$43:F206))</f>
         <v/>
       </c>
     </row>
@@ -3975,10 +4164,10 @@
       <c r="C207" s="16" t="n"/>
       <c r="D207" s="16" t="n"/>
       <c r="E207" s="16" t="n"/>
-      <c r="F207" s="20" t="n"/>
+      <c r="F207" s="22" t="n"/>
       <c r="G207" s="16" t="n"/>
-      <c r="H207" s="21">
-        <f>IF(C207="","",SUMPRODUCT(($C$27:C207=C207)*(2*($D$27:D207="Доход")-1)*$F$27:F207))</f>
+      <c r="H207" s="23">
+        <f>IF(C207="","",SUMPRODUCT(($C$43:C207=C207)*(2*($D$43:D207="Доход")-1)*$F$43:F207))</f>
         <v/>
       </c>
     </row>
@@ -3987,10 +4176,10 @@
       <c r="C208" s="16" t="n"/>
       <c r="D208" s="16" t="n"/>
       <c r="E208" s="16" t="n"/>
-      <c r="F208" s="20" t="n"/>
+      <c r="F208" s="22" t="n"/>
       <c r="G208" s="16" t="n"/>
-      <c r="H208" s="21">
-        <f>IF(C208="","",SUMPRODUCT(($C$27:C208=C208)*(2*($D$27:D208="Доход")-1)*$F$27:F208))</f>
+      <c r="H208" s="23">
+        <f>IF(C208="","",SUMPRODUCT(($C$43:C208=C208)*(2*($D$43:D208="Доход")-1)*$F$43:F208))</f>
         <v/>
       </c>
     </row>
@@ -3999,10 +4188,10 @@
       <c r="C209" s="16" t="n"/>
       <c r="D209" s="16" t="n"/>
       <c r="E209" s="16" t="n"/>
-      <c r="F209" s="20" t="n"/>
+      <c r="F209" s="22" t="n"/>
       <c r="G209" s="16" t="n"/>
-      <c r="H209" s="21">
-        <f>IF(C209="","",SUMPRODUCT(($C$27:C209=C209)*(2*($D$27:D209="Доход")-1)*$F$27:F209))</f>
+      <c r="H209" s="23">
+        <f>IF(C209="","",SUMPRODUCT(($C$43:C209=C209)*(2*($D$43:D209="Доход")-1)*$F$43:F209))</f>
         <v/>
       </c>
     </row>
@@ -4011,10 +4200,10 @@
       <c r="C210" s="16" t="n"/>
       <c r="D210" s="16" t="n"/>
       <c r="E210" s="16" t="n"/>
-      <c r="F210" s="20" t="n"/>
+      <c r="F210" s="22" t="n"/>
       <c r="G210" s="16" t="n"/>
-      <c r="H210" s="21">
-        <f>IF(C210="","",SUMPRODUCT(($C$27:C210=C210)*(2*($D$27:D210="Доход")-1)*$F$27:F210))</f>
+      <c r="H210" s="23">
+        <f>IF(C210="","",SUMPRODUCT(($C$43:C210=C210)*(2*($D$43:D210="Доход")-1)*$F$43:F210))</f>
         <v/>
       </c>
     </row>
@@ -4023,10 +4212,10 @@
       <c r="C211" s="16" t="n"/>
       <c r="D211" s="16" t="n"/>
       <c r="E211" s="16" t="n"/>
-      <c r="F211" s="20" t="n"/>
+      <c r="F211" s="22" t="n"/>
       <c r="G211" s="16" t="n"/>
-      <c r="H211" s="21">
-        <f>IF(C211="","",SUMPRODUCT(($C$27:C211=C211)*(2*($D$27:D211="Доход")-1)*$F$27:F211))</f>
+      <c r="H211" s="23">
+        <f>IF(C211="","",SUMPRODUCT(($C$43:C211=C211)*(2*($D$43:D211="Доход")-1)*$F$43:F211))</f>
         <v/>
       </c>
     </row>
@@ -4035,10 +4224,10 @@
       <c r="C212" s="16" t="n"/>
       <c r="D212" s="16" t="n"/>
       <c r="E212" s="16" t="n"/>
-      <c r="F212" s="20" t="n"/>
+      <c r="F212" s="22" t="n"/>
       <c r="G212" s="16" t="n"/>
-      <c r="H212" s="21">
-        <f>IF(C212="","",SUMPRODUCT(($C$27:C212=C212)*(2*($D$27:D212="Доход")-1)*$F$27:F212))</f>
+      <c r="H212" s="23">
+        <f>IF(C212="","",SUMPRODUCT(($C$43:C212=C212)*(2*($D$43:D212="Доход")-1)*$F$43:F212))</f>
         <v/>
       </c>
     </row>
@@ -4047,10 +4236,10 @@
       <c r="C213" s="16" t="n"/>
       <c r="D213" s="16" t="n"/>
       <c r="E213" s="16" t="n"/>
-      <c r="F213" s="20" t="n"/>
+      <c r="F213" s="22" t="n"/>
       <c r="G213" s="16" t="n"/>
-      <c r="H213" s="21">
-        <f>IF(C213="","",SUMPRODUCT(($C$27:C213=C213)*(2*($D$27:D213="Доход")-1)*$F$27:F213))</f>
+      <c r="H213" s="23">
+        <f>IF(C213="","",SUMPRODUCT(($C$43:C213=C213)*(2*($D$43:D213="Доход")-1)*$F$43:F213))</f>
         <v/>
       </c>
     </row>
@@ -4059,10 +4248,10 @@
       <c r="C214" s="16" t="n"/>
       <c r="D214" s="16" t="n"/>
       <c r="E214" s="16" t="n"/>
-      <c r="F214" s="20" t="n"/>
+      <c r="F214" s="22" t="n"/>
       <c r="G214" s="16" t="n"/>
-      <c r="H214" s="21">
-        <f>IF(C214="","",SUMPRODUCT(($C$27:C214=C214)*(2*($D$27:D214="Доход")-1)*$F$27:F214))</f>
+      <c r="H214" s="23">
+        <f>IF(C214="","",SUMPRODUCT(($C$43:C214=C214)*(2*($D$43:D214="Доход")-1)*$F$43:F214))</f>
         <v/>
       </c>
     </row>
@@ -4071,10 +4260,10 @@
       <c r="C215" s="16" t="n"/>
       <c r="D215" s="16" t="n"/>
       <c r="E215" s="16" t="n"/>
-      <c r="F215" s="20" t="n"/>
+      <c r="F215" s="22" t="n"/>
       <c r="G215" s="16" t="n"/>
-      <c r="H215" s="21">
-        <f>IF(C215="","",SUMPRODUCT(($C$27:C215=C215)*(2*($D$27:D215="Доход")-1)*$F$27:F215))</f>
+      <c r="H215" s="23">
+        <f>IF(C215="","",SUMPRODUCT(($C$43:C215=C215)*(2*($D$43:D215="Доход")-1)*$F$43:F215))</f>
         <v/>
       </c>
     </row>
@@ -4083,10 +4272,10 @@
       <c r="C216" s="16" t="n"/>
       <c r="D216" s="16" t="n"/>
       <c r="E216" s="16" t="n"/>
-      <c r="F216" s="20" t="n"/>
+      <c r="F216" s="22" t="n"/>
       <c r="G216" s="16" t="n"/>
-      <c r="H216" s="21">
-        <f>IF(C216="","",SUMPRODUCT(($C$27:C216=C216)*(2*($D$27:D216="Доход")-1)*$F$27:F216))</f>
+      <c r="H216" s="23">
+        <f>IF(C216="","",SUMPRODUCT(($C$43:C216=C216)*(2*($D$43:D216="Доход")-1)*$F$43:F216))</f>
         <v/>
       </c>
     </row>
@@ -4095,10 +4284,10 @@
       <c r="C217" s="16" t="n"/>
       <c r="D217" s="16" t="n"/>
       <c r="E217" s="16" t="n"/>
-      <c r="F217" s="20" t="n"/>
+      <c r="F217" s="22" t="n"/>
       <c r="G217" s="16" t="n"/>
-      <c r="H217" s="21">
-        <f>IF(C217="","",SUMPRODUCT(($C$27:C217=C217)*(2*($D$27:D217="Доход")-1)*$F$27:F217))</f>
+      <c r="H217" s="23">
+        <f>IF(C217="","",SUMPRODUCT(($C$43:C217=C217)*(2*($D$43:D217="Доход")-1)*$F$43:F217))</f>
         <v/>
       </c>
     </row>
@@ -4107,10 +4296,10 @@
       <c r="C218" s="16" t="n"/>
       <c r="D218" s="16" t="n"/>
       <c r="E218" s="16" t="n"/>
-      <c r="F218" s="20" t="n"/>
+      <c r="F218" s="22" t="n"/>
       <c r="G218" s="16" t="n"/>
-      <c r="H218" s="21">
-        <f>IF(C218="","",SUMPRODUCT(($C$27:C218=C218)*(2*($D$27:D218="Доход")-1)*$F$27:F218))</f>
+      <c r="H218" s="23">
+        <f>IF(C218="","",SUMPRODUCT(($C$43:C218=C218)*(2*($D$43:D218="Доход")-1)*$F$43:F218))</f>
         <v/>
       </c>
     </row>
@@ -4119,10 +4308,10 @@
       <c r="C219" s="16" t="n"/>
       <c r="D219" s="16" t="n"/>
       <c r="E219" s="16" t="n"/>
-      <c r="F219" s="20" t="n"/>
+      <c r="F219" s="22" t="n"/>
       <c r="G219" s="16" t="n"/>
-      <c r="H219" s="21">
-        <f>IF(C219="","",SUMPRODUCT(($C$27:C219=C219)*(2*($D$27:D219="Доход")-1)*$F$27:F219))</f>
+      <c r="H219" s="23">
+        <f>IF(C219="","",SUMPRODUCT(($C$43:C219=C219)*(2*($D$43:D219="Доход")-1)*$F$43:F219))</f>
         <v/>
       </c>
     </row>
@@ -4131,10 +4320,10 @@
       <c r="C220" s="16" t="n"/>
       <c r="D220" s="16" t="n"/>
       <c r="E220" s="16" t="n"/>
-      <c r="F220" s="20" t="n"/>
+      <c r="F220" s="22" t="n"/>
       <c r="G220" s="16" t="n"/>
-      <c r="H220" s="21">
-        <f>IF(C220="","",SUMPRODUCT(($C$27:C220=C220)*(2*($D$27:D220="Доход")-1)*$F$27:F220))</f>
+      <c r="H220" s="23">
+        <f>IF(C220="","",SUMPRODUCT(($C$43:C220=C220)*(2*($D$43:D220="Доход")-1)*$F$43:F220))</f>
         <v/>
       </c>
     </row>
@@ -4143,10 +4332,10 @@
       <c r="C221" s="16" t="n"/>
       <c r="D221" s="16" t="n"/>
       <c r="E221" s="16" t="n"/>
-      <c r="F221" s="20" t="n"/>
+      <c r="F221" s="22" t="n"/>
       <c r="G221" s="16" t="n"/>
-      <c r="H221" s="21">
-        <f>IF(C221="","",SUMPRODUCT(($C$27:C221=C221)*(2*($D$27:D221="Доход")-1)*$F$27:F221))</f>
+      <c r="H221" s="23">
+        <f>IF(C221="","",SUMPRODUCT(($C$43:C221=C221)*(2*($D$43:D221="Доход")-1)*$F$43:F221))</f>
         <v/>
       </c>
     </row>
@@ -4155,10 +4344,10 @@
       <c r="C222" s="16" t="n"/>
       <c r="D222" s="16" t="n"/>
       <c r="E222" s="16" t="n"/>
-      <c r="F222" s="20" t="n"/>
+      <c r="F222" s="22" t="n"/>
       <c r="G222" s="16" t="n"/>
-      <c r="H222" s="21">
-        <f>IF(C222="","",SUMPRODUCT(($C$27:C222=C222)*(2*($D$27:D222="Доход")-1)*$F$27:F222))</f>
+      <c r="H222" s="23">
+        <f>IF(C222="","",SUMPRODUCT(($C$43:C222=C222)*(2*($D$43:D222="Доход")-1)*$F$43:F222))</f>
         <v/>
       </c>
     </row>
@@ -4167,10 +4356,10 @@
       <c r="C223" s="16" t="n"/>
       <c r="D223" s="16" t="n"/>
       <c r="E223" s="16" t="n"/>
-      <c r="F223" s="20" t="n"/>
+      <c r="F223" s="22" t="n"/>
       <c r="G223" s="16" t="n"/>
-      <c r="H223" s="21">
-        <f>IF(C223="","",SUMPRODUCT(($C$27:C223=C223)*(2*($D$27:D223="Доход")-1)*$F$27:F223))</f>
+      <c r="H223" s="23">
+        <f>IF(C223="","",SUMPRODUCT(($C$43:C223=C223)*(2*($D$43:D223="Доход")-1)*$F$43:F223))</f>
         <v/>
       </c>
     </row>
@@ -4179,10 +4368,10 @@
       <c r="C224" s="16" t="n"/>
       <c r="D224" s="16" t="n"/>
       <c r="E224" s="16" t="n"/>
-      <c r="F224" s="20" t="n"/>
+      <c r="F224" s="22" t="n"/>
       <c r="G224" s="16" t="n"/>
-      <c r="H224" s="21">
-        <f>IF(C224="","",SUMPRODUCT(($C$27:C224=C224)*(2*($D$27:D224="Доход")-1)*$F$27:F224))</f>
+      <c r="H224" s="23">
+        <f>IF(C224="","",SUMPRODUCT(($C$43:C224=C224)*(2*($D$43:D224="Доход")-1)*$F$43:F224))</f>
         <v/>
       </c>
     </row>
@@ -4191,10 +4380,10 @@
       <c r="C225" s="16" t="n"/>
       <c r="D225" s="16" t="n"/>
       <c r="E225" s="16" t="n"/>
-      <c r="F225" s="20" t="n"/>
+      <c r="F225" s="22" t="n"/>
       <c r="G225" s="16" t="n"/>
-      <c r="H225" s="21">
-        <f>IF(C225="","",SUMPRODUCT(($C$27:C225=C225)*(2*($D$27:D225="Доход")-1)*$F$27:F225))</f>
+      <c r="H225" s="23">
+        <f>IF(C225="","",SUMPRODUCT(($C$43:C225=C225)*(2*($D$43:D225="Доход")-1)*$F$43:F225))</f>
         <v/>
       </c>
     </row>
@@ -4203,420 +4392,231 @@
       <c r="C226" s="16" t="n"/>
       <c r="D226" s="16" t="n"/>
       <c r="E226" s="16" t="n"/>
-      <c r="F226" s="20" t="n"/>
+      <c r="F226" s="22" t="n"/>
       <c r="G226" s="16" t="n"/>
-      <c r="H226" s="21">
-        <f>IF(C226="","",SUMPRODUCT(($C$27:C226=C226)*(2*($D$27:D226="Доход")-1)*$F$27:F226))</f>
+      <c r="H226" s="23">
+        <f>IF(C226="","",SUMPRODUCT(($C$43:C226=C226)*(2*($D$43:D226="Доход")-1)*$F$43:F226))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="227">
+      <c r="B227" s="16" t="n"/>
+      <c r="C227" s="16" t="n"/>
+      <c r="D227" s="16" t="n"/>
+      <c r="E227" s="16" t="n"/>
+      <c r="F227" s="22" t="n"/>
+      <c r="G227" s="16" t="n"/>
+      <c r="H227" s="23">
+        <f>IF(C227="","",SUMPRODUCT(($C$43:C227=C227)*(2*($D$43:D227="Доход")-1)*$F$43:F227))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="228">
+      <c r="B228" s="16" t="n"/>
+      <c r="C228" s="16" t="n"/>
+      <c r="D228" s="16" t="n"/>
+      <c r="E228" s="16" t="n"/>
+      <c r="F228" s="22" t="n"/>
+      <c r="G228" s="16" t="n"/>
+      <c r="H228" s="23">
+        <f>IF(C228="","",SUMPRODUCT(($C$43:C228=C228)*(2*($D$43:D228="Доход")-1)*$F$43:F228))</f>
         <v/>
       </c>
     </row>
     <row r="229">
-      <c r="D229" s="5" t="inlineStr">
-        <is>
-          <t>ДОХОДЫ ПО КАТЕГОРИЯМ (месяц)</t>
-        </is>
-      </c>
-      <c r="E229" s="6" t="n"/>
-      <c r="F229" s="6" t="n"/>
-      <c r="H229" s="7" t="inlineStr">
-        <is>
-          <t>РАСХОДЫ ПО КАТЕГОРИЯМ (месяц)</t>
-        </is>
-      </c>
-      <c r="I229" s="8" t="n"/>
-      <c r="J229" s="8" t="n"/>
-      <c r="L229" s="13" t="inlineStr">
-        <is>
-          <t>ДИНАМИКА ЗА ГОД</t>
-        </is>
-      </c>
-      <c r="M229" s="14" t="n"/>
-      <c r="N229" s="14" t="n"/>
+      <c r="B229" s="16" t="n"/>
+      <c r="C229" s="16" t="n"/>
+      <c r="D229" s="16" t="n"/>
+      <c r="E229" s="16" t="n"/>
+      <c r="F229" s="22" t="n"/>
+      <c r="G229" s="16" t="n"/>
+      <c r="H229" s="23">
+        <f>IF(C229="","",SUMPRODUCT(($C$43:C229=C229)*(2*($D$43:D229="Доход")-1)*$F$43:F229))</f>
+        <v/>
+      </c>
     </row>
     <row r="230">
-      <c r="D230" s="18" t="inlineStr">
-        <is>
-          <t>Категория</t>
-        </is>
-      </c>
-      <c r="E230" s="18" t="inlineStr">
-        <is>
-          <t>Сумма</t>
-        </is>
-      </c>
-      <c r="F230" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="H230" s="22" t="inlineStr">
-        <is>
-          <t>Категория</t>
-        </is>
-      </c>
-      <c r="I230" s="22" t="inlineStr">
-        <is>
-          <t>Сумма</t>
-        </is>
-      </c>
-      <c r="J230" s="22" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="L230" s="15" t="inlineStr">
-        <is>
-          <t>Месяц</t>
-        </is>
-      </c>
-      <c r="M230" s="15" t="inlineStr">
-        <is>
-          <t>Доход</t>
-        </is>
-      </c>
-      <c r="N230" s="15" t="inlineStr">
-        <is>
-          <t>Расход</t>
-        </is>
+      <c r="B230" s="16" t="n"/>
+      <c r="C230" s="16" t="n"/>
+      <c r="D230" s="16" t="n"/>
+      <c r="E230" s="16" t="n"/>
+      <c r="F230" s="22" t="n"/>
+      <c r="G230" s="16" t="n"/>
+      <c r="H230" s="23">
+        <f>IF(C230="","",SUMPRODUCT(($C$43:C230=C230)*(2*($D$43:D230="Доход")-1)*$F$43:F230))</f>
+        <v/>
       </c>
     </row>
     <row r="231">
-      <c r="D231" s="16" t="inlineStr">
-        <is>
-          <t>Зарплата</t>
-        </is>
-      </c>
-      <c r="E231" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*($E$27:$E$226="Зарплата")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="F231" s="23">
-        <f>IFERROR(E231/$B$6,0)</f>
-        <v/>
-      </c>
-      <c r="H231" s="16" t="inlineStr">
-        <is>
-          <t>Аренда</t>
-        </is>
-      </c>
-      <c r="I231" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Аренда")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J231" s="23">
-        <f>IFERROR(I231/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L231" s="16">
-        <f>TEXT(DATE($F$3,1,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M231" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=1)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N231" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=1)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B231" s="16" t="n"/>
+      <c r="C231" s="16" t="n"/>
+      <c r="D231" s="16" t="n"/>
+      <c r="E231" s="16" t="n"/>
+      <c r="F231" s="22" t="n"/>
+      <c r="G231" s="16" t="n"/>
+      <c r="H231" s="23">
+        <f>IF(C231="","",SUMPRODUCT(($C$43:C231=C231)*(2*($D$43:D231="Доход")-1)*$F$43:F231))</f>
         <v/>
       </c>
     </row>
     <row r="232">
-      <c r="D232" s="16" t="inlineStr">
-        <is>
-          <t>Заказы</t>
-        </is>
-      </c>
-      <c r="E232" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*($E$27:$E$226="Заказы")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="F232" s="23">
-        <f>IFERROR(E232/$B$6,0)</f>
-        <v/>
-      </c>
-      <c r="H232" s="16" t="inlineStr">
-        <is>
-          <t>Продукты</t>
-        </is>
-      </c>
-      <c r="I232" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Продукты")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J232" s="23">
-        <f>IFERROR(I232/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L232" s="16">
-        <f>TEXT(DATE($F$3,2,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M232" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=2)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N232" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=2)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B232" s="16" t="n"/>
+      <c r="C232" s="16" t="n"/>
+      <c r="D232" s="16" t="n"/>
+      <c r="E232" s="16" t="n"/>
+      <c r="F232" s="22" t="n"/>
+      <c r="G232" s="16" t="n"/>
+      <c r="H232" s="23">
+        <f>IF(C232="","",SUMPRODUCT(($C$43:C232=C232)*(2*($D$43:D232="Доход")-1)*$F$43:F232))</f>
         <v/>
       </c>
     </row>
     <row r="233">
-      <c r="D233" s="16" t="inlineStr">
-        <is>
-          <t>Подарок</t>
-        </is>
-      </c>
-      <c r="E233" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*($E$27:$E$226="Подарок")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="F233" s="23">
-        <f>IFERROR(E233/$B$6,0)</f>
-        <v/>
-      </c>
-      <c r="H233" s="16" t="inlineStr">
-        <is>
-          <t>Обучение</t>
-        </is>
-      </c>
-      <c r="I233" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Обучение")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J233" s="23">
-        <f>IFERROR(I233/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L233" s="16">
-        <f>TEXT(DATE($F$3,3,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M233" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=3)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N233" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=3)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B233" s="16" t="n"/>
+      <c r="C233" s="16" t="n"/>
+      <c r="D233" s="16" t="n"/>
+      <c r="E233" s="16" t="n"/>
+      <c r="F233" s="22" t="n"/>
+      <c r="G233" s="16" t="n"/>
+      <c r="H233" s="23">
+        <f>IF(C233="","",SUMPRODUCT(($C$43:C233=C233)*(2*($D$43:D233="Доход")-1)*$F$43:F233))</f>
         <v/>
       </c>
     </row>
     <row r="234">
-      <c r="H234" s="16" t="inlineStr">
-        <is>
-          <t>Кредит</t>
-        </is>
-      </c>
-      <c r="I234" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Кредит")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J234" s="23">
-        <f>IFERROR(I234/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L234" s="16">
-        <f>TEXT(DATE($F$3,4,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M234" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=4)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N234" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=4)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B234" s="16" t="n"/>
+      <c r="C234" s="16" t="n"/>
+      <c r="D234" s="16" t="n"/>
+      <c r="E234" s="16" t="n"/>
+      <c r="F234" s="22" t="n"/>
+      <c r="G234" s="16" t="n"/>
+      <c r="H234" s="23">
+        <f>IF(C234="","",SUMPRODUCT(($C$43:C234=C234)*(2*($D$43:D234="Доход")-1)*$F$43:F234))</f>
         <v/>
       </c>
     </row>
     <row r="235">
-      <c r="H235" s="16" t="inlineStr">
-        <is>
-          <t>Субподряд</t>
-        </is>
-      </c>
-      <c r="I235" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Субподряд")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J235" s="23">
-        <f>IFERROR(I235/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L235" s="16">
-        <f>TEXT(DATE($F$3,5,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M235" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=5)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N235" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=5)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B235" s="16" t="n"/>
+      <c r="C235" s="16" t="n"/>
+      <c r="D235" s="16" t="n"/>
+      <c r="E235" s="16" t="n"/>
+      <c r="F235" s="22" t="n"/>
+      <c r="G235" s="16" t="n"/>
+      <c r="H235" s="23">
+        <f>IF(C235="","",SUMPRODUCT(($C$43:C235=C235)*(2*($D$43:D235="Доход")-1)*$F$43:F235))</f>
         <v/>
       </c>
     </row>
     <row r="236">
-      <c r="H236" s="16" t="inlineStr">
-        <is>
-          <t>Ипотека</t>
-        </is>
-      </c>
-      <c r="I236" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Ипотека")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J236" s="23">
-        <f>IFERROR(I236/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L236" s="16">
-        <f>TEXT(DATE($F$3,6,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M236" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=6)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N236" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=6)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B236" s="16" t="n"/>
+      <c r="C236" s="16" t="n"/>
+      <c r="D236" s="16" t="n"/>
+      <c r="E236" s="16" t="n"/>
+      <c r="F236" s="22" t="n"/>
+      <c r="G236" s="16" t="n"/>
+      <c r="H236" s="23">
+        <f>IF(C236="","",SUMPRODUCT(($C$43:C236=C236)*(2*($D$43:D236="Доход")-1)*$F$43:F236))</f>
         <v/>
       </c>
     </row>
     <row r="237">
-      <c r="H237" s="16" t="inlineStr">
-        <is>
-          <t>Подарок</t>
-        </is>
-      </c>
-      <c r="I237" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Подарок")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J237" s="23">
-        <f>IFERROR(I237/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L237" s="16">
-        <f>TEXT(DATE($F$3,7,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M237" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=7)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N237" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=7)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B237" s="16" t="n"/>
+      <c r="C237" s="16" t="n"/>
+      <c r="D237" s="16" t="n"/>
+      <c r="E237" s="16" t="n"/>
+      <c r="F237" s="22" t="n"/>
+      <c r="G237" s="16" t="n"/>
+      <c r="H237" s="23">
+        <f>IF(C237="","",SUMPRODUCT(($C$43:C237=C237)*(2*($D$43:D237="Доход")-1)*$F$43:F237))</f>
         <v/>
       </c>
     </row>
     <row r="238">
-      <c r="H238" s="16" t="inlineStr">
-        <is>
-          <t>Аутсорс</t>
-        </is>
-      </c>
-      <c r="I238" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*($E$27:$E$226="Аутсорс")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=MATCH($C$3,Справочник!$L$3:$L$14,0))*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="J238" s="23">
-        <f>IFERROR(I238/$D$6,0)</f>
-        <v/>
-      </c>
-      <c r="L238" s="16">
-        <f>TEXT(DATE($F$3,8,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M238" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=8)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N238" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=8)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B238" s="16" t="n"/>
+      <c r="C238" s="16" t="n"/>
+      <c r="D238" s="16" t="n"/>
+      <c r="E238" s="16" t="n"/>
+      <c r="F238" s="22" t="n"/>
+      <c r="G238" s="16" t="n"/>
+      <c r="H238" s="23">
+        <f>IF(C238="","",SUMPRODUCT(($C$43:C238=C238)*(2*($D$43:D238="Доход")-1)*$F$43:F238))</f>
         <v/>
       </c>
     </row>
     <row r="239">
-      <c r="L239" s="16">
-        <f>TEXT(DATE($F$3,9,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M239" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=9)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N239" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=9)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B239" s="16" t="n"/>
+      <c r="C239" s="16" t="n"/>
+      <c r="D239" s="16" t="n"/>
+      <c r="E239" s="16" t="n"/>
+      <c r="F239" s="22" t="n"/>
+      <c r="G239" s="16" t="n"/>
+      <c r="H239" s="23">
+        <f>IF(C239="","",SUMPRODUCT(($C$43:C239=C239)*(2*($D$43:D239="Доход")-1)*$F$43:F239))</f>
         <v/>
       </c>
     </row>
     <row r="240">
-      <c r="L240" s="16">
-        <f>TEXT(DATE($F$3,10,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M240" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=10)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N240" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=10)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B240" s="16" t="n"/>
+      <c r="C240" s="16" t="n"/>
+      <c r="D240" s="16" t="n"/>
+      <c r="E240" s="16" t="n"/>
+      <c r="F240" s="22" t="n"/>
+      <c r="G240" s="16" t="n"/>
+      <c r="H240" s="23">
+        <f>IF(C240="","",SUMPRODUCT(($C$43:C240=C240)*(2*($D$43:D240="Доход")-1)*$F$43:F240))</f>
         <v/>
       </c>
     </row>
     <row r="241">
-      <c r="L241" s="16">
-        <f>TEXT(DATE($F$3,11,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M241" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=11)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N241" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=11)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B241" s="16" t="n"/>
+      <c r="C241" s="16" t="n"/>
+      <c r="D241" s="16" t="n"/>
+      <c r="E241" s="16" t="n"/>
+      <c r="F241" s="22" t="n"/>
+      <c r="G241" s="16" t="n"/>
+      <c r="H241" s="23">
+        <f>IF(C241="","",SUMPRODUCT(($C$43:C241=C241)*(2*($D$43:D241="Доход")-1)*$F$43:F241))</f>
         <v/>
       </c>
     </row>
     <row r="242">
-      <c r="L242" s="16">
-        <f>TEXT(DATE($F$3,12,1),"mmm yy")</f>
-        <v/>
-      </c>
-      <c r="M242" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Доход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=12)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
-        <v/>
-      </c>
-      <c r="N242" s="16">
-        <f>SUMPRODUCT(($D$27:$D$226="Расход")*(YEAR($B$27:$B$226+0)=$F$3)*(MONTH($B$27:$B$226+0)=12)*(COUNTIF(Справочник!$C$3:$C$10,$E$27:$E$226)=0)*$F$27:$F$226)</f>
+      <c r="B242" s="16" t="n"/>
+      <c r="C242" s="16" t="n"/>
+      <c r="D242" s="16" t="n"/>
+      <c r="E242" s="16" t="n"/>
+      <c r="F242" s="22" t="n"/>
+      <c r="G242" s="16" t="n"/>
+      <c r="H242" s="23">
+        <f>IF(C242="","",SUMPRODUCT(($C$43:C242=C242)*(2*($D$43:D242="Доход")-1)*$F$43:F242))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="L25:N25"/>
     <mergeCell ref="F5:H5"/>
+    <mergeCell ref="B41:H41"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="F6:H8"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D5:E5"/>
-    <mergeCell ref="L229:N229"/>
     <mergeCell ref="D6:E8"/>
     <mergeCell ref="B6:C8"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="H229:J229"/>
-    <mergeCell ref="D229:F229"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="H25:J25"/>
   </mergeCells>
   <conditionalFormatting sqref="C13:C22">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D27:D226">
+  <conditionalFormatting sqref="D43:D242">
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>D27="Доход"</formula>
+      <formula>D43="Доход"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>D27="Расход"</formula>
+      <formula>D43="Расход"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
@@ -4626,13 +4626,13 @@
     <dataValidation sqref="F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочник!$M$3:$M$12</formula1>
     </dataValidation>
-    <dataValidation sqref="C27:C226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C43:C242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочник!$K$3:$K$9</formula1>
     </dataValidation>
-    <dataValidation sqref="D27:D226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D43:D242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Доход,Расход"</formula1>
     </dataValidation>
-    <dataValidation sqref="E27:E226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E43:E242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочник!$J$3:$J$20</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>